<commit_message>
Atualiza currículo e controle público de vagas
</commit_message>
<xml_diff>
--- a/planilhas/Controle_Candidaturas_Fintech_Guilherme_PUBLICO.xlsx
+++ b/planilhas/Controle_Candidaturas_Fintech_Guilherme_PUBLICO.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidaturas" sheetId="1" r:id="Ra95f308f7d8e4e8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log de auditoria" sheetId="2" r:id="R6c0f24fa49794ab9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidaturas" sheetId="1" r:id="R19ddb00af5ca4b5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log de auditoria" sheetId="2" r:id="Rb878a634a4ea4c18"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -174,7 +174,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="63">
+  <x:cellXfs count="64">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -315,6 +315,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -500,7 +503,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CandidaturasTable" displayName="CandidaturasTable" ref="A9:K108" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CandidaturasTable" displayName="CandidaturasTable" ref="A9:K171" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Status"/>
     <x:tableColumn id="2" name="Empresa"/>
@@ -753,7 +756,10 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>Tecnologia, dados, IA e operações técnicas. Versão pública: dados pessoais e links privados removidos. Fonte atualizada em 21/09/2026.</x:v>
+        <x:v>Tecnologia, dados, IA e operações técnicas. Versão pública: dados pessoais e links privados removidos. Fonte atualizada em 02/10/2026.</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>Tecnologia, dados, IA e operações técnicas. Currículo mestre e ciclo de candidaturas atualizados em 02/10/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -761,13 +767,13 @@
         <x:v>Regra salarial</x:v>
       </x:c>
       <x:c r="B5" s="6" t="str">
-        <x:v>R$ 4.000</x:v>
+        <x:v>R$ 3.000 (Indeed atual)</x:v>
       </x:c>
       <x:c r="C5" s="6" t="str">
         <x:v>Escopo</x:v>
       </x:c>
       <x:c r="D5" s="6" t="str">
-        <x:v>Sem comercial, suporte ou QA</x:v>
+        <x:v>Sem comercial, suporte, QA ou vagas sênior; pleno só se requisitos forem compatíveis com júnior</x:v>
       </x:c>
       <x:c r="E5" s="6" t="str">
         <x:v>Disponibilidade</x:v>
@@ -787,24 +793,24 @@
         <x:v>Candidaturas confirmadas</x:v>
       </x:c>
       <x:c r="B7" s="9" t="n">
-        <x:f>SUM(L10:L108)</x:f>
-        <x:v>62</x:v>
+        <x:f>SUM(L10:L171)</x:f>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C7" s="8"/>
       <x:c r="D7" s="8" t="str">
         <x:v>Itens em controle</x:v>
       </x:c>
       <x:c r="E7" s="9" t="n">
-        <x:f>COUNTA(A10:A108)</x:f>
-        <x:v>99</x:v>
+        <x:f>COUNTA(A10:A171)</x:f>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="F7" s="8"/>
       <x:c r="G7" s="8" t="str">
         <x:v>Pendentes</x:v>
       </x:c>
       <x:c r="H7" s="9" t="n">
-        <x:f>SUM(M10:M108)</x:f>
-        <x:v>31</x:v>
+        <x:f>SUM(M10:M171)</x:f>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
@@ -2622,7 +2628,7 @@
         <x:v>São Paulo, presencial</x:v>
       </x:c>
       <x:c r="F51" s="16" t="str">
-        <x:v>https://jobs.ashbyhq.com/enter-ai/09fb5102-783f-42d4-95a5-0c294ea5c1a4/application</x:v>
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
       </x:c>
       <x:c r="G51" s="18" t="str">
         <x:v>IA de triagem informada</x:v>
@@ -4216,19 +4222,19 @@
         <x:v>Acessar na plataforma (link privado removido)</x:v>
       </x:c>
       <x:c r="G88" s="18" t="str">
-        <x:v>Sem audiovisual declarado</x:v>
+        <x:v>Fit Cultural e testes complementares previstos; formato audiovisual não informado</x:v>
       </x:c>
       <x:c r="H88" s="18" t="str">
-        <x:v>Acompanhar e-mail; validar formato de cada próxima etapa antes de iniciar</x:v>
+        <x:v>Acompanhar e-mail; validar formato de cada etapa antes de iniciar</x:v>
       </x:c>
       <x:c r="I88" s="19" t="str">
-        <x:v>21/09/2026</x:v>
+        <x:v>30/09/2026</x:v>
       </x:c>
       <x:c r="J88" s="18" t="str">
-        <x:v>Candidatura personalizada enviada e confirmada pela Gupy em 21/09. A apresentação destaca projetos próprios em Python, APIs, SQL e IA aplicada; foram selecionadas SQL, API REST e Python. A vaga aceita superior em andamento, inglês intermediário, Python/Java básico e projeto acadêmico de IA.</x:v>
+        <x:v>Candidatura retomada, personalizada e finalizada na Gupy em 30/09. A apresentação destacou ADS em fase final, Python, APIs REST, SQL/PostgreSQL, Git, Docker, IA/LLM aplicada e inglês intermediário. As respostas já registradas no portal foram preservadas; cloud e ferramentas específicas foram tratadas como aprendizado.</x:v>
       </x:c>
       <x:c r="K88" s="24" t="str">
-        <x:v>Sim — confirmação Gupy 21/09</x:v>
+        <x:v>Portal — confirmação Gupy 30/09</x:v>
       </x:c>
       <x:c r="L88" t="n">
         <x:f>IF(LEFT(K88,3)="Sim",1,0)+IF(LEFT(K88,6)="Portal",1,0)</x:f>
@@ -4327,7 +4333,7 @@
     </x:row>
     <x:row r="91" ht="60" customHeight="1">
       <x:c r="A91" s="23" t="str">
-        <x:v>Pendente — validar vaga Indeed</x:v>
+        <x:v>Pendente — reCAPTCHA</x:v>
       </x:c>
       <x:c r="B91" s="15" t="str">
         <x:v>Black Lion</x:v>
@@ -4339,7 +4345,7 @@
         <x:v>Desenvolvimento</x:v>
       </x:c>
       <x:c r="E91" s="15" t="str">
-        <x:v>São Paulo/SP, híbrido (3x presencial)</x:v>
+        <x:v>São Paulo/SP, híbrido (3x por semana)</x:v>
       </x:c>
       <x:c r="F91" s="16" t="str">
         <x:v>https://br.indeed.com/viewjob?jk=98039e0bd9a2fb44</x:v>
@@ -4348,16 +4354,16 @@
         <x:v>Sem audiovisual declarado</x:v>
       </x:c>
       <x:c r="H91" s="18" t="str">
-        <x:v>Revalidar anúncio, salário e formulário antes de personalizar; só avançar se a vaga ainda estiver ativa</x:v>
+        <x:v>Abrir em Minhas Vagas no Indeed e concluir o reCAPTCHA/Enviar pessoalmente</x:v>
       </x:c>
       <x:c r="I91" s="19" t="str">
-        <x:v>20/09/2026</x:v>
+        <x:v>30/09/2026</x:v>
       </x:c>
       <x:c r="J91" s="18" t="str">
-        <x:v>Pesquisa Indeed: aderência forte em fintech, TypeScript/JavaScript, APIs REST e Git. Node.js, MySQL, NestJS, React Native, Redis e JWT são pontos de estudo, não experiências a alegar. Salário não divulgado.</x:v>
+        <x:v>Candidatura personalizada chegou a 100% no Indeed com currículo selecionado. GitHub, remuneração atual aproximada de R$6 mil, disponibilidade presencial e pretensão mínima foram preenchidos de forma factual. Salário divulgado de R$3.000/mês; envio final bloqueado por reCAPTCHA, não contornado.</x:v>
       </x:c>
       <x:c r="K91" s="24" t="str">
-        <x:v>Não aplicável — não enviada</x:v>
+        <x:v>Não — rascunho 100% no Indeed</x:v>
       </x:c>
       <x:c r="L91" t="n">
         <x:f>IF(LEFT(K91,3)="Sim",1,0)+IF(LEFT(K91,6)="Portal",1,0)</x:f>
@@ -5099,14 +5105,2733 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="109">
+    <x:row r="109" ht="84" customHeight="1">
       <x:c r="A109" s="32" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B109" s="63" t="str">
+        <x:v>Afya</x:v>
+      </x:c>
+      <x:c r="C109" s="63" t="str">
+        <x:v>Analista de Dados Júnior</x:v>
+      </x:c>
+      <x:c r="D109" s="63" t="str">
+        <x:v>Dados e IA</x:v>
+      </x:c>
+      <x:c r="E109" s="63" t="str">
+        <x:v>Remoto; descrição também cita híbrido em São Paulo/SP</x:v>
+      </x:c>
+      <x:c r="F109" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G109" s="63" t="str">
+        <x:v>Entrevista Inteligente na etapa seguinte; formato não informado</x:v>
+      </x:c>
+      <x:c r="H109" s="63" t="str">
+        <x:v>Acompanhar e-mail; validar o formato antes de iniciar qualquer entrevista</x:v>
+      </x:c>
+      <x:c r="I109" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J109" s="63" t="str">
+        <x:v>Candidatura finalizada e confirmada na Gupy em 30/09. Personalização destacou SQL, Python, PostgreSQL, Git, APIs, automações, validação de integridade e documentação. Power BI e dbt foram tratados como temas de aprofundamento, não como experiência consolidada. Respostas factuais: não precisa de adaptação; remuneração atual aproximada de R$6 mil em freelances; sem parentesco.</x:v>
+      </x:c>
+      <x:c r="K109" s="63" t="str">
+        <x:v>Portal — confirmação Gupy 30/09</x:v>
+      </x:c>
+      <x:c r="L109" t="n">
+        <x:f>IF(LEFT(K109,3)="Sim",1,0)+IF(LEFT(K109,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M109" t="n">
+        <x:f>IF(LEFT(A109,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="84" customHeight="1">
+      <x:c r="A110" s="63" t="str">
+        <x:v>Enviada por e-mail</x:v>
+      </x:c>
+      <x:c r="B110" s="63" t="str">
+        <x:v>MOST Specialist Technologies</x:v>
+      </x:c>
+      <x:c r="C110" s="63" t="str">
+        <x:v>Full Stack Developer (Python) — Hiperautomação</x:v>
+      </x:c>
+      <x:c r="D110" s="63" t="str">
+        <x:v>Desenvolvimento e automação</x:v>
+      </x:c>
+      <x:c r="E110" s="63" t="str">
+        <x:v>Remoto; estágio de 6h</x:v>
+      </x:c>
+      <x:c r="F110" s="63" t="str">
+        <x:v>https://most.com.br/vagas/full-stack-developer-python-hiperautomacao</x:v>
+      </x:c>
+      <x:c r="G110" s="63" t="str">
+        <x:v>Desafio técnico e apresentação técnica previstos; formato audiovisual do bate-papo não informado</x:v>
+      </x:c>
+      <x:c r="H110" s="63" t="str">
+        <x:v>Aguardar retorno do RH; realizar pessoalmente qualquer desafio técnico ou entrevista</x:v>
+      </x:c>
+      <x:c r="I110" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J110" s="63" t="str">
+        <x:v>Candidatura personalizada enviada por e-mail ao RH da MOST em 30/09, com currículo técnico público, GitHub e LinkedIn. O Gmail exibiu 'Mensagem enviada'. A vaga anuncia bolsa oficial de R$4.000/mês e tem forte aderência em Python, Docker, APIs, JavaScript/TypeScript, Git e Linux. O desafio técnico não foi iniciado e qualquer avaliação deve ser feita pessoalmente.</x:v>
+      </x:c>
+      <x:c r="K110" s="63" t="str">
+        <x:v>E-mail enviado — Gmail confirmou o envio em 30/09; recibo da empresa pendente</x:v>
+      </x:c>
+      <x:c r="L110" t="n">
+        <x:f>IF(LEFT(K110,3)="Sim",1,0)+IF(LEFT(K110,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M110" t="n">
+        <x:f>IF(LEFT(A110,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="84" customHeight="1">
+      <x:c r="A111" s="63" t="str">
+        <x:v>Pendente — dados cadastrais</x:v>
+      </x:c>
+      <x:c r="B111" s="63" t="str">
+        <x:v>Ana Recrutamento e Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="C111" s="63" t="str">
+        <x:v>Desenvolvedor Full Stack — Indústria</x:v>
+      </x:c>
+      <x:c r="D111" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E111" s="63" t="str">
+        <x:v>São Ludgero/SC, híbrido; mudança possível</x:v>
+      </x:c>
+      <x:c r="F111" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=e61be2010aa61b81</x:v>
+      </x:c>
+      <x:c r="G111" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H111" s="63" t="str">
+        <x:v>Preencher país, estado, cidade, bairro, endereço e CEP no Indeed; depois revisar e enviar</x:v>
+      </x:c>
+      <x:c r="I111" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J111" s="63" t="str">
+        <x:v>Rascunho salvo no Indeed a 50%. Currículo Indeed selecionado; cargo pretendido e pretensão de R$5.000 preenchidos. A vaga pede dois anos e experiência sólida, portanto deve seguir como candidatura stretch e transparente. Dados de endereço completos não foram fornecidos e não foram inventados.</x:v>
+      </x:c>
+      <x:c r="K111" s="63" t="str">
+        <x:v>Não — rascunho salvo no Indeed</x:v>
+      </x:c>
+      <x:c r="L111" t="n">
+        <x:f>IF(LEFT(K111,3)="Sim",1,0)+IF(LEFT(K111,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M111" t="n">
+        <x:f>IF(LEFT(A111,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="84" customHeight="1">
+      <x:c r="A112" s="63" t="str">
+        <x:v>Pendente — currículo obrigatório</x:v>
+      </x:c>
+      <x:c r="B112" s="63" t="str">
+        <x:v>iblue Consulting</x:v>
+      </x:c>
+      <x:c r="C112" s="63" t="str">
+        <x:v>[MG] Analista Desenvolvedor Fullstack (.NET/Angular) Júnior</x:v>
+      </x:c>
+      <x:c r="D112" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E112" s="63" t="str">
+        <x:v>Rio de Janeiro/RJ, híbrido (1x por semana)</x:v>
+      </x:c>
+      <x:c r="F112" s="63" t="str">
+        <x:v>https://jobs.quickin.io/iblueconsulting/apply?job_id=6ab6b0b1d34f680013c82b51</x:v>
+      </x:c>
+      <x:c r="G112" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H112" s="63" t="str">
+        <x:v>Anexar currículo no Quickin; revisar respostas e concluir o envio</x:v>
+      </x:c>
+      <x:c r="I112" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J112" s="63" t="str">
+        <x:v>A vaga é aderente em .NET, C#, ASP.NET Web API, SQL, Git, TypeScript, APIs REST e CI/CD. Angular continua como tema de estudo. O formulário Quickin foi aberto e o envio não foi confirmado; o upload do currículo é o bloqueio operacional identificado.</x:v>
+      </x:c>
+      <x:c r="K112" s="63" t="str">
+        <x:v>Não — formulário Quickin não enviado</x:v>
+      </x:c>
+      <x:c r="L112" t="n">
+        <x:f>IF(LEFT(K112,3)="Sim",1,0)+IF(LEFT(K112,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M112" t="n">
+        <x:f>IF(LEFT(A112,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="84" customHeight="1">
+      <x:c r="A113" s="63" t="str">
+        <x:v>Pendente — currículo obrigatório</x:v>
+      </x:c>
+      <x:c r="B113" s="63" t="str">
+        <x:v>YSSY</x:v>
+      </x:c>
+      <x:c r="C113" s="63" t="str">
+        <x:v>Engenheiro de Dados Júnior</x:v>
+      </x:c>
+      <x:c r="D113" s="63" t="str">
+        <x:v>Dados e IA</x:v>
+      </x:c>
+      <x:c r="E113" s="63" t="str">
+        <x:v>Barueri/SP, híbrido</x:v>
+      </x:c>
+      <x:c r="F113" s="63" t="str">
+        <x:v>https://jobs.quickin.io/yssy/apply?job_id=6aa80b234fd9860013f43709</x:v>
+      </x:c>
+      <x:c r="G113" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H113" s="63" t="str">
+        <x:v>Anexar currículo no Quickin e preencher os dados de endereço solicitados; revisar e enviar</x:v>
+      </x:c>
+      <x:c r="I113" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J113" s="63" t="str">
+        <x:v>Alta aderência em Python, SQL, modelagem e integração. A página oficial Quickin exige currículo anexado; o arquivo não pode ser transmitido pelo navegador nesta sessão. Não foram criados dados de endereço inexistentes.</x:v>
+      </x:c>
+      <x:c r="K113" s="63" t="str">
+        <x:v>Não — formulário Quickin não enviado</x:v>
+      </x:c>
+      <x:c r="L113" t="n">
+        <x:f>IF(LEFT(K113,3)="Sim",1,0)+IF(LEFT(K113,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M113" t="n">
+        <x:f>IF(LEFT(A113,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="84" customHeight="1">
+      <x:c r="A114" s="63" t="str">
+        <x:v>Pendente — dados cadastrais</x:v>
+      </x:c>
+      <x:c r="B114" s="63" t="str">
+        <x:v>Cakto Pay</x:v>
+      </x:c>
+      <x:c r="C114" s="63" t="str">
+        <x:v>Desenvolvedor(a) Front-end — Júnior (React.js)</x:v>
+      </x:c>
+      <x:c r="D114" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E114" s="63" t="str">
+        <x:v>Não informado</x:v>
+      </x:c>
+      <x:c r="F114" s="63" t="str">
+        <x:v>https://cakto.vagas.solides.com.br/vaga/880773?origem=indeed</x:v>
+      </x:c>
+      <x:c r="G114" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H114" s="63" t="str">
+        <x:v>Preencher estado civil, endereço completo/CEP e confirmar CNH; depois revisar e enviar</x:v>
+      </x:c>
+      <x:c r="I114" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J114" s="63" t="str">
+        <x:v>Aderência em React de projetos, JavaScript/TypeScript e APIs. Foram mantidos níveis factuais: React intermediário, inglês intermediário e espanhol básico. O Sólides exige estado civil, endereço completo, CEP e informação de CNH, que não foram inventados.</x:v>
+      </x:c>
+      <x:c r="K114" s="63" t="str">
+        <x:v>Não — formulário Sólides não enviado</x:v>
+      </x:c>
+      <x:c r="L114" t="n">
+        <x:f>IF(LEFT(K114,3)="Sim",1,0)+IF(LEFT(K114,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M114" t="n">
+        <x:f>IF(LEFT(A114,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="84" customHeight="1">
+      <x:c r="A115" s="63" t="str">
+        <x:v>Pendente — currículo obrigatório</x:v>
+      </x:c>
+      <x:c r="B115" s="63" t="str">
+        <x:v>Equifax</x:v>
+      </x:c>
+      <x:c r="C115" s="63" t="str">
+        <x:v>Cientista de Dados — Júnior</x:v>
+      </x:c>
+      <x:c r="D115" s="63" t="str">
+        <x:v>Dados e IA</x:v>
+      </x:c>
+      <x:c r="E115" s="63" t="str">
+        <x:v>Barueri/SP</x:v>
+      </x:c>
+      <x:c r="F115" s="63" t="str">
+        <x:v>https://equifax.wd5.myworkdayjobs.com/pt-BR/External/job/BRA-Barueri/Cientista-de-Dados---Jnior_J00178981/apply/applyManually</x:v>
+      </x:c>
+      <x:c r="G115" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H115" s="63" t="str">
+        <x:v>Anexar currículo no Workday; revisar demais campos e enviar</x:v>
+      </x:c>
+      <x:c r="I115" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J115" s="63" t="str">
+        <x:v>Fluxo Workday aberto para Cientista de Dados Júnior. O portal exige currículo anexado e o envio não foi confirmado. A oportunidade segue em controle por ser alinhada a Python, SQL e dados; detalhes de requisito devem ser revisados no retorno.</x:v>
+      </x:c>
+      <x:c r="K115" s="63" t="str">
+        <x:v>Não — formulário Workday não enviado</x:v>
+      </x:c>
+      <x:c r="L115" t="n">
+        <x:f>IF(LEFT(K115,3)="Sim",1,0)+IF(LEFT(K115,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M115" t="n">
+        <x:f>IF(LEFT(A115,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="84" customHeight="1">
+      <x:c r="A116" s="63" t="str">
+        <x:v>Pendente — dados cadastrais</x:v>
+      </x:c>
+      <x:c r="B116" s="63" t="str">
+        <x:v>Construtora Kazza</x:v>
+      </x:c>
+      <x:c r="C116" s="63" t="str">
+        <x:v>Analista de Dados e Automação I</x:v>
+      </x:c>
+      <x:c r="D116" s="63" t="str">
+        <x:v>Dados e automação</x:v>
+      </x:c>
+      <x:c r="E116" s="63" t="str">
+        <x:v>Salvador/BA, presencial ou híbrido conforme anúncio</x:v>
+      </x:c>
+      <x:c r="F116" s="63" t="str">
+        <x:v>https://construtorakazza.vagas.solides.com.br/vaga/916773?origem=indeed</x:v>
+      </x:c>
+      <x:c r="G116" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H116" s="63" t="str">
+        <x:v>Preencher endereço completo e confirmar CNH; depois revisar e enviar</x:v>
+      </x:c>
+      <x:c r="I116" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J116" s="63" t="str">
+        <x:v>Faixa divulgada de R$4.000–4.800 CLT. Formulário Sólides requer endereço completo e informação de CNH. Esses dados não foram fornecidos, portanto a candidatura não foi enviada.</x:v>
+      </x:c>
+      <x:c r="K116" s="63" t="str">
+        <x:v>Não — formulário Sólides não enviado</x:v>
+      </x:c>
+      <x:c r="L116" t="n">
+        <x:f>IF(LEFT(K116,3)="Sim",1,0)+IF(LEFT(K116,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M116" t="n">
+        <x:f>IF(LEFT(A116,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="84" customHeight="1">
+      <x:c r="A117" s="32" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B117" s="63" t="str">
+        <x:v>Terram Engenharia</x:v>
+      </x:c>
+      <x:c r="C117" s="63" t="str">
+        <x:v>Analista de Dados Jr</x:v>
+      </x:c>
+      <x:c r="D117" s="63" t="str">
+        <x:v>Dados e IA</x:v>
+      </x:c>
+      <x:c r="E117" s="63" t="str">
+        <x:v>Barueri/SP, presencial</x:v>
+      </x:c>
+      <x:c r="F117" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G117" s="63" t="str">
+        <x:v>Fit Cultural na etapa seguinte; formato não informado</x:v>
+      </x:c>
+      <x:c r="H117" s="63" t="str">
+        <x:v>Acompanhar e-mail; validar o formato antes de iniciar qualquer etapa</x:v>
+      </x:c>
+      <x:c r="I117" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J117" s="63" t="str">
+        <x:v>Candidatura finalizada e confirmada na Gupy em 30/09. Personalização destacou Python, SQL/PostgreSQL, APIs, automações, Excel, dados e documentação; Power BI foi mencionado apenas como tema em aprofundamento. RG, filiação, última remuneração e pretensão foram informados de forma factual. Habilidades destacadas: Python, SQL e PostgreSQL.</x:v>
+      </x:c>
+      <x:c r="K117" s="63" t="str">
+        <x:v>Portal — confirmação Gupy 30/09</x:v>
+      </x:c>
+      <x:c r="L117" t="n">
+        <x:f>IF(LEFT(K117,3)="Sim",1,0)+IF(LEFT(K117,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M117" t="n">
+        <x:f>IF(LEFT(A117,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="84" customHeight="1">
+      <x:c r="A118" s="63" t="str">
+        <x:v>Pendente — reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="B118" s="63" t="str">
+        <x:v>AM53 Tech Recruitment</x:v>
+      </x:c>
+      <x:c r="C118" s="63" t="str">
+        <x:v>Desenvolvedor(a) Júnior — Python &amp; Data Analytics</x:v>
+      </x:c>
+      <x:c r="D118" s="63" t="str">
+        <x:v>Dados e automação</x:v>
+      </x:c>
+      <x:c r="E118" s="63" t="str">
+        <x:v>São Paulo/SP</x:v>
+      </x:c>
+      <x:c r="F118" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=7935544f2ce38078</x:v>
+      </x:c>
+      <x:c r="G118" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H118" s="63" t="str">
+        <x:v>Abrir em Minhas Vagas no Indeed e concluir o reCAPTCHA/Enviar pessoalmente</x:v>
+      </x:c>
+      <x:c r="I118" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J118" s="63" t="str">
+        <x:v>Candidatura personalizada preparada a 100% no Indeed com currículo anexado e carta focada em Python, SQL/PostgreSQL, APIs, Docker, Git, Excel, tratamento de dados e automações. O botão final não ficou disponível por reCAPTCHA; não foi contornado.</x:v>
+      </x:c>
+      <x:c r="K118" s="63" t="str">
+        <x:v>Não — rascunho 100% no Indeed</x:v>
+      </x:c>
+      <x:c r="L118" t="n">
+        <x:f>IF(LEFT(K118,3)="Sim",1,0)+IF(LEFT(K118,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M118" t="n">
+        <x:f>IF(LEFT(A118,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="84" customHeight="1">
+      <x:c r="A119" s="63" t="str">
+        <x:v>Pendente — reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="B119" s="63" t="str">
+        <x:v>COBRAPE</x:v>
+      </x:c>
+      <x:c r="C119" s="63" t="str">
+        <x:v>Programador Junior</x:v>
+      </x:c>
+      <x:c r="D119" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E119" s="63" t="str">
+        <x:v>São Paulo/SP, CLT</x:v>
+      </x:c>
+      <x:c r="F119" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=bee9e87a7c8f21a6</x:v>
+      </x:c>
+      <x:c r="G119" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H119" s="63" t="str">
+        <x:v>Concluir o reCAPTCHA/Enviar no Indeed quando o botão final estiver habilitado</x:v>
+      </x:c>
+      <x:c r="I119" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J119" s="63" t="str">
+        <x:v>Vaga aderente em C#/.NET e banco relacional. O Indeed abriu a candidatura já a 100%, mas o botão de envio permaneceu desabilitado por reCAPTCHA. O salvamento foi solicitado, porém a plataforma não exibiu confirmação de saída; não houve candidatura enviada.</x:v>
+      </x:c>
+      <x:c r="K119" s="63" t="str">
+        <x:v>Não — envio final bloqueado no Indeed</x:v>
+      </x:c>
+      <x:c r="L119" t="n">
+        <x:f>IF(LEFT(K119,3)="Sim",1,0)+IF(LEFT(K119,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M119" t="n">
+        <x:f>IF(LEFT(A119,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="92" customHeight="1">
+      <x:c r="A120" s="32" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B120" s="63" t="str">
+        <x:v>Conviso Application Security</x:v>
+      </x:c>
+      <x:c r="C120" s="63" t="str">
+        <x:v>Junior/Pleno Front-End Engineer</x:v>
+      </x:c>
+      <x:c r="D120" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E120" s="63" t="str">
+        <x:v>Remoto</x:v>
+      </x:c>
+      <x:c r="F120" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G120" s="63" t="str">
+        <x:v>Sem audiovisual declarado; etapas futuras não verificadas</x:v>
+      </x:c>
+      <x:c r="H120" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal; validar o formato de qualquer etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="I120" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J120" s="63" t="str">
+        <x:v>Candidatura personalizada e finalizada na Gupy. Destacou JavaScript/TypeScript, React de projetos, Python/FastAPI, C#/.NET, APIs REST, PostgreSQL, Docker, Git e testes; Vue foi tratado como aprendizado, não experiência em produção. Pretensão: R$5–6 mil CLT, negociável conforme escopo e benefícios.</x:v>
+      </x:c>
+      <x:c r="K120" s="63" t="str">
+        <x:v>Portal — confirmação Gupy 30/09</x:v>
+      </x:c>
+      <x:c r="L120" t="n">
+        <x:f>IF(LEFT(K120,3)="Sim",1,0)+IF(LEFT(K120,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M120" t="n">
+        <x:f>IF(LEFT(A120,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="92" customHeight="1">
+      <x:c r="A121" s="63" t="str">
+        <x:v>Pendente — questionário técnico</x:v>
+      </x:c>
+      <x:c r="B121" s="63" t="str">
+        <x:v>Vertigo Tecnologia</x:v>
+      </x:c>
+      <x:c r="C121" s="63" t="str">
+        <x:v>Analista de IA — Júnior</x:v>
+      </x:c>
+      <x:c r="D121" s="63" t="str">
+        <x:v>Dados e IA</x:v>
+      </x:c>
+      <x:c r="E121" s="63" t="str">
+        <x:v>Remoto</x:v>
+      </x:c>
+      <x:c r="F121" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=4ecd51d1ae592034</x:v>
+      </x:c>
+      <x:c r="G121" s="63" t="str">
+        <x:v>Questionário técnico escrito; sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H121" s="63" t="str">
+        <x:v>Responder pessoalmente ao questionário técnico e concluir o envio no Indeed</x:v>
+      </x:c>
+      <x:c r="I121" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J121" s="63" t="str">
+        <x:v>Rascunho salvo a 50% com currículo, LinkedIn, pretensão de R$6.000 e disponibilidade remota. Restam perguntas técnicas de múltipla escolha sobre AWS, critérios de aceitação e requisitos; não foram respondidas nesta sessão.</x:v>
+      </x:c>
+      <x:c r="K121" s="63" t="str">
+        <x:v>Não — rascunho salvo no Indeed</x:v>
+      </x:c>
+      <x:c r="L121" t="n">
+        <x:f>IF(LEFT(K121,3)="Sim",1,0)+IF(LEFT(K121,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M121" t="n">
+        <x:f>IF(LEFT(A121,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="92" customHeight="1">
+      <x:c r="A122" s="63" t="str">
+        <x:v>Pendente — questionário técnico</x:v>
+      </x:c>
+      <x:c r="B122" s="63" t="str">
+        <x:v>Extractta</x:v>
+      </x:c>
+      <x:c r="C122" s="63" t="str">
+        <x:v>Desenvolvedor Backend Júnior C# / .NET</x:v>
+      </x:c>
+      <x:c r="D122" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E122" s="63" t="str">
+        <x:v>Remoto; estágio</x:v>
+      </x:c>
+      <x:c r="F122" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=9e455e565eb371b9</x:v>
+      </x:c>
+      <x:c r="G122" s="63" t="str">
+        <x:v>Questionário técnico escrito; sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H122" s="63" t="str">
+        <x:v>Responder pessoalmente ao questionário técnico e concluir o envio no Indeed</x:v>
+      </x:c>
+      <x:c r="I122" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J122" s="63" t="str">
+        <x:v>Rascunho salvo a 50% com currículo, LinkedIn, pretensão de R$4.000 e respostas factuais. Restam questões técnicas sobre qualidade de código, SQL/índices, APIs REST seguras e fluxo Git; não foram respondidas nesta sessão.</x:v>
+      </x:c>
+      <x:c r="K122" s="63" t="str">
+        <x:v>Não — rascunho salvo no Indeed</x:v>
+      </x:c>
+      <x:c r="L122" t="n">
+        <x:f>IF(LEFT(K122,3)="Sim",1,0)+IF(LEFT(K122,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M122" t="n">
+        <x:f>IF(LEFT(A122,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="92" customHeight="1">
+      <x:c r="A123" s="63" t="str">
+        <x:v>Pendente — Profiler comportamental</x:v>
+      </x:c>
+      <x:c r="B123" s="63" t="str">
+        <x:v>ELA DECORA</x:v>
+      </x:c>
+      <x:c r="C123" s="63" t="str">
+        <x:v>Desenvolvedor(a) Full Stack Júnior | IA + SaaS</x:v>
+      </x:c>
+      <x:c r="D123" s="63" t="str">
+        <x:v>Desenvolvimento e IA</x:v>
+      </x:c>
+      <x:c r="E123" s="63" t="str">
+        <x:v>Bauru/SP; CLT/PJ</x:v>
+      </x:c>
+      <x:c r="F123" s="63" t="str">
+        <x:v>https://eladecora.vagas.solides.com.br/vaga/888981?origem=indeed</x:v>
+      </x:c>
+      <x:c r="G123" s="63" t="str">
+        <x:v>Profiler comportamental obrigatório; formato audiovisual não confirmado</x:v>
+      </x:c>
+      <x:c r="H123" s="63" t="str">
+        <x:v>Concluir o Profiler pessoalmente e revisar a candidatura</x:v>
+      </x:c>
+      <x:c r="I123" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J123" s="63" t="str">
+        <x:v>Login com Google realizado; a Sólides exige o Profiler antes de salvar a candidatura. Não houve candidatura confirmada. A vaga é aderente a TypeScript, React/Node de projetos, SQL, Git, Docker e APIs.</x:v>
+      </x:c>
+      <x:c r="K123" s="63" t="str">
+        <x:v>Não — candidatura não salva (Profiler obrigatório)</x:v>
+      </x:c>
+      <x:c r="L123" t="n">
+        <x:f>IF(LEFT(K123,3)="Sim",1,0)+IF(LEFT(K123,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M123" t="n">
+        <x:f>IF(LEFT(A123,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="92" customHeight="1">
+      <x:c r="A124" s="63" t="str">
+        <x:v>Pendente — Profiler comportamental</x:v>
+      </x:c>
+      <x:c r="B124" s="63" t="str">
+        <x:v>UNIX Logística</x:v>
+      </x:c>
+      <x:c r="C124" s="63" t="str">
+        <x:v>Desenvolvedor Júnior de Automação, Integrações e IA</x:v>
+      </x:c>
+      <x:c r="D124" s="63" t="str">
+        <x:v>Automação, integrações e IA</x:v>
+      </x:c>
+      <x:c r="E124" s="63" t="str">
+        <x:v>São Paulo/SP, presencial</x:v>
+      </x:c>
+      <x:c r="F124" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=07d8ef0b1c75ef31</x:v>
+      </x:c>
+      <x:c r="G124" s="63" t="str">
+        <x:v>Profiler comportamental obrigatório; formato audiovisual não confirmado</x:v>
+      </x:c>
+      <x:c r="H124" s="63" t="str">
+        <x:v>Concluir o Profiler pessoalmente e revisar a candidatura</x:v>
+      </x:c>
+      <x:c r="I124" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J124" s="63" t="str">
+        <x:v>Vaga CLT com salário divulgado de R$4.500. A Sólides exige o Profiler antes de salvar a candidatura; não houve candidatura confirmada. Boa aderência em Python, APIs, SQL, Docker e IA; n8n é tema de estudo.</x:v>
+      </x:c>
+      <x:c r="K124" s="63" t="str">
+        <x:v>Não — candidatura não salva (Profiler obrigatório)</x:v>
+      </x:c>
+      <x:c r="L124" t="n">
+        <x:f>IF(LEFT(K124,3)="Sim",1,0)+IF(LEFT(K124,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M124" t="n">
+        <x:f>IF(LEFT(A124,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="92" customHeight="1">
+      <x:c r="A125" s="63" t="str">
+        <x:v>Pendente — currículo obrigatório</x:v>
+      </x:c>
+      <x:c r="B125" s="63" t="str">
+        <x:v>Overlabs</x:v>
+      </x:c>
+      <x:c r="C125" s="63" t="str">
+        <x:v>Desenvolvedor FullStack (Node/React)</x:v>
+      </x:c>
+      <x:c r="D125" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E125" s="63" t="str">
+        <x:v>Remoto; PJ</x:v>
+      </x:c>
+      <x:c r="F125" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=741b4fd7fbcf3396</x:v>
+      </x:c>
+      <x:c r="G125" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H125" s="63" t="str">
+        <x:v>Anexar CV no formulário Mindsight, revisar os dados e enviar</x:v>
+      </x:c>
+      <x:c r="I125" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J125" s="63" t="str">
+        <x:v>Formulário externo exige anexo de currículo; não houve envio nem salvamento confirmado. Aderência em Node/React de projetos, TypeScript, APIs, SQL, Git e Docker.</x:v>
+      </x:c>
+      <x:c r="K125" s="63" t="str">
+        <x:v>Não — formulário Mindsight não enviado</x:v>
+      </x:c>
+      <x:c r="L125" t="n">
+        <x:f>IF(LEFT(K125,3)="Sim",1,0)+IF(LEFT(K125,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M125" t="n">
+        <x:f>IF(LEFT(A125,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="92" customHeight="1">
+      <x:c r="A126" s="63" t="str">
+        <x:v>Pendente — currículo obrigatório</x:v>
+      </x:c>
+      <x:c r="B126" s="63" t="str">
+        <x:v>Datum</x:v>
+      </x:c>
+      <x:c r="C126" s="63" t="str">
+        <x:v>Pessoa Engenheira de Dados Júnior</x:v>
+      </x:c>
+      <x:c r="D126" s="63" t="str">
+        <x:v>Dados e IA</x:v>
+      </x:c>
+      <x:c r="E126" s="63" t="str">
+        <x:v>Remoto</x:v>
+      </x:c>
+      <x:c r="F126" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=3828c5fb1a294d79</x:v>
+      </x:c>
+      <x:c r="G126" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H126" s="63" t="str">
+        <x:v>Anexar CV no formulário externo, revisar os dados e enviar</x:v>
+      </x:c>
+      <x:c r="I126" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J126" s="63" t="str">
+        <x:v>Formulário externo exige currículo anexado; não houve envio nem salvamento confirmado. Aderência em Python, SQL, Git e conceitos de GCP, com prática de dados e integrações em projetos.</x:v>
+      </x:c>
+      <x:c r="K126" s="63" t="str">
+        <x:v>Não — formulário externo não enviado</x:v>
+      </x:c>
+      <x:c r="L126" t="n">
+        <x:f>IF(LEFT(K126,3)="Sim",1,0)+IF(LEFT(K126,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M126" t="n">
+        <x:f>IF(LEFT(A126,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="92" customHeight="1">
+      <x:c r="A127" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B127" s="63" t="str">
+        <x:v>AuthSoft (via Jobbol)</x:v>
+      </x:c>
+      <x:c r="C127" s="63" t="str">
+        <x:v>Desenvolvedor Júnior</x:v>
+      </x:c>
+      <x:c r="D127" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E127" s="63" t="str">
+        <x:v>Remoto; Salvador/BA</x:v>
+      </x:c>
+      <x:c r="F127" s="63" t="str">
+        <x:v>https://www.jobbol.com.br/vaga/29386875985</x:v>
+      </x:c>
+      <x:c r="G127" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H127" s="63" t="str">
+        <x:v>Acompanhar o e-mail e o portal Jobbol; validar o formato de qualquer próxima etapa</x:v>
+      </x:c>
+      <x:c r="I127" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J127" s="63" t="str">
+        <x:v>Candidatura enviada pelo fluxo originado no Indeed, com currículo anexado e dados revisados. Confirmação exibida com protocolo LK9591784. Vaga de entrada para C#/.NET, WinForms, SQL Server/PostgreSQL, Git, testes e código legado; salário da vaga não foi divulgado, e a página mostra apenas média estimada local de R$3.500.</x:v>
+      </x:c>
+      <x:c r="K127" s="63" t="str">
+        <x:v>Sim — protocolo Jobbol LK9591784 30/09</x:v>
+      </x:c>
+      <x:c r="L127" t="n">
+        <x:f>IF(LEFT(K127,3)="Sim",1,0)+IF(LEFT(K127,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M127" t="n">
+        <x:f>IF(LEFT(A127,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="92" customHeight="1">
+      <x:c r="A128" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B128" s="63" t="str">
+        <x:v>Construmarket</x:v>
+      </x:c>
+      <x:c r="C128" s="63" t="str">
+        <x:v>Desenvolvedor(a) Júnior</x:v>
+      </x:c>
+      <x:c r="D128" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E128" s="63" t="str">
+        <x:v>Remoto</x:v>
+      </x:c>
+      <x:c r="F128" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G128" s="63" t="str">
+        <x:v>Fit Cultural e teste técnico previstos; formato audiovisual não informado</x:v>
+      </x:c>
+      <x:c r="H128" s="63" t="str">
+        <x:v>Acompanhar e-mail; realizar pessoalmente qualquer avaliação e validar o formato antes de iniciar</x:v>
+      </x:c>
+      <x:c r="I128" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J128" s="63" t="str">
+        <x:v>Candidatura personalizada e finalizada na Gupy. Destacou projetos próprios em C#/.NET, TypeScript, React, SQL/PostgreSQL, Git, Docker e testes. Angular e AngularJS foram apresentados como tecnologias em estudo para o legado, não como experiência consolidada.</x:v>
+      </x:c>
+      <x:c r="K128" s="63" t="str">
+        <x:v>Portal — confirmação Gupy 30/09</x:v>
+      </x:c>
+      <x:c r="L128" t="n">
+        <x:f>IF(LEFT(K128,3)="Sim",1,0)+IF(LEFT(K128,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M128" t="n">
+        <x:f>IF(LEFT(A128,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="92" customHeight="1">
+      <x:c r="A129" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B129" s="63" t="str">
+        <x:v>Libbs Farmacêutica (Oficial)</x:v>
+      </x:c>
+      <x:c r="C129" s="63" t="str">
+        <x:v>Desenvolvedor de Automação e IA Jr</x:v>
+      </x:c>
+      <x:c r="D129" s="63" t="str">
+        <x:v>Automação e IA</x:v>
+      </x:c>
+      <x:c r="E129" s="63" t="str">
+        <x:v>Remoto</x:v>
+      </x:c>
+      <x:c r="F129" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G129" s="63" t="str">
+        <x:v>Etapas futuras incluem abordagem telefônica, entrevista e case; formato audiovisual do case não informado</x:v>
+      </x:c>
+      <x:c r="H129" s="63" t="str">
+        <x:v>Acompanhar e-mail; validar formato e realizar pessoalmente qualquer case ou etapa de entrevista</x:v>
+      </x:c>
+      <x:c r="I129" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J129" s="63" t="str">
+        <x:v>Candidatura personalizada e finalizada na Gupy antes do encerramento. Destacou Python/FastAPI, C#/.NET, SQL/PostgreSQL, APIs, Docker, Git, testes, logs e automação; RPA, BPM, Power Automate e Lecom foram tratados como temas de aprendizado.</x:v>
+      </x:c>
+      <x:c r="K129" s="63" t="str">
+        <x:v>Portal — confirmação Gupy 30/09</x:v>
+      </x:c>
+      <x:c r="L129" t="n">
+        <x:f>IF(LEFT(K129,3)="Sim",1,0)+IF(LEFT(K129,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M129" t="n">
+        <x:f>IF(LEFT(A129,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="92" customHeight="1">
+      <x:c r="A130" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B130" s="63" t="str">
+        <x:v>Bellinati Perez</x:v>
+      </x:c>
+      <x:c r="C130" s="63" t="str">
+        <x:v>Analista de Dados Júnior</x:v>
+      </x:c>
+      <x:c r="D130" s="63" t="str">
+        <x:v>Dados e IA</x:v>
+      </x:c>
+      <x:c r="E130" s="63" t="str">
+        <x:v>Curitiba/PR, presencial</x:v>
+      </x:c>
+      <x:c r="F130" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G130" s="63" t="str">
+        <x:v>Teste técnico previsto; sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H130" s="63" t="str">
+        <x:v>Acompanhar e-mail; realizar pessoalmente qualquer teste e validar o formato antes de iniciar</x:v>
+      </x:c>
+      <x:c r="I130" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J130" s="63" t="str">
+        <x:v>Candidatura personalizada e finalizada na Gupy. Declarou Excel avançado, Python, SQL/PostgreSQL, APIs e integração de dados de projetos. A experiência em BI/Power BI foi informada com transparência como área de aprendizado; disponibilidade presencial em Curitiba foi confirmada.</x:v>
+      </x:c>
+      <x:c r="K130" s="63" t="str">
+        <x:v>Portal — confirmação Gupy 30/09</x:v>
+      </x:c>
+      <x:c r="L130" t="n">
+        <x:f>IF(LEFT(K130,3)="Sim",1,0)+IF(LEFT(K130,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M130" t="n">
+        <x:f>IF(LEFT(A130,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="92" customHeight="1">
+      <x:c r="A131" s="63" t="str">
+        <x:v>Pendente — vídeo obrigatório</x:v>
+      </x:c>
+      <x:c r="B131" s="63" t="str">
+        <x:v>PERILLO ENGENHARIA LTDA</x:v>
+      </x:c>
+      <x:c r="C131" s="63" t="str">
+        <x:v>Desenvolvedor Full Stack Jr</x:v>
+      </x:c>
+      <x:c r="D131" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E131" s="63" t="str">
+        <x:v>Piracicaba/SP, presencial; PJ</x:v>
+      </x:c>
+      <x:c r="F131" s="63" t="str">
+        <x:v>https://perillojobs.vagas.solides.com.br/vaga/840448?origem=indeed</x:v>
+      </x:c>
+      <x:c r="G131" s="63" t="str">
+        <x:v>Vídeo de apresentação obrigatório</x:v>
+      </x:c>
+      <x:c r="H131" s="63" t="str">
+        <x:v>Gravar e enviar a apresentação pessoalmente; revisar RG antes de concluir a candidatura</x:v>
+      </x:c>
+      <x:c r="I131" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J131" s="63" t="str">
+        <x:v>Vaga de R$5.000–6.000 PJ com aderência alta em TypeScript/Node, React, PostgreSQL, REST, Git, Docker, CI/CD e testes. O portal exige vídeo de apresentação e RG como campos obrigatórios; a candidatura não foi concluída para respeitar o protocolo audiovisual.</x:v>
+      </x:c>
+      <x:c r="K131" s="63" t="str">
+        <x:v>Não — candidatura não concluída (vídeo obrigatório)</x:v>
+      </x:c>
+      <x:c r="L131" t="n">
+        <x:f>IF(LEFT(K131,3)="Sim",1,0)+IF(LEFT(K131,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M131" t="n">
+        <x:f>IF(LEFT(A131,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="92" customHeight="1">
+      <x:c r="A132" s="32" t="str">
+        <x:v>Pendente — dados cadastrais</x:v>
+      </x:c>
+      <x:c r="B132" s="63" t="str">
+        <x:v>Avanade (Accenture)</x:v>
+      </x:c>
+      <x:c r="C132" s="63" t="str">
+        <x:v>Desenvolvedor(a) FullStack Junior</x:v>
+      </x:c>
+      <x:c r="D132" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E132" s="63" t="str">
+        <x:v>São Paulo/SP</x:v>
+      </x:c>
+      <x:c r="F132" s="63" t="str">
+        <x:v>https://accenture.wd103.myworkdayjobs.com/pt-BR/AvanadeCareers/job/Sao-Paulo-Torre-Paineira/Desenvolvedor-a--FullStack_R00352707/apply</x:v>
+      </x:c>
+      <x:c r="G132" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H132" s="63" t="str">
+        <x:v>Preencher endereço completo no Workday, revisar os dados e enviar</x:v>
+      </x:c>
+      <x:c r="I132" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J132" s="63" t="str">
+        <x:v>Fluxo originado no Indeed. Login com Google concluído no Workday, mas a candidatura exige endereço completo (logradouro, cidade, bairro, estado e CEP) antes de salvar. Esses dados não foram fornecidos nem inventados. Alta aderência em C#/.NET, React, TypeScript, APIs REST, SQL, testes e Git; Azure DevOps é tema de aprendizado.</x:v>
+      </x:c>
+      <x:c r="K132" s="63" t="str">
+        <x:v>Não — formulário Workday não enviado</x:v>
+      </x:c>
+      <x:c r="L132" t="n">
+        <x:f>IF(LEFT(K132,3)="Sim",1,0)+IF(LEFT(K132,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M132" t="n">
+        <x:f>IF(LEFT(A132,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="92" customHeight="1">
+      <x:c r="A133" s="32" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B133" s="63" t="str">
+        <x:v>Vagas MRM Brasil</x:v>
+      </x:c>
+      <x:c r="C133" s="63" t="str">
+        <x:v>Desenvolvedor Fullstack Jr</x:v>
+      </x:c>
+      <x:c r="D133" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E133" s="63" t="str">
+        <x:v>São Paulo/SP, híbrido (3x por semana; Vila Madalena)</x:v>
+      </x:c>
+      <x:c r="F133" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G133" s="63" t="str">
+        <x:v>Entrevistas técnica e de RH previstas; sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H133" s="63" t="str">
+        <x:v>Acompanhar e-mail; validar formato de cada etapa e realizar pessoalmente qualquer entrevista ou avaliação</x:v>
+      </x:c>
+      <x:c r="I133" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J133" s="63" t="str">
+        <x:v>Candidatura personalizada e finalizada na Gupy em 30/09. A vaga aceita primeira experiência técnica e projetos pessoais. O texto destacou APIs REST, integrações, SQL/PostgreSQL, Docker, Git, testes, C#/.NET, Python/FastAPI, JavaScript/TypeScript e uso criterioso de IA. Disponibilidade híbrida confirmada; inglês intermediário e pretensão a partir de R$3 mil foram informados.</x:v>
+      </x:c>
+      <x:c r="K133" s="63" t="str">
+        <x:v>Portal — confirmação Gupy 30/09</x:v>
+      </x:c>
+      <x:c r="L133" t="n">
+        <x:f>IF(LEFT(K133,3)="Sim",1,0)+IF(LEFT(K133,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M133" t="n">
+        <x:f>IF(LEFT(A133,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134" ht="92" customHeight="1">
+      <x:c r="A134" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B134" s="63" t="str">
+        <x:v>Instituto de Pesquisas Eldorado</x:v>
+      </x:c>
+      <x:c r="C134" s="63" t="str">
+        <x:v>Pessoa desenvolvedora Machine Learning</x:v>
+      </x:c>
+      <x:c r="D134" s="63" t="str">
+        <x:v>Dados e IA</x:v>
+      </x:c>
+      <x:c r="E134" s="63" t="str">
+        <x:v>Brasília/DF, híbrido (2x presencial; mudança disponível)</x:v>
+      </x:c>
+      <x:c r="F134" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G134" s="63" t="str">
+        <x:v>Entrevistas com área e RH previstas; sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H134" s="63" t="str">
+        <x:v>Acompanhar e-mail; validar formato e realizar pessoalmente qualquer entrevista ou avaliação</x:v>
+      </x:c>
+      <x:c r="I134" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J134" s="63" t="str">
+        <x:v>Candidatura personalizada e finalizada na Gupy. Apresentação transparente: Python, APIs, SQL/PostgreSQL, dados, Docker, cloud e IA aplicada; bibliotecas e modelagem de ML estão em aprofundamento, sem alegar experiência profissional em ML. Habilidades: Python, SQL e Google Cloud Platform. Disponibilidade híbrida e mudança confirmadas; pretensão a partir de R$3 mil.</x:v>
+      </x:c>
+      <x:c r="K134" s="63" t="str">
+        <x:v>Portal — confirmação Gupy 30/09</x:v>
+      </x:c>
+      <x:c r="L134" t="n">
+        <x:f>IF(LEFT(K134,3)="Sim",1,0)+IF(LEFT(K134,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M134" t="n">
+        <x:f>IF(LEFT(A134,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="92" customHeight="1">
+      <x:c r="A135" s="63" t="str">
+        <x:v>Pendente — reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="B135" s="63" t="str">
+        <x:v>Lyncas</x:v>
+      </x:c>
+      <x:c r="C135" s="63" t="str">
+        <x:v>Desenvolvedor FullStack Júnior | Node e React</x:v>
+      </x:c>
+      <x:c r="D135" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E135" s="63" t="str">
+        <x:v>São Paulo/SP, híbrido</x:v>
+      </x:c>
+      <x:c r="F135" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=6e7370b4d29e3b69</x:v>
+      </x:c>
+      <x:c r="G135" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H135" s="63" t="str">
+        <x:v>Abrir em Minhas Vagas no Indeed, concluir o reCAPTCHA normal e enviar pessoalmente</x:v>
+      </x:c>
+      <x:c r="I135" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J135" s="63" t="str">
+        <x:v>Candidatura personalizada chegou a 100% no Indeed e foi salva por 14 dias. Currículo selecionado; dados factuais: ADS em andamento, React/Next e Node/Nest em projetos (menos de um ano), foco principal em backend, Git, Docker, GCP, testes e IA/ChatGPT. Pretensão registrada em R$3.000 PJ e CLT; envio final bloqueado por reCAPTCHA, não contornado.</x:v>
+      </x:c>
+      <x:c r="K135" s="63" t="str">
+        <x:v>Não — rascunho 100% no Indeed</x:v>
+      </x:c>
+      <x:c r="L135" t="n">
+        <x:f>IF(LEFT(K135,3)="Sim",1,0)+IF(LEFT(K135,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M135" t="n">
+        <x:f>IF(LEFT(A135,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" ht="92" customHeight="1">
+      <x:c r="A136" s="63" t="str">
+        <x:v>Pendente — reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="B136" s="63" t="str">
+        <x:v>Valor Real Empreendimentos</x:v>
+      </x:c>
+      <x:c r="C136" s="63" t="str">
+        <x:v>Desenvolvedor Full Stack Júnior</x:v>
+      </x:c>
+      <x:c r="D136" s="63" t="str">
+        <x:v>Desenvolvimento e IA</x:v>
+      </x:c>
+      <x:c r="E136" s="63" t="str">
+        <x:v>Curitiba/PR, presencial; PJ</x:v>
+      </x:c>
+      <x:c r="F136" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=5d3f5ace8e47efff</x:v>
+      </x:c>
+      <x:c r="G136" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H136" s="63" t="str">
+        <x:v>Abrir em Minhas Vagas no Indeed, concluir o reCAPTCHA normal e enviar pessoalmente</x:v>
+      </x:c>
+      <x:c r="I136" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J136" s="63" t="str">
+        <x:v>Candidatura personalizada chegou a 100% no Indeed e foi salva por 14 dias. Perfil e respostas factuais destacaram JavaScript/TypeScript, React, SQL/PostgreSQL, APIs REST, Git, Python, Docker, Linux e IA/LLM em projetos. Salário informado de R$3.000 e disponibilidade para Curitiba; envio final bloqueado por reCAPTCHA, não contornado.</x:v>
+      </x:c>
+      <x:c r="K136" s="63" t="str">
+        <x:v>Não — rascunho 100% no Indeed</x:v>
+      </x:c>
+      <x:c r="L136" t="n">
+        <x:f>IF(LEFT(K136,3)="Sim",1,0)+IF(LEFT(K136,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M136" t="n">
+        <x:f>IF(LEFT(A136,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" ht="92" customHeight="1">
+      <x:c r="A137" s="63" t="str">
+        <x:v>Pendente — reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="B137" s="63" t="str">
+        <x:v>Luby</x:v>
+      </x:c>
+      <x:c r="C137" s="63" t="str">
+        <x:v>Profissional Fullstack (IA/Javascript) Trainee/Júnior</x:v>
+      </x:c>
+      <x:c r="D137" s="63" t="str">
+        <x:v>Desenvolvimento e IA</x:v>
+      </x:c>
+      <x:c r="E137" s="63" t="str">
+        <x:v>Remoto</x:v>
+      </x:c>
+      <x:c r="F137" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=553ff80e554c6463</x:v>
+      </x:c>
+      <x:c r="G137" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H137" s="63" t="str">
+        <x:v>Abrir em Minhas Vagas no Indeed, concluir o reCAPTCHA normal e enviar pessoalmente</x:v>
+      </x:c>
+      <x:c r="I137" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J137" s="63" t="str">
+        <x:v>Candidatura chegou a 100% no Indeed com currículo técnico selecionado e respostas previamente revisadas. O envio final foi bloqueado por reCAPTCHA; o rascunho foi salvo por 14 dias e a verificação não foi contornada.</x:v>
+      </x:c>
+      <x:c r="K137" s="63" t="str">
+        <x:v>Não — rascunho 100% no Indeed</x:v>
+      </x:c>
+      <x:c r="L137" t="n">
+        <x:f>IF(LEFT(K137,3)="Sim",1,0)+IF(LEFT(K137,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M137" t="n">
+        <x:f>IF(LEFT(A137,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138" ht="92" customHeight="1">
+      <x:c r="A138" s="63" t="str">
+        <x:v>Pendente — falha de formulário</x:v>
+      </x:c>
+      <x:c r="B138" s="63" t="str">
+        <x:v>ISA Saúde</x:v>
+      </x:c>
+      <x:c r="C138" s="63" t="str">
+        <x:v>Desenvolvedor(a) Full Stack</x:v>
+      </x:c>
+      <x:c r="D138" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E138" s="63" t="str">
+        <x:v>Não informado</x:v>
+      </x:c>
+      <x:c r="F138" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G138" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H138" s="63" t="str">
+        <x:v>Retomar no portal Gupy; a página de perguntas da empresa não carregou</x:v>
+      </x:c>
+      <x:c r="I138" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J138" s="63" t="str">
+        <x:v>A vaga tem aderência em JavaScript/TypeScript, React/Next, Node, APIs e PostgreSQL. Dados iniciais foram preenchidos de forma factual, mas a página de perguntas personalizadas ficou em branco e não avançou após salvar. Nenhuma candidatura finalizada foi confirmada.</x:v>
+      </x:c>
+      <x:c r="K138" s="63" t="str">
+        <x:v>Não — plataforma não avançou</x:v>
+      </x:c>
+      <x:c r="L138" t="n">
+        <x:f>IF(LEFT(K138,3)="Sim",1,0)+IF(LEFT(K138,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M138" t="n">
+        <x:f>IF(LEFT(A138,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139" ht="92" customHeight="1">
+      <x:c r="A139" s="63" t="str">
+        <x:v>Pendente — CNH a confirmar</x:v>
+      </x:c>
+      <x:c r="B139" s="63" t="str">
+        <x:v>ZOUPHY Tecnologia</x:v>
+      </x:c>
+      <x:c r="C139" s="63" t="str">
+        <x:v>Desenvolvedor Front-end (React)</x:v>
+      </x:c>
+      <x:c r="D139" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E139" s="63" t="str">
+        <x:v>Barueri/SP, híbrido (3x2); Cooperado</x:v>
+      </x:c>
+      <x:c r="F139" s="63" t="str">
+        <x:v>https://zouphy.vagas.solides.com.br/vaga/518220?origem=indeed</x:v>
+      </x:c>
+      <x:c r="G139" s="63" t="str">
+        <x:v>Vídeo de apresentação opcional; não iniciado</x:v>
+      </x:c>
+      <x:c r="H139" s="63" t="str">
+        <x:v>Confirmar se possui CNH válida e informar pretensão antes de concluir; manter vídeo opcional sem iniciar</x:v>
+      </x:c>
+      <x:c r="I139" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J139" s="63" t="str">
+        <x:v>Perfil Sólides revisado com dados factuais e nome completo corrigido. A vaga é aderente a JavaScript/TypeScript, React de projetos, Git, Docker e CI/CD. A plataforma exige CNH válida e pretensão salarial; como a informação de CNH não foi fornecida, a candidatura não foi enviada.</x:v>
+      </x:c>
+      <x:c r="K139" s="63" t="str">
+        <x:v>Não — CNH obrigatória não confirmada</x:v>
+      </x:c>
+      <x:c r="L139" t="n">
+        <x:f>IF(LEFT(K139,3)="Sim",1,0)+IF(LEFT(K139,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M139" t="n">
+        <x:f>IF(LEFT(A139,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140" ht="94" customHeight="1">
+      <x:c r="A140" s="32" t="str">
+        <x:v>Pendente — reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="B140" s="63" t="str">
+        <x:v>Engemoura Tecnologia Energética</x:v>
+      </x:c>
+      <x:c r="C140" s="63" t="str">
+        <x:v>Desenvolvedor</x:v>
+      </x:c>
+      <x:c r="D140" s="63" t="str">
+        <x:v>Desenvolvimento e automação</x:v>
+      </x:c>
+      <x:c r="E140" s="63" t="str">
+        <x:v>São Paulo/SP, presencial</x:v>
+      </x:c>
+      <x:c r="F140" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=e855bb6ab23a9103</x:v>
+      </x:c>
+      <x:c r="G140" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H140" s="63" t="str">
+        <x:v>Abrir em Minhas Vagas no Indeed, concluir o reCAPTCHA normal e enviar pessoalmente</x:v>
+      </x:c>
+      <x:c r="I140" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J140" s="63" t="str">
+        <x:v>Vaga com salário oficial de R$3.000–6.000. A candidatura chegou a 100% no Indeed e foi salva por 14 dias, com currículo técnico selecionado. Aderência em React, TypeScript, REST, Git, testes, SQL, automação e IA; PHP, RPA, n8n e SQL Server permanecem como temas de aprendizado. O envio final ficou bloqueado por reCAPTCHA, não contornado.</x:v>
+      </x:c>
+      <x:c r="K140" s="63" t="str">
+        <x:v>Não — rascunho 100% no Indeed</x:v>
+      </x:c>
+      <x:c r="L140" t="n">
+        <x:f>IF(LEFT(K140,3)="Sim",1,0)+IF(LEFT(K140,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M140" t="n">
+        <x:f>IF(LEFT(A140,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" ht="94" customHeight="1">
+      <x:c r="A141" s="63" t="str">
+        <x:v>Pendente — reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="B141" s="63" t="str">
+        <x:v>Digisystem</x:v>
+      </x:c>
+      <x:c r="C141" s="63" t="str">
+        <x:v>Analista de Desenvolvimento Jr</x:v>
+      </x:c>
+      <x:c r="D141" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E141" s="63" t="str">
+        <x:v>São Paulo/SP, híbrido; CLT</x:v>
+      </x:c>
+      <x:c r="F141" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=cd766d5302c29bc1</x:v>
+      </x:c>
+      <x:c r="G141" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H141" s="63" t="str">
+        <x:v>Abrir em Minhas Vagas no Indeed, concluir o reCAPTCHA normal e enviar pessoalmente</x:v>
+      </x:c>
+      <x:c r="I141" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J141" s="63" t="str">
+        <x:v>Candidatura chegou a 100% e foi salva por 14 dias. A vaga aceita 0–2 anos, estágio, projetos acadêmicos ou pessoais e exige linguagem de programação, SQL, APIs REST, Git e testes — todos alinhados ao currículo técnico. O envio final ficou bloqueado por reCAPTCHA, não contornado.</x:v>
+      </x:c>
+      <x:c r="K141" s="63" t="str">
+        <x:v>Não — rascunho 100% no Indeed</x:v>
+      </x:c>
+      <x:c r="L141" t="n">
+        <x:f>IF(LEFT(K141,3)="Sim",1,0)+IF(LEFT(K141,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M141" t="n">
+        <x:f>IF(LEFT(A141,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142" ht="94" customHeight="1">
+      <x:c r="A142" s="63" t="str">
+        <x:v>Pendente — reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="B142" s="63" t="str">
+        <x:v>Keyrus Brazil</x:v>
+      </x:c>
+      <x:c r="C142" s="63" t="str">
+        <x:v>Data Engineer Jr (Snowflake)</x:v>
+      </x:c>
+      <x:c r="D142" s="63" t="str">
+        <x:v>Dados e IA</x:v>
+      </x:c>
+      <x:c r="E142" s="63" t="str">
+        <x:v>São Paulo/SP, presencial/híbrido não declarado</x:v>
+      </x:c>
+      <x:c r="F142" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=c80baa59d4edaac6</x:v>
+      </x:c>
+      <x:c r="G142" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H142" s="63" t="str">
+        <x:v>Abrir em Minhas Vagas no Indeed, concluir o reCAPTCHA normal e enviar pessoalmente</x:v>
+      </x:c>
+      <x:c r="I142" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J142" s="63" t="str">
+        <x:v>Candidatura chegou a 100% e foi salva por 14 dias. A vaga aceita formação em andamento e tem aderência em SQL, Python, ETL/ELT, testes de dados e GCP. Snowflake, dbt e orquestração foram tratados como gaps de estudo, sem alegar experiência inexistente. O envio final ficou bloqueado por reCAPTCHA, não contornado.</x:v>
+      </x:c>
+      <x:c r="K142" s="63" t="str">
+        <x:v>Não — rascunho 100% no Indeed</x:v>
+      </x:c>
+      <x:c r="L142" t="n">
+        <x:f>IF(LEFT(K142,3)="Sim",1,0)+IF(LEFT(K142,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M142" t="n">
+        <x:f>IF(LEFT(A142,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143" ht="94" customHeight="1">
+      <x:c r="A143" s="63" t="str">
+        <x:v>Pendente — reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="B143" s="63" t="str">
+        <x:v>VESTE SA ESTILO</x:v>
+      </x:c>
+      <x:c r="C143" s="63" t="str">
+        <x:v>Desenvolvedor Full Stack - Jr</x:v>
+      </x:c>
+      <x:c r="D143" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E143" s="63" t="str">
+        <x:v>São Paulo/SP, presencial/híbrido não declarado; CLT</x:v>
+      </x:c>
+      <x:c r="F143" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=bcbac382c1760b0c</x:v>
+      </x:c>
+      <x:c r="G143" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H143" s="63" t="str">
+        <x:v>Abrir em Minhas Vagas no Indeed, concluir o reCAPTCHA normal e enviar pessoalmente</x:v>
+      </x:c>
+      <x:c r="I143" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J143" s="63" t="str">
+        <x:v>Candidatura chegou a 100% e foi salva por 14 dias, com currículo técnico selecionado. Aderência em React, TypeScript, Node, APIs REST, Git, testes e correção de bugs; VTEX é diferencial em aprendizado. O envio final ficou bloqueado por reCAPTCHA, não contornado.</x:v>
+      </x:c>
+      <x:c r="K143" s="63" t="str">
+        <x:v>Não — rascunho 100% no Indeed</x:v>
+      </x:c>
+      <x:c r="L143" t="n">
+        <x:f>IF(LEFT(K143,3)="Sim",1,0)+IF(LEFT(K143,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M143" t="n">
+        <x:f>IF(LEFT(A143,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144" ht="94" customHeight="1">
+      <x:c r="A144" s="63" t="str">
+        <x:v>Pendente — tempo de experiência a confirmar</x:v>
+      </x:c>
+      <x:c r="B144" s="63" t="str">
+        <x:v>Assertiv Benefícios e Seguros</x:v>
+      </x:c>
+      <x:c r="C144" s="63" t="str">
+        <x:v>Analista de desenvolvedor JavaScript</x:v>
+      </x:c>
+      <x:c r="D144" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E144" s="63" t="str">
+        <x:v>São Paulo/SP</x:v>
+      </x:c>
+      <x:c r="F144" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=778889bd1597e8a1</x:v>
+      </x:c>
+      <x:c r="G144" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H144" s="63" t="str">
+        <x:v>Confirmar período real de experiência que possa ser declarado; só então revisar e enviar</x:v>
+      </x:c>
+      <x:c r="I144" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J144" s="63" t="str">
+        <x:v>Currículo técnico foi selecionado e o formulário avançou a 50%. A empresa exige no mínimo 1 ano numérico de experiência em uma lista ampla de tecnologias e também no cargo de Analista JavaScript. Como não há período verificável fornecido para declarar esse requisito, o processo foi salvo sem inventar tempo de experiência.</x:v>
+      </x:c>
+      <x:c r="K144" s="63" t="str">
+        <x:v>Não — rascunho 50% no Indeed</x:v>
+      </x:c>
+      <x:c r="L144" t="n">
+        <x:f>IF(LEFT(K144,3)="Sim",1,0)+IF(LEFT(K144,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M144" t="n">
+        <x:f>IF(LEFT(A144,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145" ht="94" customHeight="1">
+      <x:c r="A145" s="63" t="str">
+        <x:v>Pendente — dado pessoal faltante</x:v>
+      </x:c>
+      <x:c r="B145" s="63" t="str">
+        <x:v>Saquers Tech</x:v>
+      </x:c>
+      <x:c r="C145" s="63" t="str">
+        <x:v>Desenvolvedor(a) Node I</x:v>
+      </x:c>
+      <x:c r="D145" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E145" s="63" t="str">
+        <x:v>Porto Alegre/RS, presencial</x:v>
+      </x:c>
+      <x:c r="F145" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G145" s="63" t="str">
+        <x:v>Triagem, conversas com Pessoas e Cultura e liderança; sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H145" s="63" t="str">
+        <x:v>Informar o nome completo do pai para responder a pergunta obrigatória e continuar</x:v>
+      </x:c>
+      <x:c r="I145" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J145" s="63" t="str">
+        <x:v>Vaga aderente a Node.js, JavaScript, APIs REST, Git/GitHub, SQL, React, TypeScript, Docker e testes. A Gupy exige RG, nome completo da mãe, nome completo do pai, pretensão e comentário de experiência C/C++/JavaScript. RG e nome da mãe são conhecidos; o nome do pai não foi fornecido, portanto a candidatura não foi concluída nem foi inventado dado pessoal.</x:v>
+      </x:c>
+      <x:c r="K145" s="63" t="str">
+        <x:v>Não — perguntas obrigatórias não concluídas</x:v>
+      </x:c>
+      <x:c r="L145" t="n">
+        <x:f>IF(LEFT(K145,3)="Sim",1,0)+IF(LEFT(K145,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M145" t="n">
+        <x:f>IF(LEFT(A145,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146" ht="94" customHeight="1">
+      <x:c r="A146" s="63" t="str">
+        <x:v>Pendente — dados acadêmicos</x:v>
+      </x:c>
+      <x:c r="B146" s="63" t="str">
+        <x:v>v(dev) / Grupo Visagio</x:v>
+      </x:c>
+      <x:c r="C146" s="63" t="str">
+        <x:v>Visagio Talentos — Estágio: Desenvolvedor(a) de Software</x:v>
+      </x:c>
+      <x:c r="D146" s="63" t="str">
+        <x:v>Desenvolvimento, dados e automação</x:v>
+      </x:c>
+      <x:c r="E146" s="63" t="str">
+        <x:v>Remoto; banco de talentos</x:v>
+      </x:c>
+      <x:c r="F146" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G146" s="63" t="str">
+        <x:v>Etapas online e entrevistas futuras; sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H146" s="63" t="str">
+        <x:v>Informar CR e grade horária real da faculdade para continuar</x:v>
+      </x:c>
+      <x:c r="I146" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J146" s="63" t="str">
+        <x:v>Banco de talentos de estágio com formação em andamento e sem experiência formal obrigatória. A Gupy exige Coeficiente de Rendimento e grade horária detalhada; esses dados não foram fornecidos e não foram estimados. A candidatura não foi concluída.</x:v>
+      </x:c>
+      <x:c r="K146" s="63" t="str">
+        <x:v>Não — perguntas obrigatórias não concluídas</x:v>
+      </x:c>
+      <x:c r="L146" t="n">
+        <x:f>IF(LEFT(K146,3)="Sim",1,0)+IF(LEFT(K146,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M146" t="n">
+        <x:f>IF(LEFT(A146,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147" ht="94" customHeight="1">
+      <x:c r="A147" s="63" t="str">
+        <x:v>Pendente — reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="B147" s="63" t="str">
+        <x:v>NSTECH / eFrete</x:v>
+      </x:c>
+      <x:c r="C147" s="63" t="str">
+        <x:v>Analista de Dados Jr</x:v>
+      </x:c>
+      <x:c r="D147" s="63" t="str">
+        <x:v>Dados e IA</x:v>
+      </x:c>
+      <x:c r="E147" s="63" t="str">
+        <x:v>São Paulo/SP, híbrido (Moema)</x:v>
+      </x:c>
+      <x:c r="F147" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=90c50de3798b486a</x:v>
+      </x:c>
+      <x:c r="G147" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H147" s="63" t="str">
+        <x:v>Abrir em Minhas Vagas no Indeed, concluir o reCAPTCHA normal e enviar pessoalmente</x:v>
+      </x:c>
+      <x:c r="I147" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J147" s="63" t="str">
+        <x:v>Candidatura chegou a 100% e foi salva por 14 dias. Dados factuais preenchidos: LinkedIn, CPF, disponibilidade híbrida, pretensão CLT de R$4.500 e autoidentificação. Aderência em SQL/PostgreSQL, Python, Excel e dados; Power BI e PDI/Pentaho estão em aprofundamento. O envio final ficou bloqueado por reCAPTCHA, não contornado.</x:v>
+      </x:c>
+      <x:c r="K147" s="63" t="str">
+        <x:v>Não — rascunho 100% no Indeed</x:v>
+      </x:c>
+      <x:c r="L147" t="n">
+        <x:f>IF(LEFT(K147,3)="Sim",1,0)+IF(LEFT(K147,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M147" t="n">
+        <x:f>IF(LEFT(A147,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148" ht="94" customHeight="1">
+      <x:c r="A148" s="63" t="str">
+        <x:v>Pendente — reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="B148" s="63" t="str">
+        <x:v>TechBrabo / MONT SEGURO</x:v>
+      </x:c>
+      <x:c r="C148" s="63" t="str">
+        <x:v>Desenvolvedor Full Stack Jr</x:v>
+      </x:c>
+      <x:c r="D148" s="63" t="str">
+        <x:v>Desenvolvimento e IA</x:v>
+      </x:c>
+      <x:c r="E148" s="63" t="str">
+        <x:v>Brasília/DF, presencial; PJ</x:v>
+      </x:c>
+      <x:c r="F148" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=e1f7406e162b0c90</x:v>
+      </x:c>
+      <x:c r="G148" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H148" s="63" t="str">
+        <x:v>Abrir em Minhas Vagas no Indeed, concluir o reCAPTCHA normal e enviar pessoalmente</x:v>
+      </x:c>
+      <x:c r="I148" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J148" s="63" t="str">
+        <x:v>Vaga com salário oficial de R$3.300 PJ. Candidatura chegou a 100% e foi salva por 14 dias, com currículo selecionado e dados cadastrais factuais informados. Aderência em Python, React de projetos, APIs, Docker, CI/CD e IA; Django, n8n e Make permanecem como temas de estudo. O envio final ficou bloqueado por reCAPTCHA, não contornado.</x:v>
+      </x:c>
+      <x:c r="K148" s="63" t="str">
+        <x:v>Não — rascunho 100% no Indeed</x:v>
+      </x:c>
+      <x:c r="L148" t="n">
+        <x:f>IF(LEFT(K148,3)="Sim",1,0)+IF(LEFT(K148,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M148" t="n">
+        <x:f>IF(LEFT(A148,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" ht="94" customHeight="1">
+      <x:c r="A149" s="63" t="str">
+        <x:v>Pendente — Profiler comportamental</x:v>
+      </x:c>
+      <x:c r="B149" s="63" t="str">
+        <x:v>Grupo Costa Norte de Comunicação</x:v>
+      </x:c>
+      <x:c r="C149" s="63" t="str">
+        <x:v>Desenvolvedor de Software - Júnior</x:v>
+      </x:c>
+      <x:c r="D149" s="63" t="str">
+        <x:v>Desenvolvimento e automação</x:v>
+      </x:c>
+      <x:c r="E149" s="63" t="str">
+        <x:v>Bertioga/SP, presencial; CLT</x:v>
+      </x:c>
+      <x:c r="F149" s="63" t="str">
+        <x:v>https://grupocostanorte.vagas.solides.com.br/vaga/914427?origem=indeed</x:v>
+      </x:c>
+      <x:c r="G149" s="63" t="str">
+        <x:v>Profiler comportamental apresentado pela plataforma; vídeo opcional não iniciado</x:v>
+      </x:c>
+      <x:c r="H149" s="63" t="str">
+        <x:v>Concluir o Profiler pessoalmente e retornar à Sólides para efetuar a candidatura</x:v>
+      </x:c>
+      <x:c r="I149" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J149" s="63" t="str">
+        <x:v>Vaga com salário oficial de R$3.500 CLT e boa aderência em Python, JavaScript/TypeScript, SQL, Git, APIs, testes e documentação. O currículo Sólides foi revisado e salvo sem vídeo; a plataforma passou a exigir/mostrar Profiler antes do avanço final. A candidatura não foi enviada.</x:v>
+      </x:c>
+      <x:c r="K149" s="63" t="str">
+        <x:v>Não — currículo salvo, candidatura não confirmada</x:v>
+      </x:c>
+      <x:c r="L149" t="n">
+        <x:f>IF(LEFT(K149,3)="Sim",1,0)+IF(LEFT(K149,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M149" t="n">
+        <x:f>IF(LEFT(A149,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150" ht="94" customHeight="1">
+      <x:c r="A150" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B150" s="63" t="str">
+        <x:v>IVO Services (via Jobbol)</x:v>
+      </x:c>
+      <x:c r="C150" s="63" t="str">
+        <x:v>Analista de Sistemas em Aplicações e Full Stack Júnior</x:v>
+      </x:c>
+      <x:c r="D150" s="63" t="str">
+        <x:v>Desenvolvimento e integrações</x:v>
+      </x:c>
+      <x:c r="E150" s="63" t="str">
+        <x:v>São Paulo/SP, híbrido</x:v>
+      </x:c>
+      <x:c r="F150" s="63" t="str">
+        <x:v>https://www.jobbol.com.br/vaga/29387065797</x:v>
+      </x:c>
+      <x:c r="G150" s="63" t="str">
+        <x:v>Contato posterior por WhatsApp informado pelo portal; sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H150" s="63" t="str">
+        <x:v>Acompanhar o e-mail e o contato escrito do recrutador; validar o formato de qualquer nova etapa</x:v>
+      </x:c>
+      <x:c r="I150" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J150" s="63" t="str">
+        <x:v>Candidatura enviada via Jobbol com nome, celular e e-mail factuais. O portal exibiu 'Candidatura registrada com sucesso!' e protocolo DX0634400, além de confirmação por e-mail. A vaga requer formação em andamento, APIs REST/JSON, SQL, Git e inglês técnico; a média salarial mostrada pela plataforma é estimativa de mercado de R$4.000, não oferta oficial.</x:v>
+      </x:c>
+      <x:c r="K150" s="63" t="str">
+        <x:v>Sim — protocolo Jobbol DX0634400 30/09</x:v>
+      </x:c>
+      <x:c r="L150" t="n">
+        <x:f>IF(LEFT(K150,3)="Sim",1,0)+IF(LEFT(K150,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M150" t="n">
+        <x:f>IF(LEFT(A150,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151" ht="86" customHeight="1">
+      <x:c r="A151" s="32" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B151" s="63" t="str">
+        <x:v>Kriativa (via Jobbol)</x:v>
+      </x:c>
+      <x:c r="C151" s="63" t="str">
+        <x:v>Desenvolvedor Júnior de Automação</x:v>
+      </x:c>
+      <x:c r="D151" s="63" t="str">
+        <x:v>Desenvolvimento e automação</x:v>
+      </x:c>
+      <x:c r="E151" s="63" t="str">
+        <x:v>Rio de Janeiro/RJ</x:v>
+      </x:c>
+      <x:c r="F151" s="63" t="str">
+        <x:v>https://www.jobbol.com.br/vaga/29386784263</x:v>
+      </x:c>
+      <x:c r="G151" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H151" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal; validar formato de qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="I151" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J151" s="63" t="str">
+        <x:v>Candidatura enviada via Jobbol para vaga com salário oficial de R$3.000. O portal exibiu 'Candidatura registrada com sucesso!' e protocolo CW1953700. Foram usados apenas dados factuais e currículo técnico; não há teste, áudio ou vídeo iniciado.</x:v>
+      </x:c>
+      <x:c r="K151" s="63" t="str">
+        <x:v>Sim — protocolo Jobbol CW1953700 30/09</x:v>
+      </x:c>
+      <x:c r="L151" t="n">
+        <x:f>IF(LEFT(K151,3)="Sim",1,0)+IF(LEFT(K151,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M151" t="n">
+        <x:f>IF(LEFT(A151,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152" ht="86" customHeight="1">
+      <x:c r="A152" s="63" t="str">
+        <x:v>Pendente — reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="B152" s="63" t="str">
+        <x:v>UP Brasil</x:v>
+      </x:c>
+      <x:c r="C152" s="63" t="str">
+        <x:v>Analista de Sistemas Jr</x:v>
+      </x:c>
+      <x:c r="D152" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E152" s="63" t="str">
+        <x:v>Uberlândia/MG, híbrido</x:v>
+      </x:c>
+      <x:c r="F152" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=a1cb53693f8fb606</x:v>
+      </x:c>
+      <x:c r="G152" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H152" s="63" t="str">
+        <x:v>Abrir em Minhas Vagas no Indeed, concluir a verificação normal e enviar pessoalmente</x:v>
+      </x:c>
+      <x:c r="I152" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J152" s="63" t="str">
+        <x:v>Candidatura personalizada chegou a 100% no Indeed e foi salva. A descrição é aderente a React, TypeScript, APIs REST, SQL e Docker. O envio final exigiu reCAPTCHA normal, que não foi contornado. Salário não divulgado no anúncio revisado.</x:v>
+      </x:c>
+      <x:c r="K152" s="63" t="str">
+        <x:v>Não — rascunho 100% no Indeed</x:v>
+      </x:c>
+      <x:c r="L152" t="n">
+        <x:f>IF(LEFT(K152,3)="Sim",1,0)+IF(LEFT(K152,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M152" t="n">
+        <x:f>IF(LEFT(A152,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="86" customHeight="1">
+      <x:c r="A153" s="63" t="str">
+        <x:v>Pendente — falha de formulário</x:v>
+      </x:c>
+      <x:c r="B153" s="63" t="str">
+        <x:v>Housi</x:v>
+      </x:c>
+      <x:c r="C153" s="63" t="str">
+        <x:v>Analista de Dados Júnior</x:v>
+      </x:c>
+      <x:c r="D153" s="63" t="str">
+        <x:v>Dados e IA</x:v>
+      </x:c>
+      <x:c r="E153" s="63" t="str">
+        <x:v>São Paulo/SP; modelo não confirmado</x:v>
+      </x:c>
+      <x:c r="F153" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=08a3368a8eed4671</x:v>
+      </x:c>
+      <x:c r="G153" s="63" t="str">
+        <x:v>Sem audiovisual declarado</x:v>
+      </x:c>
+      <x:c r="H153" s="63" t="str">
+        <x:v>Retomar por Minhas Vagas no Indeed; revisar seleção de currículo e concluir se a tela carregar</x:v>
+      </x:c>
+      <x:c r="I153" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J153" s="63" t="str">
+        <x:v>Vaga aderente a Python, SQL, análise de dados e GCP. O formulário do Indeed permaneceu carregando na etapa de currículo, mesmo após uma recarga, e o rascunho foi salvo a 38%. Não houve candidatura enviada nem dado inventado. Salário não divulgado.</x:v>
+      </x:c>
+      <x:c r="K153" s="63" t="str">
+        <x:v>Não — rascunho 38% no Indeed</x:v>
+      </x:c>
+      <x:c r="L153" t="n">
+        <x:f>IF(LEFT(K153,3)="Sim",1,0)+IF(LEFT(K153,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M153" t="n">
+        <x:f>IF(LEFT(A153,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154" ht="86" customHeight="1">
+      <x:c r="A154" s="63" t="str">
+        <x:v>Pendente — Profiler comportamental</x:v>
+      </x:c>
+      <x:c r="B154" s="63" t="str">
+        <x:v>Planeta do Bebê</x:v>
+      </x:c>
+      <x:c r="C154" s="63" t="str">
+        <x:v>Desenvolvedor(a) Júnior Python &amp; Frontend</x:v>
+      </x:c>
+      <x:c r="D154" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E154" s="63" t="str">
+        <x:v>Cotia/SP</x:v>
+      </x:c>
+      <x:c r="F154" s="63" t="str">
+        <x:v>https://planetadobebe.vagas.solides.com.br/vaga/922451?origem=indeed</x:v>
+      </x:c>
+      <x:c r="G154" s="63" t="str">
+        <x:v>Profiler comportamental obrigatório; vídeo não iniciado</x:v>
+      </x:c>
+      <x:c r="H154" s="63" t="str">
+        <x:v>Concluir o Profiler pessoalmente e retornar à Sólides para efetuar a candidatura</x:v>
+      </x:c>
+      <x:c r="I154" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J154" s="63" t="str">
+        <x:v>Perfil Sólides foi revisado e salvo com dados existentes. A plataforma exigiu o Profiler antes do envio; ele não foi iniciado nem respondido. A vaga tem alta aderência em Python, JavaScript/TypeScript, APIs, SQL, Git, Docker e testes. Salário não divulgado.</x:v>
+      </x:c>
+      <x:c r="K154" s="63" t="str">
+        <x:v>Não — perfil salvo, candidatura não confirmada</x:v>
+      </x:c>
+      <x:c r="L154" t="n">
+        <x:f>IF(LEFT(K154,3)="Sim",1,0)+IF(LEFT(K154,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M154" t="n">
+        <x:f>IF(LEFT(A154,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155" ht="86" customHeight="1">
+      <x:c r="A155" s="63" t="str">
+        <x:v>Encerrada — vaga expirada</x:v>
+      </x:c>
+      <x:c r="B155" s="63" t="str">
+        <x:v>Partner Soluções Empresariais</x:v>
+      </x:c>
+      <x:c r="C155" s="63" t="str">
+        <x:v>Desenvolvedor de Sistemas Júnior</x:v>
+      </x:c>
+      <x:c r="D155" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E155" s="63" t="str">
+        <x:v>Belo Horizonte/MG</x:v>
+      </x:c>
+      <x:c r="F155" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=d27699dec8cafae4</x:v>
+      </x:c>
+      <x:c r="G155" s="63" t="str">
+        <x:v>Não aplicável — anúncio expirado</x:v>
+      </x:c>
+      <x:c r="H155" s="63" t="str">
+        <x:v>Não candidatar; monitorar repostagem equivalente</x:v>
+      </x:c>
+      <x:c r="I155" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J155" s="63" t="str">
+        <x:v>Anúncio com faixa publicada de R$3.000–5.000 foi aberto no ciclo atual, mas o Indeed confirmou que a vaga expirou antes de qualquer candidatura. Registro mantido para evitar nova tentativa e duplicidade.</x:v>
+      </x:c>
+      <x:c r="K155" s="63" t="str">
+        <x:v>Não aplicável — vaga expirada</x:v>
+      </x:c>
+      <x:c r="L155" t="n">
+        <x:f>IF(LEFT(K155,3)="Sim",1,0)+IF(LEFT(K155,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M155" t="n">
+        <x:f>IF(LEFT(A155,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156" ht="86" customHeight="1">
+      <x:c r="A156" s="63" t="str">
+        <x:v>Pendente — candidatura a iniciar</x:v>
+      </x:c>
+      <x:c r="B156" s="63" t="str">
+        <x:v>Juriscont</x:v>
+      </x:c>
+      <x:c r="C156" s="63" t="str">
+        <x:v>Desenvolvedor Full Stack</x:v>
+      </x:c>
+      <x:c r="D156" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E156" s="63" t="str">
+        <x:v>São Paulo/SP, presencial (Berrini)</x:v>
+      </x:c>
+      <x:c r="F156" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=ef8b72cc9c69fb77</x:v>
+      </x:c>
+      <x:c r="G156" s="63" t="str">
+        <x:v>Sem audiovisual declarado no anúncio</x:v>
+      </x:c>
+      <x:c r="H156" s="63" t="str">
+        <x:v>Revalidar o anúncio, personalizar com React/Node/APIs/SQL/Git e iniciar pelo Indeed</x:v>
+      </x:c>
+      <x:c r="I156" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J156" s="63" t="str">
+        <x:v>Vaga ativa no levantamento, com faixa oficial de R$4.000–5.500. Boa aderência a React, Node, APIs REST, SQL e Git. Nenhum formulário foi iniciado nesta sessão porque a conexão do navegador caiu; revalidar antes de enviar.</x:v>
+      </x:c>
+      <x:c r="K156" s="63" t="str">
+        <x:v>Não — candidatura ainda não iniciada</x:v>
+      </x:c>
+      <x:c r="L156" t="n">
+        <x:f>IF(LEFT(K156,3)="Sim",1,0)+IF(LEFT(K156,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M156" t="n">
+        <x:f>IF(LEFT(A156,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157" ht="86" customHeight="1">
+      <x:c r="A157" s="63" t="str">
+        <x:v>Pendente — candidatura a iniciar</x:v>
+      </x:c>
+      <x:c r="B157" s="63" t="str">
+        <x:v>RH Sales Center</x:v>
+      </x:c>
+      <x:c r="C157" s="63" t="str">
+        <x:v>Engenheiro de Automação e Integração com IA</x:v>
+      </x:c>
+      <x:c r="D157" s="63" t="str">
+        <x:v>Automação, integrações e IA</x:v>
+      </x:c>
+      <x:c r="E157" s="63" t="str">
+        <x:v>São Paulo/SP</x:v>
+      </x:c>
+      <x:c r="F157" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=17b24a1cb5262487</x:v>
+      </x:c>
+      <x:c r="G157" s="63" t="str">
+        <x:v>Sem audiovisual declarado no anúncio</x:v>
+      </x:c>
+      <x:c r="H157" s="63" t="str">
+        <x:v>Revalidar o anúncio, personalizar com APIs, webhooks, PostgreSQL, Docker e IA aplicada</x:v>
+      </x:c>
+      <x:c r="I157" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J157" s="63" t="str">
+        <x:v>Vaga ativa no levantamento com salário oficial de R$5.500. Boa aderência a APIs REST, webhooks, PostgreSQL, MongoDB, filas, Docker, integração de LLMs e RAG em projetos. Nenhum formulário iniciado nesta sessão; revalidar a condição da vaga antes de enviar.</x:v>
+      </x:c>
+      <x:c r="K157" s="63" t="str">
+        <x:v>Não — candidatura ainda não iniciada</x:v>
+      </x:c>
+      <x:c r="L157" t="n">
+        <x:f>IF(LEFT(K157,3)="Sim",1,0)+IF(LEFT(K157,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M157" t="n">
+        <x:f>IF(LEFT(A157,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158" ht="86" customHeight="1">
+      <x:c r="A158" s="63" t="str">
+        <x:v>Pendente — candidatura a iniciar</x:v>
+      </x:c>
+      <x:c r="B158" s="63" t="str">
+        <x:v>ASC Brazil</x:v>
+      </x:c>
+      <x:c r="C158" s="63" t="str">
+        <x:v>Assistente Desenvolvedor de IA</x:v>
+      </x:c>
+      <x:c r="D158" s="63" t="str">
+        <x:v>Dados e IA</x:v>
+      </x:c>
+      <x:c r="E158" s="63" t="str">
+        <x:v>Uberlândia/MG, híbrido; CLT</x:v>
+      </x:c>
+      <x:c r="F158" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=84b7681a2e8fb5c0</x:v>
+      </x:c>
+      <x:c r="G158" s="63" t="str">
+        <x:v>Sem audiovisual declarado no anúncio</x:v>
+      </x:c>
+      <x:c r="H158" s="63" t="str">
+        <x:v>Revalidar o anúncio, personalizar com LLM APIs, Node, PostgreSQL, Git e IA aplicada</x:v>
+      </x:c>
+      <x:c r="I158" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J158" s="63" t="str">
+        <x:v>Vaga ativa no levantamento com salário oficial de R$3.500–3.575. Aderência em APIs de LLM, Node de projetos, PostgreSQL, Git e integração de IA. LangChain, LlamaIndex, RAG e bancos vetoriais são temas de estudo, sem alegar experiência consolidada.</x:v>
+      </x:c>
+      <x:c r="K158" s="63" t="str">
+        <x:v>Não — candidatura ainda não iniciada</x:v>
+      </x:c>
+      <x:c r="L158" t="n">
+        <x:f>IF(LEFT(K158,3)="Sim",1,0)+IF(LEFT(K158,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M158" t="n">
+        <x:f>IF(LEFT(A158,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159" ht="86" customHeight="1">
+      <x:c r="A159" s="63" t="str">
+        <x:v>Pendente — candidatura a iniciar</x:v>
+      </x:c>
+      <x:c r="B159" s="63" t="str">
+        <x:v>IB Comércio e Indústria</x:v>
+      </x:c>
+      <x:c r="C159" s="63" t="str">
+        <x:v>Analista Júnior de Dados e BI</x:v>
+      </x:c>
+      <x:c r="D159" s="63" t="str">
+        <x:v>Dados e IA</x:v>
+      </x:c>
+      <x:c r="E159" s="63" t="str">
+        <x:v>Rio de Janeiro/RJ, presencial; CLT</x:v>
+      </x:c>
+      <x:c r="F159" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=db72337e74b7a47f</x:v>
+      </x:c>
+      <x:c r="G159" s="63" t="str">
+        <x:v>Sem audiovisual declarado no anúncio</x:v>
+      </x:c>
+      <x:c r="H159" s="63" t="str">
+        <x:v>Revalidar o anúncio, personalizar com Python, SQL, Excel e automação de dados</x:v>
+      </x:c>
+      <x:c r="I159" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J159" s="63" t="str">
+        <x:v>Vaga ativa no levantamento com salário oficial de R$3.500–4.000 e graduação em andamento aceita. Boa aderência em Python, SQL, Excel e automação de dados. Power BI, n8n, Airflow e Streamlit devem ser apresentados como aprofundamento quando solicitados.</x:v>
+      </x:c>
+      <x:c r="K159" s="63" t="str">
+        <x:v>Não — candidatura ainda não iniciada</x:v>
+      </x:c>
+      <x:c r="L159" t="n">
+        <x:f>IF(LEFT(K159,3)="Sim",1,0)+IF(LEFT(K159,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M159" t="n">
+        <x:f>IF(LEFT(A159,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" ht="86" customHeight="1">
+      <x:c r="A160" s="63" t="str">
+        <x:v>Pendente — candidatura a iniciar</x:v>
+      </x:c>
+      <x:c r="B160" s="63" t="str">
+        <x:v>Partners Comunicação</x:v>
+      </x:c>
+      <x:c r="C160" s="63" t="str">
+        <x:v>Desenvolvedor Full Stack</x:v>
+      </x:c>
+      <x:c r="D160" s="63" t="str">
+        <x:v>Desenvolvimento e IA</x:v>
+      </x:c>
+      <x:c r="E160" s="63" t="str">
+        <x:v>Belo Horizonte/MG, híbrido; PJ</x:v>
+      </x:c>
+      <x:c r="F160" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=120afa593ebe364a</x:v>
+      </x:c>
+      <x:c r="G160" s="63" t="str">
+        <x:v>Sem audiovisual declarado no anúncio</x:v>
+      </x:c>
+      <x:c r="H160" s="63" t="str">
+        <x:v>Revalidar o anúncio, personalizar com APIs, PostgreSQL, Git, Docker e IA aplicada</x:v>
+      </x:c>
+      <x:c r="I160" s="63" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="J160" s="63" t="str">
+        <x:v>Vaga ativa no levantamento com faixa oficial de R$4.000 PJ. Boa aderência a desenvolvimento full stack, APIs, PostgreSQL, Git, Docker e integração de IA. Nenhuma candidatura iniciou porque a conexão do Firefox com o Indeed caiu; revalidar antes de enviar.</x:v>
+      </x:c>
+      <x:c r="K160" s="63" t="str">
+        <x:v>Não — candidatura ainda não iniciada</x:v>
+      </x:c>
+      <x:c r="L160" t="n">
+        <x:f>IF(LEFT(K160,3)="Sim",1,0)+IF(LEFT(K160,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M160" t="n">
+        <x:f>IF(LEFT(A160,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A161" s="32" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B161" s="63" t="str">
+        <x:v>Empresa Confidencial</x:v>
+      </x:c>
+      <x:c r="C161" s="63" t="str">
+        <x:v>Desenvolvedor(a) .NET Backend</x:v>
+      </x:c>
+      <x:c r="D161" s="63" t="str">
+        <x:v>Desenvolvimento backend</x:v>
+      </x:c>
+      <x:c r="E161" s="63" t="str">
+        <x:v>São Paulo/SP; PJ; remuneração a combinar</x:v>
+      </x:c>
+      <x:c r="F161" s="63" t="str">
+        <x:v>https://www.catho.com.br/vagas/desenvolvedora-.net-backend/38631621</x:v>
+      </x:c>
+      <x:c r="G161" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H161" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal. Se houver contato, atualizar respostas sobre experiência profissional full stack conforme currículo atual.</x:v>
+      </x:c>
+      <x:c r="I161" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J161" s="63" t="str">
+        <x:v>Candidatura confirmada no portal Catho com a mensagem ‘CV enviado!’. Formulário anterior trouxe respostas que precisam refletir o histórico profissional atualizado caso o recrutador retome o contato.</x:v>
+      </x:c>
+      <x:c r="K161" s="63" t="str">
+        <x:v>Portal — CV enviado 02/10</x:v>
+      </x:c>
+      <x:c r="L161" t="n">
+        <x:f>IF(LEFT(K161,3)="Sim",1,0)+IF(LEFT(K161,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M161" t="n">
+        <x:f>IF(LEFT(A161,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A162" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B162" s="63" t="str">
+        <x:v>UNIFISA</x:v>
+      </x:c>
+      <x:c r="C162" s="63" t="str">
+        <x:v>Desenvolvedor(a) CRM Jr - Automação e Integrações</x:v>
+      </x:c>
+      <x:c r="D162" s="63" t="str">
+        <x:v>Automação e integrações</x:v>
+      </x:c>
+      <x:c r="E162" s="63" t="str">
+        <x:v>São Paulo/SP; CLT; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F162" s="63" t="str">
+        <x:v>https://www.catho.com.br/vagas/desenvolvedora-crm-jr-automacao-e-integracoes-marketing/38627517</x:v>
+      </x:c>
+      <x:c r="G162" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H162" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal; preparar exemplos reais de APIs, webhooks, PHP/Python e automação.</x:v>
+      </x:c>
+      <x:c r="I162" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J162" s="63" t="str">
+        <x:v>Candidatura confirmada no portal Catho com a mensagem ‘CV enviado!’. Aderência em automação, APIs, webhooks e integração entre sistemas.</x:v>
+      </x:c>
+      <x:c r="K162" s="63" t="str">
+        <x:v>Portal — CV enviado 02/10</x:v>
+      </x:c>
+      <x:c r="L162" t="n">
+        <x:f>IF(LEFT(K162,3)="Sim",1,0)+IF(LEFT(K162,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M162" t="n">
+        <x:f>IF(LEFT(A162,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A163" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B163" s="63" t="str">
+        <x:v>Empresa Confidencial</x:v>
+      </x:c>
+      <x:c r="C163" s="63" t="str">
+        <x:v>Desenvolvedor(a) Front-End - Vue.js</x:v>
+      </x:c>
+      <x:c r="D163" s="63" t="str">
+        <x:v>Desenvolvimento frontend</x:v>
+      </x:c>
+      <x:c r="E163" s="63" t="str">
+        <x:v>São Paulo/SP; remoto; PJ; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F163" s="63" t="str">
+        <x:v>https://www.infojobs.com.br/vaga-de-desenvolvedora-front-end-vuejs-em-sao-paulo__12069792.aspx</x:v>
+      </x:c>
+      <x:c r="G163" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H163" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal; reforçar React/TypeScript e experiência de frontend em conversa posterior.</x:v>
+      </x:c>
+      <x:c r="I163" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J163" s="63" t="str">
+        <x:v>Candidatura confirmada no InfoJobs com carta de apresentação anexada. Vue.js foi tratado com precisão, sem alegar experiência profissional específica não comprovada.</x:v>
+      </x:c>
+      <x:c r="K163" s="63" t="str">
+        <x:v>Portal — candidatura confirmada 02/10</x:v>
+      </x:c>
+      <x:c r="L163" t="n">
+        <x:f>IF(LEFT(K163,3)="Sim",1,0)+IF(LEFT(K163,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M163" t="n">
+        <x:f>IF(LEFT(A163,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A164" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B164" s="63" t="str">
+        <x:v>Funcional Recursos Humanos</x:v>
+      </x:c>
+      <x:c r="C164" s="63" t="str">
+        <x:v>Desenvolvedor TI</x:v>
+      </x:c>
+      <x:c r="D164" s="63" t="str">
+        <x:v>Desenvolvimento e integrações</x:v>
+      </x:c>
+      <x:c r="E164" s="63" t="str">
+        <x:v>São Paulo/SP; CLT presencial; salário divulgado R$ 7.000</x:v>
+      </x:c>
+      <x:c r="F164" s="63" t="str">
+        <x:v>https://www.infojobs.com.br/vaga-de-desenvolvedor-ti-em-sao-paulo__12065974.aspx</x:v>
+      </x:c>
+      <x:c r="G164" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H164" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal; preparar exemplos de desenvolvimento, SQL, Git/GitHub e integrações.</x:v>
+      </x:c>
+      <x:c r="I164" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J164" s="63" t="str">
+        <x:v>Candidatura confirmada no InfoJobs com carta de apresentação anexada. Faixa salarial oficial divulgada: R$ 7.000/mês.</x:v>
+      </x:c>
+      <x:c r="K164" s="63" t="str">
+        <x:v>Portal — candidatura confirmada 02/10</x:v>
+      </x:c>
+      <x:c r="L164" t="n">
+        <x:f>IF(LEFT(K164,3)="Sim",1,0)+IF(LEFT(K164,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M164" t="n">
+        <x:f>IF(LEFT(A164,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A165" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B165" s="63" t="str">
+        <x:v>Empresarial Valestra Negócios e Investimentos</x:v>
+      </x:c>
+      <x:c r="C165" s="63" t="str">
+        <x:v>Analista de BI Júnior</x:v>
+      </x:c>
+      <x:c r="D165" s="63" t="str">
+        <x:v>Dados e BI</x:v>
+      </x:c>
+      <x:c r="E165" s="63" t="str">
+        <x:v>São Paulo/SP; presencial; remuneração a combinar</x:v>
+      </x:c>
+      <x:c r="F165" s="63" t="str">
+        <x:v>https://www.infojobs.com.br/vaga-de-analista-bi-junior-em-sao-paulo__12036637.aspx</x:v>
+      </x:c>
+      <x:c r="G165" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H165" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal; preparar exemplos de SQL, Excel, dados e automação, sem apresentar BI corporativo como experiência formal.</x:v>
+      </x:c>
+      <x:c r="I165" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J165" s="63" t="str">
+        <x:v>Candidatura confirmada no InfoJobs com carta de apresentação anexada. Formação superior foi declarada em andamento, conforme a realidade.</x:v>
+      </x:c>
+      <x:c r="K165" s="63" t="str">
+        <x:v>Portal — candidatura confirmada 02/10</x:v>
+      </x:c>
+      <x:c r="L165" t="n">
+        <x:f>IF(LEFT(K165,3)="Sim",1,0)+IF(LEFT(K165,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M165" t="n">
+        <x:f>IF(LEFT(A165,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A166" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B166" s="63" t="str">
+        <x:v>Kalunga</x:v>
+      </x:c>
+      <x:c r="C166" s="63" t="str">
+        <x:v>Analista de Sistemas Backend</x:v>
+      </x:c>
+      <x:c r="D166" s="63" t="str">
+        <x:v>Desenvolvimento backend</x:v>
+      </x:c>
+      <x:c r="E166" s="63" t="str">
+        <x:v>São Paulo/SP; CLT presencial; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F166" s="63" t="str">
+        <x:v>https://www.infojobs.com.br/vaga-de-analista-sistemas-backend-em-sao-paulo__12069489.aspx</x:v>
+      </x:c>
+      <x:c r="G166" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H166" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal; preparar exemplos de C#/.NET, APIs REST, PostgreSQL/SQL, Git e testes.</x:v>
+      </x:c>
+      <x:c r="I166" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J166" s="63" t="str">
+        <x:v>Candidatura confirmada no InfoJobs com carta de apresentação anexada. Boa aderência a C#/.NET, APIs e backend; SQL Server/EF/Dapper são pontos de estudo.</x:v>
+      </x:c>
+      <x:c r="K166" s="63" t="str">
+        <x:v>Portal — candidatura confirmada 02/10</x:v>
+      </x:c>
+      <x:c r="L166" t="n">
+        <x:f>IF(LEFT(K166,3)="Sim",1,0)+IF(LEFT(K166,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M166" t="n">
+        <x:f>IF(LEFT(A166,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A167" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B167" s="63" t="str">
+        <x:v>Empresa Confidencial</x:v>
+      </x:c>
+      <x:c r="C167" s="63" t="str">
+        <x:v>Analista de Dados e BI Jr</x:v>
+      </x:c>
+      <x:c r="D167" s="63" t="str">
+        <x:v>Dados e BI</x:v>
+      </x:c>
+      <x:c r="E167" s="63" t="str">
+        <x:v>Barueri/SP; remoto; CLT/PJ; salário divulgado R$ 3.000 a R$ 3.500</x:v>
+      </x:c>
+      <x:c r="F167" s="63" t="str">
+        <x:v>https://www.infojobs.com.br/vaga-de-analista-dados-bi-jr-em-sao-paulo__11941704.aspx</x:v>
+      </x:c>
+      <x:c r="G167" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H167" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal; manter foco em SQL, Excel, Python, PostgreSQL e automação de dados.</x:v>
+      </x:c>
+      <x:c r="I167" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J167" s="63" t="str">
+        <x:v>Candidatura confirmada no InfoJobs com carta de apresentação anexada. Autoavaliação de experiência formal em Data/BI permaneceu factual; salário solicitado: R$ 3.500, negociável.</x:v>
+      </x:c>
+      <x:c r="K167" s="63" t="str">
+        <x:v>Portal — candidatura confirmada 02/10</x:v>
+      </x:c>
+      <x:c r="L167" t="n">
+        <x:f>IF(LEFT(K167,3)="Sim",1,0)+IF(LEFT(K167,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M167" t="n">
+        <x:f>IF(LEFT(A167,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="66" hidden="0" customHeight="1">
+      <x:c r="A168" s="63" t="str">
+        <x:v>Enviada — revisar resposta se houver contato</x:v>
+      </x:c>
+      <x:c r="B168" s="63" t="str">
+        <x:v>Luft Logistics / Luft Agro</x:v>
+      </x:c>
+      <x:c r="C168" s="63" t="str">
+        <x:v>Desenvolvedor Full Stack</x:v>
+      </x:c>
+      <x:c r="D168" s="63" t="str">
+        <x:v>Desenvolvimento full stack</x:v>
+      </x:c>
+      <x:c r="E168" s="63" t="str">
+        <x:v>Barueri/SP; CLT presencial; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F168" s="63" t="str">
+        <x:v>https://www.infojobs.com.br/vaga-de-desenvolver-full-stack-em-sao-paulo__12036465.aspx</x:v>
+      </x:c>
+      <x:c r="G168" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H168" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal. Se houver contato, corrigir a resposta anterior: há experiência profissional full stack na Performance Lab desde dez/2025 e atuação freelancer de software/automação via CNPJ.</x:v>
+      </x:c>
+      <x:c r="I168" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J168" s="63" t="str">
+        <x:v>Candidatura confirmada no InfoJobs com carta de apresentação anexada. A resposta inicial sobre experiência profissional full stack/Node ficou desatualizada diante do currículo factual revisado; não reenviar nem duplicar a candidatura.</x:v>
+      </x:c>
+      <x:c r="K168" s="63" t="str">
+        <x:v>Portal — candidatura confirmada 02/10</x:v>
+      </x:c>
+      <x:c r="L168" t="n">
+        <x:f>IF(LEFT(K168,3)="Sim",1,0)+IF(LEFT(K168,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M168" t="n">
+        <x:f>IF(LEFT(A168,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A169" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B169" s="63" t="str">
+        <x:v>Novo Tempo RH</x:v>
+      </x:c>
+      <x:c r="C169" s="63" t="str">
+        <x:v>Desenvolvedor Jr</x:v>
+      </x:c>
+      <x:c r="D169" s="63" t="str">
+        <x:v>Desenvolvimento</x:v>
+      </x:c>
+      <x:c r="E169" s="63" t="str">
+        <x:v>Poá/SP; temporário presencial; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F169" s="63" t="str">
+        <x:v>https://www.infojobs.com.br/vaga-de-desenvolvedor-jr-em-sao-paulo__11971270.aspx</x:v>
+      </x:c>
+      <x:c r="G169" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H169" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal; preparar exemplos de C#, JavaScript, SQL e Git; destaque que ADS está em andamento.</x:v>
+      </x:c>
+      <x:c r="I169" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J169" s="63" t="str">
+        <x:v>Candidatura confirmada no InfoJobs com carta de apresentação anexada. A vaga aceita ADS em andamento e tem aderência técnica real.</x:v>
+      </x:c>
+      <x:c r="K169" s="63" t="str">
+        <x:v>Portal — candidatura confirmada 02/10</x:v>
+      </x:c>
+      <x:c r="L169" t="n">
+        <x:f>IF(LEFT(K169,3)="Sim",1,0)+IF(LEFT(K169,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M169" t="n">
+        <x:f>IF(LEFT(A169,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A170" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B170" s="63" t="str">
+        <x:v>Teledinâmica</x:v>
+      </x:c>
+      <x:c r="C170" s="63" t="str">
+        <x:v>Desenvolvedor - Foco em Back-End</x:v>
+      </x:c>
+      <x:c r="D170" s="63" t="str">
+        <x:v>Desenvolvimento backend</x:v>
+      </x:c>
+      <x:c r="E170" s="63" t="str">
+        <x:v>São Paulo/SP; híbrido; PJ; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F170" s="63" t="str">
+        <x:v>https://www.infojobs.com.br/vaga-de-desenvolvedor-foco-back-end-em-sao-paulo__11978071.aspx</x:v>
+      </x:c>
+      <x:c r="G170" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H170" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal; preparar exemplos de Node/TypeScript, Python, PostgreSQL, APIs, webhooks, Docker e cloud.</x:v>
+      </x:c>
+      <x:c r="I170" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J170" s="63" t="str">
+        <x:v>Candidatura confirmada no InfoJobs com carta de apresentação anexada. Boa aderência a backend, APIs, PostgreSQL, Docker e integração de sistemas.</x:v>
+      </x:c>
+      <x:c r="K170" s="63" t="str">
+        <x:v>Portal — candidatura confirmada 02/10</x:v>
+      </x:c>
+      <x:c r="L170" t="n">
+        <x:f>IF(LEFT(K170,3)="Sim",1,0)+IF(LEFT(K170,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M170" t="n">
+        <x:f>IF(LEFT(A170,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A171" s="63" t="str">
+        <x:v>Pendente — confirmação de localização</x:v>
+      </x:c>
+      <x:c r="B171" s="63" t="str">
+        <x:v>Macam Brasil</x:v>
+      </x:c>
+      <x:c r="C171" s="63" t="str">
+        <x:v>Desenvolvedor de Software - Armários Inteligentes</x:v>
+      </x:c>
+      <x:c r="D171" s="63" t="str">
+        <x:v>Desenvolvimento de software</x:v>
+      </x:c>
+      <x:c r="E171" s="63" t="str">
+        <x:v>São Paulo/SP; CLT; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F171" s="63" t="str">
+        <x:v>https://www.infojobs.com.br/vaga-de-desenvolvedora-software-armarios-inteligentes-em-sao-paulo__12051243.aspx</x:v>
+      </x:c>
+      <x:c r="G171" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H171" s="63" t="str">
+        <x:v>Responder somente se confirmar a pergunta obrigatória sobre morar na região de Pirituba/Jaraguá.</x:v>
+      </x:c>
+      <x:c r="I171" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J171" s="63" t="str">
+        <x:v>Formulário não enviado: a pergunta obrigatória sobre residir em Pirituba/Jaraguá não foi respondida porque a informação de endereço não foi confirmada. Nenhuma informação foi inventada.</x:v>
+      </x:c>
+      <x:c r="K171" s="63" t="str">
+        <x:v>Não — pergunta obrigatória pendente</x:v>
+      </x:c>
+      <x:c r="L171" t="n">
+        <x:f>IF(LEFT(K171,3)="Sim",1,0)+IF(LEFT(K171,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M171" t="n">
+        <x:f>IF(LEFT(A171,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" s="32" t="str">
         <x:v>Nota: ‘Sim’ significa recibo de e-mail localizado; ‘Portal’ significa confirmação/etapa verificada no portal. E-mails de inscrição iniciada não são tratados como candidatura enviada. Não há dados pessoais sensíveis nesta planilha.</x:v>
       </x:c>
+      <x:c r="B172" s="63"/>
+      <x:c r="C172" s="63"/>
+      <x:c r="D172" s="63"/>
+      <x:c r="E172" s="63"/>
+      <x:c r="F172" s="63"/>
+      <x:c r="G172" s="63"/>
+      <x:c r="H172" s="63"/>
+      <x:c r="I172" s="63"/>
+      <x:c r="J172" s="63"/>
+      <x:c r="K172" s="63"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A109:K109"/>
+    <x:mergeCell ref="A172:K172"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A10:A108">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Enviada"/>
@@ -5124,7 +7849,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a4a3520c9004c25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec6b5206a6c94d6e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6420,6 +9145,1133 @@
         <x:v>Registrar apenas para monitorar repostagem; não houve candidatura. Inglês fluente é requisito e o perfil informado é B1.</x:v>
       </x:c>
     </x:row>
+    <x:row r="60" ht="54" customHeight="1">
+      <x:c r="A60" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B60" s="28" t="str">
+        <x:v>Indeed → Gupy — Afya</x:v>
+      </x:c>
+      <x:c r="C60" s="28" t="str">
+        <x:v>Analista de Dados Júnior</x:v>
+      </x:c>
+      <x:c r="D60" s="28" t="str">
+        <x:v>Candidatura personalizada e envio final</x:v>
+      </x:c>
+      <x:c r="E60" s="28" t="str">
+        <x:v>A Gupy exibiu ‘Candidatura finalizada!’. A apresentação foi adaptada a SQL, Python, PostgreSQL, APIs, automações, documentação e validação de integridade, sem alegar domínio de Power BI ou dbt.</x:v>
+      </x:c>
+      <x:c r="F60" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G60" s="30" t="str">
+        <x:v>Acompanhar e-mail; validar o formato de cada etapa antes de iniciar, especialmente a Entrevista Inteligente.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="54" customHeight="1">
+      <x:c r="A61" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B61" s="28" t="str">
+        <x:v>Indeed → MOST</x:v>
+      </x:c>
+      <x:c r="C61" s="28" t="str">
+        <x:v>Full Stack Developer (Python) — Hiperautomação</x:v>
+      </x:c>
+      <x:c r="D61" s="28" t="str">
+        <x:v>Triagem e formulário oficial</x:v>
+      </x:c>
+      <x:c r="E61" s="28" t="str">
+        <x:v>Vaga remota de estágio de 6h com bolsa oficial de R$4.000. O Google Form exige upload de currículo; o formulário e o desafio técnico não foram enviados/iniciados nesta sessão.</x:v>
+      </x:c>
+      <x:c r="F61" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G61" s="30" t="str">
+        <x:v>Anexar currículo no formulário; realizar qualquer desafio técnico pessoalmente.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="54" customHeight="1">
+      <x:c r="A62" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B62" s="28" t="str">
+        <x:v>Indeed — rascunhos e formulários externos</x:v>
+      </x:c>
+      <x:c r="C62" s="28" t="str">
+        <x:v>Ana Recrutamento, iblue, YSSY, Cakto, Equifax e Kazza</x:v>
+      </x:c>
+      <x:c r="D62" s="28" t="str">
+        <x:v>Registro de pendências operacionais</x:v>
+      </x:c>
+      <x:c r="E62" s="28" t="str">
+        <x:v>Foram registrados rascunhos e formulários bloqueados por dados cadastrais não fornecidos ou upload obrigatório de currículo. Nenhum dado de endereço, CNH, estado civil ou arquivo foi inventado/substituído.</x:v>
+      </x:c>
+      <x:c r="F62" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G62" s="30" t="str">
+        <x:v>Retomar cada item com o dado ou anexo correspondente; revisar antes de enviar.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="54" customHeight="1">
+      <x:c r="A63" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B63" s="28" t="str">
+        <x:v>Indeed</x:v>
+      </x:c>
+      <x:c r="C63" s="28" t="str">
+        <x:v>Ciclo de busca de desenvolvimento, dados e IA</x:v>
+      </x:c>
+      <x:c r="D63" s="28" t="str">
+        <x:v>Limitação de plataforma</x:v>
+      </x:c>
+      <x:c r="E63" s="28" t="str">
+        <x:v>O Indeed salvou rascunhos quando possível. Botões finais protegidos por reCAPTCHA e uma página de pesquisa com Cloudflare não foram contornados.</x:v>
+      </x:c>
+      <x:c r="F63" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G63" s="30" t="str">
+        <x:v>Retomar a busca pelo Indeed quando o acesso normal estiver liberado; não burlar verificações.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="54" customHeight="1">
+      <x:c r="A64" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B64" s="28" t="str">
+        <x:v>Indeed → Gupy — Terram Engenharia</x:v>
+      </x:c>
+      <x:c r="C64" s="28" t="str">
+        <x:v>Analista de Dados Jr</x:v>
+      </x:c>
+      <x:c r="D64" s="28" t="str">
+        <x:v>Candidatura personalizada e envio final</x:v>
+      </x:c>
+      <x:c r="E64" s="28" t="str">
+        <x:v>A Gupy exibiu ‘Candidatura finalizada!’. A apresentação destacou Python, SQL/PostgreSQL, automações, APIs, Excel e documentação, tratando Power BI como tema de aprofundamento.</x:v>
+      </x:c>
+      <x:c r="F64" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G64" s="30" t="str">
+        <x:v>Acompanhar Fit Cultural e demais fases; validar o formato antes de iniciar qualquer avaliação.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="54" customHeight="1">
+      <x:c r="A65" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B65" s="28" t="str">
+        <x:v>Indeed — AM53 Tech Recruitment</x:v>
+      </x:c>
+      <x:c r="C65" s="28" t="str">
+        <x:v>Desenvolvedor(a) Júnior — Python &amp; Data Analytics</x:v>
+      </x:c>
+      <x:c r="D65" s="28" t="str">
+        <x:v>Personalização e rascunho final</x:v>
+      </x:c>
+      <x:c r="E65" s="28" t="str">
+        <x:v>Currículo e carta personalizada foram preparados. A candidatura chegou a 100%, mas o botão final não ficou disponível por reCAPTCHA; a verificação não foi contornada.</x:v>
+      </x:c>
+      <x:c r="F65" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G65" s="30" t="str">
+        <x:v>Retomar por Minhas Vagas no Indeed para concluir o envio quando a verificação normal estiver habilitada.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="54" customHeight="1">
+      <x:c r="A66" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B66" s="28" t="str">
+        <x:v>Indeed — COBRAPE</x:v>
+      </x:c>
+      <x:c r="C66" s="28" t="str">
+        <x:v>Programador Junior</x:v>
+      </x:c>
+      <x:c r="D66" s="28" t="str">
+        <x:v>Revisão e tentativa de envio</x:v>
+      </x:c>
+      <x:c r="E66" s="28" t="str">
+        <x:v>A vaga é aderente a C#/.NET e banco relacional. A tela abriu a 100%, mas ‘Enviar sua candidatura’ permaneceu desabilitado por reCAPTCHA. Nenhuma verificação foi burlada.</x:v>
+      </x:c>
+      <x:c r="F66" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G66" s="30" t="str">
+        <x:v>Concluir pelo Indeed quando o botão final estiver disponível; confirmar o recibo antes de marcar como enviada.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="62" customHeight="1">
+      <x:c r="A67" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B67" s="28" t="str">
+        <x:v>Indeed → Gupy — Conviso</x:v>
+      </x:c>
+      <x:c r="C67" s="28" t="str">
+        <x:v>Junior/Pleno Front-End Engineer</x:v>
+      </x:c>
+      <x:c r="D67" s="28" t="str">
+        <x:v>Candidatura personalizada e envio final</x:v>
+      </x:c>
+      <x:c r="E67" s="28" t="str">
+        <x:v>A Gupy exibiu ‘Candidatura finalizada!’. O texto adaptado destacou JavaScript/TypeScript, React de projetos, APIs, PostgreSQL, Docker, Git e testes, tratando Vue como aprendizado.</x:v>
+      </x:c>
+      <x:c r="F67" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G67" s="30" t="str">
+        <x:v>Acompanhar e-mail; validar o formato de qualquer próxima etapa antes de iniciar.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="62" customHeight="1">
+      <x:c r="A68" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B68" s="28" t="str">
+        <x:v>Indeed — Black Lion</x:v>
+      </x:c>
+      <x:c r="C68" s="28" t="str">
+        <x:v>Desenvolvedor(a) Full Stack Júnior | Fintech</x:v>
+      </x:c>
+      <x:c r="D68" s="28" t="str">
+        <x:v>Rascunho final e bloqueio de reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="E68" s="28" t="str">
+        <x:v>Currículo e respostas factuais chegaram a 100%. A vaga divulga R$3.000/mês, mas o envio final ficou protegido por reCAPTCHA; a verificação não foi contornada.</x:v>
+      </x:c>
+      <x:c r="F68" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G68" s="30" t="str">
+        <x:v>Concluir normalmente pelo Indeed em Minhas Vagas e confirmar o recibo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="62" customHeight="1">
+      <x:c r="A69" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B69" s="28" t="str">
+        <x:v>Indeed — Vertigo e Extractta</x:v>
+      </x:c>
+      <x:c r="C69" s="28" t="str">
+        <x:v>Analista de IA Jr; Backend Jr C#/.NET</x:v>
+      </x:c>
+      <x:c r="D69" s="28" t="str">
+        <x:v>Questionários técnicos escritos</x:v>
+      </x:c>
+      <x:c r="E69" s="28" t="str">
+        <x:v>Os rascunhos foram salvos no Indeed. Restam perguntas técnicas de múltipla escolha; nenhuma resposta de avaliação foi atribuída ao candidato.</x:v>
+      </x:c>
+      <x:c r="F69" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G69" s="30" t="str">
+        <x:v>Responder pessoalmente aos questionários e enviar; confirmar os recibos.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="62" customHeight="1">
+      <x:c r="A70" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B70" s="28" t="str">
+        <x:v>Indeed → Sólides — ELA DECORA e UNIX Logística</x:v>
+      </x:c>
+      <x:c r="C70" s="28" t="str">
+        <x:v>Full Stack Jr IA/SaaS; Dev Jr Automação/IA</x:v>
+      </x:c>
+      <x:c r="D70" s="28" t="str">
+        <x:v>Profiler comportamental obrigatório</x:v>
+      </x:c>
+      <x:c r="E70" s="28" t="str">
+        <x:v>Ambas exigem Profiler antes de salvar a candidatura. A UNIX divulga R$4.500 CLT; não houve candidatura confirmada.</x:v>
+      </x:c>
+      <x:c r="F70" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G70" s="30" t="str">
+        <x:v>Realizar pessoalmente a avaliação comportamental e revisar as candidaturas.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="62" customHeight="1">
+      <x:c r="A71" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B71" s="28" t="str">
+        <x:v>Indeed — Overlabs e Datum</x:v>
+      </x:c>
+      <x:c r="C71" s="28" t="str">
+        <x:v>FullStack Node/React; Engenheira de Dados Jr</x:v>
+      </x:c>
+      <x:c r="D71" s="28" t="str">
+        <x:v>Upload obrigatório de currículo</x:v>
+      </x:c>
+      <x:c r="E71" s="28" t="str">
+        <x:v>Os formulários externos exigem CV anexado e não registraram envio. Nenhum arquivo foi simulado ou substituído.</x:v>
+      </x:c>
+      <x:c r="F71" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G71" s="30" t="str">
+        <x:v>Anexar o currículo manualmente, revisar e enviar.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="62" customHeight="1">
+      <x:c r="A72" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B72" s="28" t="str">
+        <x:v>Indeed → Jobbol — AuthSoft</x:v>
+      </x:c>
+      <x:c r="C72" s="28" t="str">
+        <x:v>Desenvolvedor Júnior</x:v>
+      </x:c>
+      <x:c r="D72" s="28" t="str">
+        <x:v>Candidatura enviada</x:v>
+      </x:c>
+      <x:c r="E72" s="28" t="str">
+        <x:v>Candidatura enviada com currículo anexado; confirmação da plataforma exibiu protocolo LK9591784 e aviso de e-mail de confirmação.</x:v>
+      </x:c>
+      <x:c r="F72" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G72" s="30" t="str">
+        <x:v>Acompanhar e-mail e portal Jobbol; validar formato de qualquer nova etapa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="62" customHeight="1">
+      <x:c r="A73" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B73" s="28" t="str">
+        <x:v>Indeed → Gupy — Construmarket</x:v>
+      </x:c>
+      <x:c r="C73" s="28" t="str">
+        <x:v>Desenvolvedor(a) Júnior</x:v>
+      </x:c>
+      <x:c r="D73" s="28" t="str">
+        <x:v>Candidatura personalizada e envio final</x:v>
+      </x:c>
+      <x:c r="E73" s="28" t="str">
+        <x:v>A Gupy exibiu ‘Candidatura finalizada!’. A apresentação valorizou C#/.NET, TypeScript, APIs, SQL/PostgreSQL, Docker, Git e testes, sem declarar Angular como experiência consolidada.</x:v>
+      </x:c>
+      <x:c r="F73" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G73" s="30" t="str">
+        <x:v>Acompanhar Fit Cultural/teste; qualquer avaliação deve ser feita pessoalmente e com formato validado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="62" customHeight="1">
+      <x:c r="A74" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B74" s="28" t="str">
+        <x:v>Indeed → Gupy — Tokio Marine</x:v>
+      </x:c>
+      <x:c r="C74" s="28" t="str">
+        <x:v>Analista de Sistemas Júnior — Inteligência Artificial</x:v>
+      </x:c>
+      <x:c r="D74" s="28" t="str">
+        <x:v>Finalização e personalização</x:v>
+      </x:c>
+      <x:c r="E74" s="28" t="str">
+        <x:v>A candidatura foi retomada e finalizada na Gupy, com apresentação adaptada a Python, APIs, SQL, dados, IA/LLM, documentação e inglês intermediário.</x:v>
+      </x:c>
+      <x:c r="F74" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G74" s="30" t="str">
+        <x:v>Acompanhar Fit Cultural e testes complementares; validar o formato antes de iniciar.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="62" customHeight="1">
+      <x:c r="A75" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B75" s="28" t="str">
+        <x:v>Indeed → Gupy — Libbs</x:v>
+      </x:c>
+      <x:c r="C75" s="28" t="str">
+        <x:v>Desenvolvedor de Automação e IA Jr</x:v>
+      </x:c>
+      <x:c r="D75" s="28" t="str">
+        <x:v>Candidatura personalizada e envio final</x:v>
+      </x:c>
+      <x:c r="E75" s="28" t="str">
+        <x:v>A Gupy exibiu ‘Candidatura finalizada!’. O texto foi fiel a Python, APIs, SQL, Docker, Git, testes e automação; RPA/BPM foram posicionados como aprendizado.</x:v>
+      </x:c>
+      <x:c r="F75" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G75" s="30" t="str">
+        <x:v>Acompanhar abordagem telefônica, entrevista e case; realizar pessoalmente qualquer etapa avaliativa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="62" customHeight="1">
+      <x:c r="A76" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B76" s="28" t="str">
+        <x:v>Indeed → Gupy — Bellinati Perez</x:v>
+      </x:c>
+      <x:c r="C76" s="28" t="str">
+        <x:v>Analista de Dados Júnior</x:v>
+      </x:c>
+      <x:c r="D76" s="28" t="str">
+        <x:v>Candidatura personalizada e envio final</x:v>
+      </x:c>
+      <x:c r="E76" s="28" t="str">
+        <x:v>A Gupy exibiu ‘Candidatura finalizada!’. Foram preservadas respostas honestas sobre Excel, Python, SQL e BI como área em evolução.</x:v>
+      </x:c>
+      <x:c r="F76" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G76" s="30" t="str">
+        <x:v>Acompanhar e-mail; realizar pessoalmente qualquer teste técnico.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="62" customHeight="1">
+      <x:c r="A77" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B77" s="28" t="str">
+        <x:v>Indeed → Sólides — Perillo Engenharia</x:v>
+      </x:c>
+      <x:c r="C77" s="28" t="str">
+        <x:v>Desenvolvedor Full Stack Jr</x:v>
+      </x:c>
+      <x:c r="D77" s="28" t="str">
+        <x:v>Bloqueio audiovisual identificado</x:v>
+      </x:c>
+      <x:c r="E77" s="28" t="str">
+        <x:v>Vaga de R$5–6 mil PJ e aderência alta, mas o portal exige vídeo de apresentação obrigatório e RG antes de concluir. Nenhum vídeo foi iniciado.</x:v>
+      </x:c>
+      <x:c r="F77" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G77" s="30" t="str">
+        <x:v>Fazer a apresentação em vídeo pessoalmente caso decida avançar.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="62" customHeight="1">
+      <x:c r="A78" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B78" s="28" t="str">
+        <x:v>Indeed — PLACE Tecnologia/C70</x:v>
+      </x:c>
+      <x:c r="C78" s="28" t="str">
+        <x:v>Desenvolvedor de Software — Júnior</x:v>
+      </x:c>
+      <x:c r="D78" s="28" t="str">
+        <x:v>Retomada de rascunho</x:v>
+      </x:c>
+      <x:c r="E78" s="28" t="str">
+        <x:v>A página mostrou um rascunho iniciado, mas o SmartApply não carregou por reCAPTCHA. Nenhuma verificação foi contornada e não há recibo de envio.</x:v>
+      </x:c>
+      <x:c r="F78" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G78" s="30" t="str">
+        <x:v>Retomar normalmente em Minhas Vagas no Indeed; confirmar o recibo antes de considerar enviada.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="62" customHeight="1">
+      <x:c r="A79" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B79" s="28" t="str">
+        <x:v>Indeed → Avanade / Accenture Workday</x:v>
+      </x:c>
+      <x:c r="C79" s="28" t="str">
+        <x:v>Desenvolvedor(a) FullStack Junior</x:v>
+      </x:c>
+      <x:c r="D79" s="28" t="str">
+        <x:v>Triagem e bloqueio por dados cadastrais</x:v>
+      </x:c>
+      <x:c r="E79" s="28" t="str">
+        <x:v>Vaga aderente em .NET, React, TypeScript, APIs e testes. Login com Google foi concluído, mas o Workday requer endereço completo antes de salvar; nenhum endereço foi inventado.</x:v>
+      </x:c>
+      <x:c r="F79" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G79" s="30" t="str">
+        <x:v>Preencher endereço, revisar o formulário e enviar pelo Workday.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="62" customHeight="1">
+      <x:c r="A80" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B80" s="28" t="str">
+        <x:v>Indeed → e-mail — MOST</x:v>
+      </x:c>
+      <x:c r="C80" s="28" t="str">
+        <x:v>Full Stack Developer (Python) — Hiperautomação</x:v>
+      </x:c>
+      <x:c r="D80" s="28" t="str">
+        <x:v>Candidatura por e-mail</x:v>
+      </x:c>
+      <x:c r="E80" s="28" t="str">
+        <x:v>E-mail personalizado enviado ao RH da MOST com currículo técnico público, GitHub e LinkedIn. O Gmail exibiu 'Mensagem enviada'; desafio técnico não foi iniciado.</x:v>
+      </x:c>
+      <x:c r="F80" s="29" t="str">
+        <x:v>Enviado</x:v>
+      </x:c>
+      <x:c r="G80" s="30" t="str">
+        <x:v>Aguardar retorno/recibo; qualquer desafio técnico deve ser feito pessoalmente.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="62" customHeight="1">
+      <x:c r="A81" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B81" s="28" t="str">
+        <x:v>Indeed → Gupy — MRM Brasil</x:v>
+      </x:c>
+      <x:c r="C81" s="28" t="str">
+        <x:v>Desenvolvedor Fullstack Jr</x:v>
+      </x:c>
+      <x:c r="D81" s="28" t="str">
+        <x:v>Candidatura personalizada e envio final</x:v>
+      </x:c>
+      <x:c r="E81" s="28" t="str">
+        <x:v>A Gupy exibiu 'Candidatura finalizada!'. A vaga aceita primeira experiência técnica; a personalização valorizou APIs, integrações, SQL/PostgreSQL, Docker, Git, testes, C#/.NET, Python/FastAPI, JavaScript/TypeScript e uso responsável de IA.</x:v>
+      </x:c>
+      <x:c r="F81" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G81" s="30" t="str">
+        <x:v>Acompanhar e-mail; realizar pessoalmente entrevistas e avaliações.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="62" customHeight="1">
+      <x:c r="A82" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B82" s="28" t="str">
+        <x:v>Indeed → Gupy — Instituto Eldorado</x:v>
+      </x:c>
+      <x:c r="C82" s="28" t="str">
+        <x:v>Pessoa desenvolvedora Machine Learning</x:v>
+      </x:c>
+      <x:c r="D82" s="28" t="str">
+        <x:v>Candidatura personalizada e envio final</x:v>
+      </x:c>
+      <x:c r="E82" s="28" t="str">
+        <x:v>A Gupy exibiu 'Candidatura finalizada!'. A apresentação foi transparente sobre Python, SQL, dados, cloud e IA aplicada, enquanto modelagem e bibliotecas de ML foram posicionadas como aprofundamento.</x:v>
+      </x:c>
+      <x:c r="F82" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G82" s="30" t="str">
+        <x:v>Acompanhar e-mail; realizar pessoalmente entrevistas e avaliações.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="62" customHeight="1">
+      <x:c r="A83" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B83" s="28" t="str">
+        <x:v>Indeed — Lyncas, Valor Real e Luby</x:v>
+      </x:c>
+      <x:c r="C83" s="28" t="str">
+        <x:v>FullStack Jr Node/React; Full Stack Jr; Fullstack IA/Javascript Trainee/Júnior</x:v>
+      </x:c>
+      <x:c r="D83" s="28" t="str">
+        <x:v>Rascunhos 100% e reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="E83" s="28" t="str">
+        <x:v>Os três formulários ficaram completos e foram salvos por 14 dias. O envio final ficou bloqueado por reCAPTCHA; nenhuma verificação foi contornada.</x:v>
+      </x:c>
+      <x:c r="F83" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G83" s="30" t="str">
+        <x:v>Abrir Minhas Vagas no Indeed, concluir a verificação normal e enviar pessoalmente.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="62" customHeight="1">
+      <x:c r="A84" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B84" s="28" t="str">
+        <x:v>Indeed → Gupy — ISA Saúde</x:v>
+      </x:c>
+      <x:c r="C84" s="28" t="str">
+        <x:v>Desenvolvedor(a) Full Stack</x:v>
+      </x:c>
+      <x:c r="D84" s="28" t="str">
+        <x:v>Falha de formulário</x:v>
+      </x:c>
+      <x:c r="E84" s="28" t="str">
+        <x:v>A página de perguntas personalizadas da Gupy permaneceu vazia e não avançou após salvar. Não houve confirmação de candidatura finalizada.</x:v>
+      </x:c>
+      <x:c r="F84" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G84" s="30" t="str">
+        <x:v>Retomar pelo portal e resolver somente o carregamento normal.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="62" customHeight="1">
+      <x:c r="A85" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B85" s="28" t="str">
+        <x:v>Indeed → Sólides — ZOUPHY</x:v>
+      </x:c>
+      <x:c r="C85" s="28" t="str">
+        <x:v>Desenvolvedor Front-end (React)</x:v>
+      </x:c>
+      <x:c r="D85" s="28" t="str">
+        <x:v>Pendência de cadastro</x:v>
+      </x:c>
+      <x:c r="E85" s="28" t="str">
+        <x:v>O perfil foi revisado; o Sólides exige CNH válida e pretensão salarial. Vídeo é opcional e não foi iniciado.</x:v>
+      </x:c>
+      <x:c r="F85" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G85" s="30" t="str">
+        <x:v>Confirmar CNH antes de preencher e enviar.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="62" customHeight="1">
+      <x:c r="A86" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B86" s="28" t="str">
+        <x:v>Indeed — XP Inc.</x:v>
+      </x:c>
+      <x:c r="C86" s="28" t="str">
+        <x:v>Engenheiro(a) de Software | Assistente e Júnior</x:v>
+      </x:c>
+      <x:c r="D86" s="28" t="str">
+        <x:v>Deduplicação</x:v>
+      </x:c>
+      <x:c r="E86" s="28" t="str">
+        <x:v>O Indeed apresentou um novo rascunho a 100%, mas já existe candidatura confirmada no controle para a mesma vaga. O rascunho foi salvo e fechado, sem novo envio.</x:v>
+      </x:c>
+      <x:c r="F86" s="29" t="str">
+        <x:v>Registrado</x:v>
+      </x:c>
+      <x:c r="G86" s="30" t="str">
+        <x:v>Manter a candidatura confirmada existente e acompanhar somente o convite PI pessoalmente.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="62" customHeight="1">
+      <x:c r="A87" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B87" s="28" t="str">
+        <x:v>Indeed → Gupy — Quality Digital</x:v>
+      </x:c>
+      <x:c r="C87" s="28" t="str">
+        <x:v>Desenvolvedor Júnior</x:v>
+      </x:c>
+      <x:c r="D87" s="28" t="str">
+        <x:v>Deduplicação e confirmação</x:v>
+      </x:c>
+      <x:c r="E87" s="28" t="str">
+        <x:v>A Gupy confirmou novamente uma candidatura para a postagem atual, mas o controle já contém candidatura confirmada para a mesma empresa e título em 21/09. Nenhuma segunda linha foi criada para não inflar a contagem.</x:v>
+      </x:c>
+      <x:c r="F87" s="29" t="str">
+        <x:v>Registrado</x:v>
+      </x:c>
+      <x:c r="G87" s="30" t="str">
+        <x:v>Acompanhar a candidatura existente e evitar novo envio duplicado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="62" customHeight="1">
+      <x:c r="A88" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B88" s="28" t="str">
+        <x:v>Indeed — Engemoura Tecnologia Energética</x:v>
+      </x:c>
+      <x:c r="C88" s="28" t="str">
+        <x:v>Desenvolvedor</x:v>
+      </x:c>
+      <x:c r="D88" s="28" t="str">
+        <x:v>Rascunho 100% e reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="E88" s="28" t="str">
+        <x:v>Currículo técnico selecionado e formulário completo, com vaga de R$3.000–6.000. Envio final bloqueado por reCAPTCHA; a verificação não foi contornada.</x:v>
+      </x:c>
+      <x:c r="F88" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G88" s="30" t="str">
+        <x:v>Concluir a verificação normal no Indeed e confirmar o recibo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="62" customHeight="1">
+      <x:c r="A89" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B89" s="28" t="str">
+        <x:v>Indeed — Digisystem</x:v>
+      </x:c>
+      <x:c r="C89" s="28" t="str">
+        <x:v>Analista de Desenvolvimento Jr</x:v>
+      </x:c>
+      <x:c r="D89" s="28" t="str">
+        <x:v>Rascunho 100% e reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="E89" s="28" t="str">
+        <x:v>Formulário completo e salvo por 14 dias. A vaga aceita projetos pessoais/estágio e formação em andamento; envio final bloqueado por reCAPTCHA.</x:v>
+      </x:c>
+      <x:c r="F89" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G89" s="30" t="str">
+        <x:v>Concluir a verificação normal no Indeed e confirmar o recibo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="62" customHeight="1">
+      <x:c r="A90" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B90" s="28" t="str">
+        <x:v>Indeed — Keyrus Brazil</x:v>
+      </x:c>
+      <x:c r="C90" s="28" t="str">
+        <x:v>Data Engineer Jr (Snowflake)</x:v>
+      </x:c>
+      <x:c r="D90" s="28" t="str">
+        <x:v>Rascunho 100% e reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="E90" s="28" t="str">
+        <x:v>Formulário completo e salvo por 14 dias; SQL, Python, GCP e ETL/ELT foram valorizados, sem alegar Snowflake/dbt como experiência. Envio final bloqueado por reCAPTCHA.</x:v>
+      </x:c>
+      <x:c r="F90" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G90" s="30" t="str">
+        <x:v>Concluir a verificação normal no Indeed e confirmar o recibo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="62" customHeight="1">
+      <x:c r="A91" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B91" s="28" t="str">
+        <x:v>Indeed — VESTE SA ESTILO</x:v>
+      </x:c>
+      <x:c r="C91" s="28" t="str">
+        <x:v>Desenvolvedor Full Stack Jr</x:v>
+      </x:c>
+      <x:c r="D91" s="28" t="str">
+        <x:v>Rascunho 100% e reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="E91" s="28" t="str">
+        <x:v>Formulário completo e salvo por 14 dias com currículo técnico. A vaga é aderente a React, TypeScript, Node, APIs, Git e testes; envio final bloqueado por reCAPTCHA.</x:v>
+      </x:c>
+      <x:c r="F91" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G91" s="30" t="str">
+        <x:v>Concluir a verificação normal no Indeed e confirmar o recibo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="62" customHeight="1">
+      <x:c r="A92" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B92" s="28" t="str">
+        <x:v>Indeed — Assertiv</x:v>
+      </x:c>
+      <x:c r="C92" s="28" t="str">
+        <x:v>Analista de desenvolvedor JavaScript</x:v>
+      </x:c>
+      <x:c r="D92" s="28" t="str">
+        <x:v>Requisito de experiência não verificável</x:v>
+      </x:c>
+      <x:c r="E92" s="28" t="str">
+        <x:v>O formulário exige ao menos um ano numérico de experiência em tecnologias e no cargo. Sem período confirmado pelo candidato, o rascunho foi salvo a 50% sem inventar tempo de experiência.</x:v>
+      </x:c>
+      <x:c r="F92" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G92" s="30" t="str">
+        <x:v>Confirmar o período factual que pode ser declarado antes de enviar.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="62" customHeight="1">
+      <x:c r="A93" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B93" s="28" t="str">
+        <x:v>Indeed → Gupy — Saquers Tech</x:v>
+      </x:c>
+      <x:c r="C93" s="28" t="str">
+        <x:v>Desenvolvedor(a) Node I</x:v>
+      </x:c>
+      <x:c r="D93" s="28" t="str">
+        <x:v>Dado pessoal obrigatório faltante</x:v>
+      </x:c>
+      <x:c r="E93" s="28" t="str">
+        <x:v>A Gupy exigiu nome completo do pai, além de RG, nome da mãe, pretensão e experiência. O dado não foi fornecido, portanto não foi inventado nem houve envio.</x:v>
+      </x:c>
+      <x:c r="F93" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G93" s="30" t="str">
+        <x:v>Informar o nome do pai para concluir as perguntas.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="62" customHeight="1">
+      <x:c r="A94" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B94" s="28" t="str">
+        <x:v>Indeed → Gupy — v(dev)/Visagio</x:v>
+      </x:c>
+      <x:c r="C94" s="28" t="str">
+        <x:v>Estágio Desenvolvedor(a) de Software</x:v>
+      </x:c>
+      <x:c r="D94" s="28" t="str">
+        <x:v>Dados acadêmicos obrigatórios</x:v>
+      </x:c>
+      <x:c r="E94" s="28" t="str">
+        <x:v>O banco de talentos exige CR e grade horária detalhada. Os dados não foram fornecidos nem estimados; não houve candidatura confirmada.</x:v>
+      </x:c>
+      <x:c r="F94" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G94" s="30" t="str">
+        <x:v>Informar CR e horários reais da faculdade.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="62" customHeight="1">
+      <x:c r="A95" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B95" s="28" t="str">
+        <x:v>Indeed — NSTECH / eFrete</x:v>
+      </x:c>
+      <x:c r="C95" s="28" t="str">
+        <x:v>Analista de Dados Jr</x:v>
+      </x:c>
+      <x:c r="D95" s="28" t="str">
+        <x:v>Rascunho 100% e reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="E95" s="28" t="str">
+        <x:v>LinkedIn, CPF, disponibilidade, pretensão e autoidentificação foram preenchidos de forma factual; rascunho salvo por 14 dias. Envio final bloqueado por reCAPTCHA.</x:v>
+      </x:c>
+      <x:c r="F95" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G95" s="30" t="str">
+        <x:v>Concluir a verificação normal no Indeed e confirmar o recibo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="62" customHeight="1">
+      <x:c r="A96" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B96" s="28" t="str">
+        <x:v>Indeed — TechBrabo / MONT SEGURO</x:v>
+      </x:c>
+      <x:c r="C96" s="28" t="str">
+        <x:v>Desenvolvedor Full Stack Jr</x:v>
+      </x:c>
+      <x:c r="D96" s="28" t="str">
+        <x:v>Rascunho 100% e reCAPTCHA</x:v>
+      </x:c>
+      <x:c r="E96" s="28" t="str">
+        <x:v>Vaga de R$3.300 PJ; currículo e dados cadastrais factuais preenchidos, rascunho salvo por 14 dias. Envio final bloqueado por reCAPTCHA.</x:v>
+      </x:c>
+      <x:c r="F96" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G96" s="30" t="str">
+        <x:v>Concluir a verificação normal no Indeed e confirmar o recibo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="62" customHeight="1">
+      <x:c r="A97" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B97" s="28" t="str">
+        <x:v>Indeed → Sólides — Grupo Costa Norte</x:v>
+      </x:c>
+      <x:c r="C97" s="28" t="str">
+        <x:v>Desenvolvedor de Software Júnior</x:v>
+      </x:c>
+      <x:c r="D97" s="28" t="str">
+        <x:v>Profiler comportamental</x:v>
+      </x:c>
+      <x:c r="E97" s="28" t="str">
+        <x:v>Currículo técnico revisado e salvo para vaga CLT de R$3.500; vídeo era opcional e não foi iniciado. A plataforma apresentou Profiler antes do avanço final; a candidatura não foi enviada.</x:v>
+      </x:c>
+      <x:c r="F97" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G97" s="30" t="str">
+        <x:v>Realizar o Profiler pessoalmente caso decida avançar.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="62" customHeight="1">
+      <x:c r="A98" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B98" s="28" t="str">
+        <x:v>Indeed → Jobbol — IVO Services</x:v>
+      </x:c>
+      <x:c r="C98" s="28" t="str">
+        <x:v>Analista de Sistemas em Aplicações e Full Stack Júnior</x:v>
+      </x:c>
+      <x:c r="D98" s="28" t="str">
+        <x:v>Candidatura enviada</x:v>
+      </x:c>
+      <x:c r="E98" s="28" t="str">
+        <x:v>Formulário enviado com dados factuais. O Jobbol exibiu 'Candidatura registrada com sucesso!' e protocolo DX0634400, além de aviso de e-mail e contato posterior escrito por WhatsApp.</x:v>
+      </x:c>
+      <x:c r="F98" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G98" s="30" t="str">
+        <x:v>Acompanhar o e-mail e o contato escrito; validar formato de qualquer próxima etapa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="62" customHeight="1">
+      <x:c r="A99" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B99" s="28" t="str">
+        <x:v>Indeed → Jobbol — Kriativa</x:v>
+      </x:c>
+      <x:c r="C99" s="28" t="str">
+        <x:v>Desenvolvedor Júnior de Automação</x:v>
+      </x:c>
+      <x:c r="D99" s="28" t="str">
+        <x:v>Candidatura enviada</x:v>
+      </x:c>
+      <x:c r="E99" s="28" t="str">
+        <x:v>O Jobbol exibiu 'Candidatura registrada com sucesso!' e protocolo CW1953700 para vaga com salário oficial de R$3.000. Nenhuma etapa audiovisual ou avaliação foi iniciada.</x:v>
+      </x:c>
+      <x:c r="F99" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G99" s="30" t="str">
+        <x:v>Acompanhar confirmação por e-mail e quaisquer etapas posteriores em formato escrito.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="62" customHeight="1">
+      <x:c r="A100" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B100" s="28" t="str">
+        <x:v>Indeed — UP Brasil, Housi e Planeta do Bebê</x:v>
+      </x:c>
+      <x:c r="C100" s="28" t="str">
+        <x:v>Analista Sistemas Jr; Analista Dados Jr; Dev Python/Frontend Jr</x:v>
+      </x:c>
+      <x:c r="D100" s="28" t="str">
+        <x:v>Rascunhos e bloqueios reais</x:v>
+      </x:c>
+      <x:c r="E100" s="28" t="str">
+        <x:v>UP Brasil ficou salvo a 100% por reCAPTCHA normal. Housi ficou salvo a 38% por carregamento do formulário. Planeta do Bebê exigiu Profiler comportamental antes do envio. Nenhum bloqueio foi burlado e nenhuma avaliação foi respondida.</x:v>
+      </x:c>
+      <x:c r="F100" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G100" s="30" t="str">
+        <x:v>Retomar por Minhas Vagas ou plataforma respectiva com a ação indicada no controle.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="62" customHeight="1">
+      <x:c r="A101" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B101" s="28" t="str">
+        <x:v>Indeed — Partner Soluções Empresariais</x:v>
+      </x:c>
+      <x:c r="C101" s="28" t="str">
+        <x:v>Desenvolvedor de Sistemas Júnior</x:v>
+      </x:c>
+      <x:c r="D101" s="28" t="str">
+        <x:v>Anúncio expirado</x:v>
+      </x:c>
+      <x:c r="E101" s="28" t="str">
+        <x:v>O Indeed confirmou que a vaga de R$3.000–5.000 expirou durante a revalidação, antes de qualquer candidatura.</x:v>
+      </x:c>
+      <x:c r="F101" s="29" t="str">
+        <x:v>Encerrado</x:v>
+      </x:c>
+      <x:c r="G101" s="30" t="str">
+        <x:v>Monitorar repostagem equivalente; não tentar candidatura no anúncio encerrado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="62" customHeight="1">
+      <x:c r="A102" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B102" s="28" t="str">
+        <x:v>Indeed — fila revalidada de salário divulgado</x:v>
+      </x:c>
+      <x:c r="C102" s="28" t="str">
+        <x:v>Juriscont, RH Sales Center, ASC Brazil, IB Comércio e Partners Comunicação</x:v>
+      </x:c>
+      <x:c r="D102" s="28" t="str">
+        <x:v>Fila de alta prioridade</x:v>
+      </x:c>
+      <x:c r="E102" s="28" t="str">
+        <x:v>Foram identificadas vagas técnicas a partir de R$3.500 e com aderência real a React/Node, APIs, SQL, Docker, automação e IA. Nenhum formulário foi iniciado depois que a conexão automática do Firefox com o Indeed foi perdida.</x:v>
+      </x:c>
+      <x:c r="F102" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G102" s="30" t="str">
+        <x:v>Retomar uma a uma, revalidar cada anúncio e personalizar a candidatura antes de enviar.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="62" customHeight="1">
+      <x:c r="A103" s="61" t="str">
+        <x:v>30/09/2026</x:v>
+      </x:c>
+      <x:c r="B103" s="28" t="str">
+        <x:v>Indeed — navegador</x:v>
+      </x:c>
+      <x:c r="C103" s="28" t="str">
+        <x:v>Sessão de automação</x:v>
+      </x:c>
+      <x:c r="D103" s="28" t="str">
+        <x:v>Conexão indisponível</x:v>
+      </x:c>
+      <x:c r="E103" s="28" t="str">
+        <x:v>A extensão/sessão que lista e controla as abas do Firefox deixou de responder. Foi feito novo teste após abrir o Firefox, mas não houve conexão de extensão; a busca e a fila foram preservadas no controle.</x:v>
+      </x:c>
+      <x:c r="F103" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G103" s="30" t="str">
+        <x:v>Reconectar a extensão do Firefox e retomar a fila por prioridade, mantendo uma aba por vez.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B104" s="28" t="str">
+        <x:v>Currículo mestre</x:v>
+      </x:c>
+      <x:c r="C104" s="28" t="str">
+        <x:v>Atualização factual do perfil</x:v>
+      </x:c>
+      <x:c r="D104" s="28" t="str">
+        <x:v>CV atualizado</x:v>
+      </x:c>
+      <x:c r="E104" s="28" t="str">
+        <x:v>Foi gerado currículo mestre em português com experiência profissional full stack na Performance Lab desde dez/2025 e atuação via CNPJ em software e automação, incluindo NOW PRO com PHP, frontend, scraping e integrações de APIs.</x:v>
+      </x:c>
+      <x:c r="F104" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G104" s="30" t="str">
+        <x:v>Usar este CV nas próximas candidaturas e substituir o arquivo nos perfis quando o Firefox voltar a responder.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B105" s="28" t="str">
+        <x:v>Catho e InfoJobs</x:v>
+      </x:c>
+      <x:c r="C105" s="28" t="str">
+        <x:v>10 candidaturas técnicas</x:v>
+      </x:c>
+      <x:c r="D105" s="28" t="str">
+        <x:v>Candidaturas confirmadas</x:v>
+      </x:c>
+      <x:c r="E105" s="28" t="str">
+        <x:v>Foram confirmadas duas candidaturas no Catho e oito no InfoJobs, com links e próximos passos registrados no controle. Foram usadas respostas factuais e cartas personalizadas; nenhuma avaliação, áudio ou vídeo foi iniciado.</x:v>
+      </x:c>
+      <x:c r="F105" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G105" s="30" t="str">
+        <x:v>Acompanhar e-mail e portais. Se recrutadores retomarem formulários antigos, atualizar as respostas que ficaram desatualizadas após a correção do histórico full stack.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B106" s="28" t="str">
+        <x:v>Firefox / perfis</x:v>
+      </x:c>
+      <x:c r="C106" s="28" t="str">
+        <x:v>Gupy, InfoJobs, Catho e Indeed</x:v>
+      </x:c>
+      <x:c r="D106" s="28" t="str">
+        <x:v>Atualização de currículo pendente</x:v>
+      </x:c>
+      <x:c r="E106" s="28" t="str">
+        <x:v>O currículo mestre está pronto para upload, mas a extensão do Firefox ficou conectada sem responder a listagem, leitura ou manipulação de abas. Nenhum perfil foi alterado sem confirmação visível.</x:v>
+      </x:c>
+      <x:c r="F106" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G106" s="30" t="str">
+        <x:v>Reconectar a sessão/ponte do Firefox, revisar as abas abertas antes de fechar e substituir o CV nos quatro portais.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B107" s="28" t="str">
+        <x:v>InfoJobs</x:v>
+      </x:c>
+      <x:c r="C107" s="28" t="str">
+        <x:v>Macam Brasil - Desenvolvedor de Software</x:v>
+      </x:c>
+      <x:c r="D107" s="28" t="str">
+        <x:v>Informação obrigatória pendente</x:v>
+      </x:c>
+      <x:c r="E107" s="28" t="str">
+        <x:v>A candidatura não foi enviada porque o formulário perguntou se o candidato mora em Pirituba/Jaraguá. O endereço não foi confirmado e a resposta não foi presumida.</x:v>
+      </x:c>
+      <x:c r="F107" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G107" s="30" t="str">
+        <x:v>Confirmar a localização real antes de responder e concluir a candidatura.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B108" s="28" t="str">
+        <x:v>Critérios de busca</x:v>
+      </x:c>
+      <x:c r="C108" s="28" t="str">
+        <x:v>Senioridade</x:v>
+      </x:c>
+      <x:c r="D108" s="28" t="str">
+        <x:v>Regra atualizada</x:v>
+      </x:c>
+      <x:c r="E108" s="28" t="str">
+        <x:v>A busca passa a excluir vagas sênior. A prioridade é júnior, trainee, assistente e entry level; vagas pleno entram somente quando os requisitos reais forem compatíveis com perfil júnior.</x:v>
+      </x:c>
+      <x:c r="F108" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G108" s="30" t="str">
+        <x:v>Aplicar esta regra à fila existente e a todas as novas pesquisas.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F6:F59">
     <x:cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="Concluído"/>
@@ -6431,7 +10283,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c7faf60f38946a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa7256f31b2b4d95"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Registra fila júnior de São Paulo
</commit_message>
<xml_diff>
--- a/planilhas/Controle_Candidaturas_Fintech_Guilherme_PUBLICO.xlsx
+++ b/planilhas/Controle_Candidaturas_Fintech_Guilherme_PUBLICO.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidaturas" sheetId="1" r:id="R19ddb00af5ca4b5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log de auditoria" sheetId="2" r:id="Rb878a634a4ea4c18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidaturas" sheetId="1" r:id="Rbadd5d02c88f434e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log de auditoria" sheetId="2" r:id="R5537a808c508450b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -503,7 +503,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CandidaturasTable" displayName="CandidaturasTable" ref="A9:K171" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CandidaturasTable" displayName="CandidaturasTable" ref="A9:K179" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Status"/>
     <x:tableColumn id="2" name="Empresa"/>
@@ -793,7 +793,7 @@
         <x:v>Candidaturas confirmadas</x:v>
       </x:c>
       <x:c r="B7" s="9" t="n">
-        <x:f>SUM(L10:L171)</x:f>
+        <x:f>SUM(L10:L179)</x:f>
         <x:v>83</x:v>
       </x:c>
       <x:c r="C7" s="8"/>
@@ -801,16 +801,16 @@
         <x:v>Itens em controle</x:v>
       </x:c>
       <x:c r="E7" s="9" t="n">
-        <x:f>COUNTA(A10:A171)</x:f>
-        <x:v>162</x:v>
+        <x:f>COUNTA(A10:A179)</x:f>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="F7" s="8"/>
       <x:c r="G7" s="8" t="str">
         <x:v>Pendentes</x:v>
       </x:c>
       <x:c r="H7" s="9" t="n">
-        <x:f>SUM(M10:M171)</x:f>
-        <x:v>71</x:v>
+        <x:f>SUM(M10:M179)</x:f>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
@@ -7814,24 +7814,368 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="172">
-      <x:c r="A172" s="32" t="str">
+    <x:row r="172" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A172" s="63" t="str">
+        <x:v>Pendente — revalidar e candidatar</x:v>
+      </x:c>
+      <x:c r="B172" s="63" t="str">
+        <x:v>Lina Infratech</x:v>
+      </x:c>
+      <x:c r="C172" s="63" t="str">
+        <x:v>Desenvolvedor(a) Backend Júnior</x:v>
+      </x:c>
+      <x:c r="D172" s="63" t="str">
+        <x:v>Desenvolvimento backend</x:v>
+      </x:c>
+      <x:c r="E172" s="63" t="str">
+        <x:v>Remoto; CLT; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F172" s="63" t="str">
+        <x:v>https://lina.factorialhr.com.br/job_posting/desenvolvedor-a-backend-junior-324661</x:v>
+      </x:c>
+      <x:c r="G172" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H172" s="63" t="str">
+        <x:v>Revalidar anúncio e personalizar com Node.js, APIs REST, Git, testes, projetos próprios e ADS em andamento.</x:v>
+      </x:c>
+      <x:c r="I172" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J172" s="63" t="str">
+        <x:v>Triagem de São Paulo/Grande SP: vaga júnior com requisitos de Node.js, REST, Git e testes. A descrição aceita experiência acadêmica, pessoal ou profissional; não foi iniciada candidatura.</x:v>
+      </x:c>
+      <x:c r="K172" s="63" t="str">
+        <x:v>Não — candidatura ainda não iniciada</x:v>
+      </x:c>
+      <x:c r="L172" t="n">
+        <x:f>IF(LEFT(K172,3)="Sim",1,0)+IF(LEFT(K172,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M172" t="n">
+        <x:f>IF(LEFT(A172,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A173" s="63" t="str">
+        <x:v>Pendente — revalidar e candidatar</x:v>
+      </x:c>
+      <x:c r="B173" s="63" t="str">
+        <x:v>TOTVS</x:v>
+      </x:c>
+      <x:c r="C173" s="63" t="str">
+        <x:v>Engenharia de Software Fullstack Júnior (Node.js/TypeScript/React)</x:v>
+      </x:c>
+      <x:c r="D173" s="63" t="str">
+        <x:v>Desenvolvimento full stack</x:v>
+      </x:c>
+      <x:c r="E173" s="63" t="str">
+        <x:v>São Paulo/SP; híbrido; remuneração oficial não divulgada</x:v>
+      </x:c>
+      <x:c r="F173" s="63" t="str">
+        <x:v>https://atracaodetalentos.totvs.app/vempratotvs/extended/</x:v>
+      </x:c>
+      <x:c r="G173" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H173" s="63" t="str">
+        <x:v>Revalidar a vaga específica no portal e personalizar com Node.js, TypeScript, React, REST, Docker, AWS, CI/CD e testes.</x:v>
+      </x:c>
+      <x:c r="I173" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J173" s="63" t="str">
+        <x:v>Triagem de São Paulo/Grande SP: requisitos relatados são aderentes à stack atual. Qualquer faixa vista em agregador deve ser tratada somente como estimativa, não como salário oficial.</x:v>
+      </x:c>
+      <x:c r="K173" s="63" t="str">
+        <x:v>Não — candidatura ainda não iniciada</x:v>
+      </x:c>
+      <x:c r="L173" t="n">
+        <x:f>IF(LEFT(K173,3)="Sim",1,0)+IF(LEFT(K173,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M173" t="n">
+        <x:f>IF(LEFT(A173,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A174" s="63" t="str">
+        <x:v>Pendente — revalidar e candidatar</x:v>
+      </x:c>
+      <x:c r="B174" s="63" t="str">
+        <x:v>Cinga Tech</x:v>
+      </x:c>
+      <x:c r="C174" s="63" t="str">
+        <x:v>Desenvolvedor(a) Júnior</x:v>
+      </x:c>
+      <x:c r="D174" s="63" t="str">
+        <x:v>Automação e integrações</x:v>
+      </x:c>
+      <x:c r="E174" s="63" t="str">
+        <x:v>São Paulo/SP; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F174" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=975d6f32548d1e93</x:v>
+      </x:c>
+      <x:c r="G174" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H174" s="63" t="str">
+        <x:v>Revalidar anúncio e personalizar com Node.js, Python, SQL, APIs, automação, IA e Git.</x:v>
+      </x:c>
+      <x:c r="I174" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J174" s="63" t="str">
+        <x:v>Triagem de São Paulo/Grande SP: vaga júnior com foco em automação e integrações, tecnicamente aderente. Nenhuma candidatura foi iniciada.</x:v>
+      </x:c>
+      <x:c r="K174" s="63" t="str">
+        <x:v>Não — candidatura ainda não iniciada</x:v>
+      </x:c>
+      <x:c r="L174" t="n">
+        <x:f>IF(LEFT(K174,3)="Sim",1,0)+IF(LEFT(K174,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M174" t="n">
+        <x:f>IF(LEFT(A174,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A175" s="63" t="str">
+        <x:v>Pendente — revalidar e candidatar</x:v>
+      </x:c>
+      <x:c r="B175" s="63" t="str">
+        <x:v>Gestalt Cravo</x:v>
+      </x:c>
+      <x:c r="C175" s="63" t="str">
+        <x:v>Desenvolvedor Full Stack N1</x:v>
+      </x:c>
+      <x:c r="D175" s="63" t="str">
+        <x:v>Desenvolvimento full stack</x:v>
+      </x:c>
+      <x:c r="E175" s="63" t="str">
+        <x:v>Barueri/SP; remoto; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F175" s="63" t="str">
+        <x:v>https://www.simplyhired.com.br/job/anb_KzXgilX2mXoA2KpxJ27gdyT4bhHS2CmkQTwPhSc9FG1xuqwAuQ</x:v>
+      </x:c>
+      <x:c r="G175" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H175" s="63" t="str">
+        <x:v>Revalidar empresa e anúncio antes de enviar; personalizar com JavaScript/TypeScript, Python, React, Node, APIs, webhooks, SQL, Docker, cloud e IA.</x:v>
+      </x:c>
+      <x:c r="I175" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J175" s="63" t="str">
+        <x:v>Triagem de São Paulo/Grande SP: descrita como júnior/N1 e sem exigência de domínio integral da stack. Link é de agregador, portanto exige validação antes de qualquer candidatura.</x:v>
+      </x:c>
+      <x:c r="K175" s="63" t="str">
+        <x:v>Não — candidatura ainda não iniciada</x:v>
+      </x:c>
+      <x:c r="L175" t="n">
+        <x:f>IF(LEFT(K175,3)="Sim",1,0)+IF(LEFT(K175,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M175" t="n">
+        <x:f>IF(LEFT(A175,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A176" s="63" t="str">
+        <x:v>Pendente — verificar duplicidade</x:v>
+      </x:c>
+      <x:c r="B176" s="63" t="str">
+        <x:v>SCS Saneamento</x:v>
+      </x:c>
+      <x:c r="C176" s="63" t="str">
+        <x:v>Desenvolvedor Full Stack Júnior</x:v>
+      </x:c>
+      <x:c r="D176" s="63" t="str">
+        <x:v>Desenvolvimento full stack</x:v>
+      </x:c>
+      <x:c r="E176" s="63" t="str">
+        <x:v>São Paulo/SP (Berrini); presencial; PJ; salário divulgado R$ 6.000 a R$ 6.500</x:v>
+      </x:c>
+      <x:c r="F176" s="63" t="str">
+        <x:v>https://scs-saneamento.pandape.infojobs.com.br/Detail/3683559</x:v>
+      </x:c>
+      <x:c r="G176" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H176" s="63" t="str">
+        <x:v>Checar se existe candidatura anterior antes de iniciar. Se não houver, personalizar com React, Node, PostgreSQL/MySQL, APIs REST e testes; Kotlin é ponto de estudo.</x:v>
+      </x:c>
+      <x:c r="I176" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J176" s="63" t="str">
+        <x:v>Triagem de São Paulo/Grande SP: vaga júnior de alta aderência e salário divulgado. Foi marcada para revisar duplicidade porque há registro histórico de possível candidatura semelhante fora do link atual.</x:v>
+      </x:c>
+      <x:c r="K176" s="63" t="str">
+        <x:v>Não — candidatura ainda não iniciada</x:v>
+      </x:c>
+      <x:c r="L176" t="n">
+        <x:f>IF(LEFT(K176,3)="Sim",1,0)+IF(LEFT(K176,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M176" t="n">
+        <x:f>IF(LEFT(A176,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A177" s="63" t="str">
+        <x:v>Pendente — revalidar e candidatar</x:v>
+      </x:c>
+      <x:c r="B177" s="63" t="str">
+        <x:v>Datum</x:v>
+      </x:c>
+      <x:c r="C177" s="63" t="str">
+        <x:v>Pessoa Desenvolvedora Java Júnior (NextGen)</x:v>
+      </x:c>
+      <x:c r="D177" s="63" t="str">
+        <x:v>Desenvolvimento backend</x:v>
+      </x:c>
+      <x:c r="E177" s="63" t="str">
+        <x:v>São Paulo/SP; híbrido (Zona Sul); remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F177" s="63" t="str">
+        <x:v>https://datum.jobs.recrut.ai/gender-predict/job/XV0CV0</x:v>
+      </x:c>
+      <x:c r="G177" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H177" s="63" t="str">
+        <x:v>Revalidar anúncio e personalizar com base em backend, APIs, SQL, Docker e capacidade de estudar Java; Java é diferencial/desenvolvimento a fortalecer.</x:v>
+      </x:c>
+      <x:c r="I177" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J177" s="63" t="str">
+        <x:v>Triagem de São Paulo/Grande SP: programa de início de carreira; experiência de um ano com Java aparece como desejável, não como requisito eliminatório. Nenhuma candidatura foi iniciada.</x:v>
+      </x:c>
+      <x:c r="K177" s="63" t="str">
+        <x:v>Não — candidatura ainda não iniciada</x:v>
+      </x:c>
+      <x:c r="L177" t="n">
+        <x:f>IF(LEFT(K177,3)="Sim",1,0)+IF(LEFT(K177,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M177" t="n">
+        <x:f>IF(LEFT(A177,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A178" s="63" t="str">
+        <x:v>Pendente — revalidar e candidatar</x:v>
+      </x:c>
+      <x:c r="B178" s="63" t="str">
+        <x:v>NOVA S.A.</x:v>
+      </x:c>
+      <x:c r="C178" s="63" t="str">
+        <x:v>Desenvolvedor de RPA Júnior</x:v>
+      </x:c>
+      <x:c r="D178" s="63" t="str">
+        <x:v>Automação e dados</x:v>
+      </x:c>
+      <x:c r="E178" s="63" t="str">
+        <x:v>São Paulo/SP; presencial; salário divulgado R$ 4.000 a R$ 5.000</x:v>
+      </x:c>
+      <x:c r="F178" s="63" t="str">
+        <x:v>https://novagencia.vagas.solides.com.br/</x:v>
+      </x:c>
+      <x:c r="G178" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H178" s="63" t="str">
+        <x:v>Revalidar vaga específica no portal e personalizar com automação, APIs, OCR, ETL, dados e IA; RPA/Power BI são pontos de estudo.</x:v>
+      </x:c>
+      <x:c r="I178" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J178" s="63" t="str">
+        <x:v>Triagem de São Paulo/Grande SP: vaga júnior com remuneração divulgada. Boa transição para automação; precisa validar requisitos específicos de RPA, ML e Power BI antes de enviar.</x:v>
+      </x:c>
+      <x:c r="K178" s="63" t="str">
+        <x:v>Não — candidatura ainda não iniciada</x:v>
+      </x:c>
+      <x:c r="L178" t="n">
+        <x:f>IF(LEFT(K178,3)="Sim",1,0)+IF(LEFT(K178,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M178" t="n">
+        <x:f>IF(LEFT(A178,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A179" s="63" t="str">
+        <x:v>Pendente — revalidar e candidatar</x:v>
+      </x:c>
+      <x:c r="B179" s="63" t="str">
+        <x:v>Saúde Link</x:v>
+      </x:c>
+      <x:c r="C179" s="63" t="str">
+        <x:v>Analista Desenvolvedor Pleno</x:v>
+      </x:c>
+      <x:c r="D179" s="63" t="str">
+        <x:v>Desenvolvimento e integrações</x:v>
+      </x:c>
+      <x:c r="E179" s="63" t="str">
+        <x:v>São Paulo/SP (Chácara Santo Antônio); CLT presencial; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F179" s="63" t="str">
+        <x:v>https://www.infojobs.com.br/vaga-de-analista-desenvolvedor-pleno-em-sao-paulo__12066791.aspx</x:v>
+      </x:c>
+      <x:c r="G179" s="63" t="str">
+        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+      </x:c>
+      <x:c r="H179" s="63" t="str">
+        <x:v>Revalidar anúncio e personalizar com sistemas web, APIs, integrações, bancos de dados, automação e Git. Informar formação em andamento de forma factual.</x:v>
+      </x:c>
+      <x:c r="I179" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J179" s="63" t="str">
+        <x:v>Exceção de pleno analisada: a descrição aceita formação completa ou em andamento e não declara anos mínimos nem inglês obrigatório. Mantida apenas por ser compatível com perfil júnior na prática; não há candidatura iniciada.</x:v>
+      </x:c>
+      <x:c r="K179" s="63" t="str">
+        <x:v>Não — candidatura ainda não iniciada</x:v>
+      </x:c>
+      <x:c r="L179" t="n">
+        <x:f>IF(LEFT(K179,3)="Sim",1,0)+IF(LEFT(K179,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M179" t="n">
+        <x:f>IF(LEFT(A179,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180">
+      <x:c r="A180" s="32" t="str">
         <x:v>Nota: ‘Sim’ significa recibo de e-mail localizado; ‘Portal’ significa confirmação/etapa verificada no portal. E-mails de inscrição iniciada não são tratados como candidatura enviada. Não há dados pessoais sensíveis nesta planilha.</x:v>
       </x:c>
-      <x:c r="B172" s="63"/>
-      <x:c r="C172" s="63"/>
-      <x:c r="D172" s="63"/>
-      <x:c r="E172" s="63"/>
-      <x:c r="F172" s="63"/>
-      <x:c r="G172" s="63"/>
-      <x:c r="H172" s="63"/>
-      <x:c r="I172" s="63"/>
-      <x:c r="J172" s="63"/>
-      <x:c r="K172" s="63"/>
+      <x:c r="B180" s="63"/>
+      <x:c r="C180" s="63"/>
+      <x:c r="D180" s="63"/>
+      <x:c r="E180" s="63"/>
+      <x:c r="F180" s="63"/>
+      <x:c r="G180" s="63"/>
+      <x:c r="H180" s="63"/>
+      <x:c r="I180" s="63"/>
+      <x:c r="J180" s="63"/>
+      <x:c r="K180" s="63"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A172:K172"/>
+    <x:mergeCell ref="A180:K180"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A10:A108">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Enviada"/>
@@ -7849,7 +8193,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec6b5206a6c94d6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59c410af76c540fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10272,6 +10616,29 @@
         <x:v>Aplicar esta regra à fila existente e a todas as novas pesquisas.</x:v>
       </x:c>
     </x:row>
+    <x:row r="109">
+      <x:c r="A109" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B109" s="28" t="str">
+        <x:v>Pesquisa São Paulo / Grande SP</x:v>
+      </x:c>
+      <x:c r="C109" s="28" t="str">
+        <x:v>Fila júnior e pleno compatível</x:v>
+      </x:c>
+      <x:c r="D109" s="28" t="str">
+        <x:v>Vagas priorizadas</x:v>
+      </x:c>
+      <x:c r="E109" s="28" t="str">
+        <x:v>Foram registradas oportunidades júnior e uma exceção pleno com requisitos júnior-compatíveis. Vagas sênior, staff, liderança e pleno com exigência acima do perfil foram excluídas da fila.</x:v>
+      </x:c>
+      <x:c r="F109" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G109" s="30" t="str">
+        <x:v>Revalidar os anúncios um a um antes de candidatar; não duplicar as candidaturas já registradas.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F6:F59">
     <x:cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="Concluído"/>
@@ -10283,7 +10650,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa7256f31b2b4d95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd37e52654137471b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza CV Performance Lab e controle publico
</commit_message>
<xml_diff>
--- a/planilhas/Controle_Candidaturas_Fintech_Guilherme_PUBLICO.xlsx
+++ b/planilhas/Controle_Candidaturas_Fintech_Guilherme_PUBLICO.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidaturas" sheetId="1" r:id="Rbadd5d02c88f434e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log de auditoria" sheetId="2" r:id="R5537a808c508450b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidaturas" sheetId="1" r:id="Rf3f3cbbff1874fc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log de auditoria" sheetId="2" r:id="R6f36761ee7774604"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -503,7 +503,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CandidaturasTable" displayName="CandidaturasTable" ref="A9:K179" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CandidaturasTable" displayName="CandidaturasTable" ref="A9:K193" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Status"/>
     <x:tableColumn id="2" name="Empresa"/>
@@ -793,24 +793,24 @@
         <x:v>Candidaturas confirmadas</x:v>
       </x:c>
       <x:c r="B7" s="9" t="n">
-        <x:f>SUM(L10:L179)</x:f>
-        <x:v>83</x:v>
+        <x:f>SUM(L10:L193)</x:f>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="C7" s="8"/>
       <x:c r="D7" s="8" t="str">
         <x:v>Itens em controle</x:v>
       </x:c>
       <x:c r="E7" s="9" t="n">
-        <x:f>COUNTA(A10:A179)</x:f>
-        <x:v>170</x:v>
+        <x:f>COUNTA(A10:A193)</x:f>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="F7" s="8"/>
       <x:c r="G7" s="8" t="str">
         <x:v>Pendentes</x:v>
       </x:c>
       <x:c r="H7" s="9" t="n">
-        <x:f>SUM(M10:M179)</x:f>
-        <x:v>79</x:v>
+        <x:f>SUM(M10:M193)</x:f>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
@@ -2871,7 +2871,7 @@
     </x:row>
     <x:row r="57" ht="90" customHeight="1">
       <x:c r="A57" s="23" t="str">
-        <x:v>Pendente — dados cadastrais</x:v>
+        <x:v>Enviada</x:v>
       </x:c>
       <x:c r="B57" s="15" t="str">
         <x:v>UOL</x:v>
@@ -2892,24 +2892,24 @@
         <x:v>Sem audiovisual declarado</x:v>
       </x:c>
       <x:c r="H57" s="18" t="str">
-        <x:v>Aguardar órgão/UF emissor do RG, nome completo do pai e naturalidade; então preencher, personalizar, revisar e pedir confirmação final</x:v>
+        <x:v>Acompanhar e-mail e portal; se houver teste, o candidato deve realizá-lo pessoalmente.</x:v>
       </x:c>
       <x:c r="I57" s="19" t="str">
-        <x:v>21/09/2026</x:v>
+        <x:v>02/10/2026</x:v>
       </x:c>
       <x:c r="J57" s="18" t="str">
-        <x:v>Formulário retomado em 21/09. As respostas factuais de não indicação e de não vínculo com a UOL foram salvas. RG, órgão/UF emissor, mãe, pai, naturalidade e pretensão são campos eliminatórios; faltam órgão/UF emissor, nome completo do pai e cidade/UF de nascimento. Boa aderência em TypeScript, React, APIs, Git, banco de dados, Docker, testes e CI/CD; sem alegar Node/NestJS ou AWS.</x:v>
+        <x:v>Candidatura finalizada na Gupy em 02/10 com currículo atualizado e apresentação personalizada. Foram destacadas experiência profissional full stack na Performance Lab, .NET/C#, React/TypeScript, PostgreSQL, APIs, integrações e testes; Node.js/NestJS ficou limitado a projetos práticos, sem inflar experiência profissional.</x:v>
       </x:c>
       <x:c r="K57" s="24" t="str">
-        <x:v>E-mail recebido — dados pendentes 21/09</x:v>
+        <x:v>Sim — finalizada na Gupy 02/10</x:v>
       </x:c>
       <x:c r="L57" t="n">
         <x:f>IF(LEFT(K57,3)="Sim",1,0)+IF(LEFT(K57,6)="Portal",1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M57" t="n">
         <x:f>IF(LEFT(A57,8)="Pendente",1,0)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="60" customHeight="1">
@@ -8158,24 +8158,626 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="180">
-      <x:c r="A180" s="32" t="str">
+    <x:row r="180" ht="66" hidden="0" customHeight="1">
+      <x:c r="A180" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B180" s="63" t="str">
+        <x:v>B2Finance / H&amp;CO</x:v>
+      </x:c>
+      <x:c r="C180" s="63" t="str">
+        <x:v>Full Stack Júnior</x:v>
+      </x:c>
+      <x:c r="D180" s="63" t="str">
+        <x:v>Desenvolvimento full stack</x:v>
+      </x:c>
+      <x:c r="E180" s="63" t="str">
+        <x:v>Remoto; PJ; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F180" s="63" t="str">
+        <x:v>https://b2financebpo.pandape.infojobs.com.br/Detail/3742624</x:v>
+      </x:c>
+      <x:c r="G180" s="63" t="str">
+        <x:v>Não informado</x:v>
+      </x:c>
+      <x:c r="H180" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal; manter currículo com Performance Lab e projetos de integração atualizado.</x:v>
+      </x:c>
+      <x:c r="I180" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J180" s="63" t="str">
+        <x:v>O portal reconheceu o e-mail como participante da seleção em 02/10. Registro incluído para evitar candidatura duplicada. A vaga aceita projetos práticos e tem aderência a React/Next, Node/Python, PostgreSQL, APIs, Git, Docker e IA.</x:v>
+      </x:c>
+      <x:c r="K180" s="63" t="str">
+        <x:v>Portal — participação já existente 02/10</x:v>
+      </x:c>
+      <x:c r="L180" t="n">
+        <x:f>IF(LEFT(K180,3)="Sim",1,0)+IF(LEFT(K180,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M180" t="n">
+        <x:f>IF(LEFT(A180,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A181" s="63" t="str">
+        <x:v>Pendente — upload de currículo</x:v>
+      </x:c>
+      <x:c r="B181" s="63" t="str">
+        <x:v>Serasa Experian</x:v>
+      </x:c>
+      <x:c r="C181" s="63" t="str">
+        <x:v>Analista de Desenvolvimento de Software I — Backend Java</x:v>
+      </x:c>
+      <x:c r="D181" s="63" t="str">
+        <x:v>Desenvolvimento backend</x:v>
+      </x:c>
+      <x:c r="E181" s="63" t="str">
+        <x:v>Home office; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F181" s="63" t="str">
+        <x:v>https://jobs.smartrecruiters.com/Experian/744000149686309-analista-de-desenvolvimento-de-software-ii</x:v>
+      </x:c>
+      <x:c r="G181" s="63" t="str">
+        <x:v>Não informado</x:v>
+      </x:c>
+      <x:c r="H181" s="63" t="str">
+        <x:v>Anexar o currículo mestre atualizado no formulário SmartRecruiters e revisar a mensagem personalizada antes do envio.</x:v>
+      </x:c>
+      <x:c r="I181" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J181" s="63" t="str">
+        <x:v>Vaga júnior compatível com Java, REST, SQL, Git, testes, Docker, CI/CD, cloud e agentes de IA. Formulário aberto, mas o portal exige upload local do PDF antes do envio; candidatura ainda não foi enviada.</x:v>
+      </x:c>
+      <x:c r="K181" s="63" t="str">
+        <x:v>Não — upload obrigatório pendente</x:v>
+      </x:c>
+      <x:c r="L181" t="n">
+        <x:f>IF(LEFT(K181,3)="Sim",1,0)+IF(LEFT(K181,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M181" t="n">
+        <x:f>IF(LEFT(A181,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182" ht="66" hidden="0" customHeight="1">
+      <x:c r="A182" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B182" s="63" t="str">
+        <x:v>SoftExpert</x:v>
+      </x:c>
+      <x:c r="C182" s="63" t="str">
+        <x:v>Desenvolvedor(a) Full Stack Júnior (PHP/React)</x:v>
+      </x:c>
+      <x:c r="D182" s="63" t="str">
+        <x:v>Desenvolvimento full stack</x:v>
+      </x:c>
+      <x:c r="E182" s="63" t="str">
+        <x:v>Remoto Brasil; CLT; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F182" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G182" s="63" t="str">
+        <x:v>Avaliação comportamental futura — realizar pessoalmente se acionada</x:v>
+      </x:c>
+      <x:c r="H182" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal. Preparar exemplos factuais de PHP, React, APIs REST, SQL/PostgreSQL e Git.</x:v>
+      </x:c>
+      <x:c r="I182" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J182" s="63" t="str">
+        <x:v>Candidatura Gupy finalizada com apresentação personalizada. Foram destacados Performance Lab/KNOTEN, PHP e frontend para NOW PRO, scraping e integrações de APIs, sem alegar experiência não comprovada.</x:v>
+      </x:c>
+      <x:c r="K182" s="63" t="str">
+        <x:v>Sim — candidatura finalizada na Gupy 02/10</x:v>
+      </x:c>
+      <x:c r="L182" t="n">
+        <x:f>IF(LEFT(K182,3)="Sim",1,0)+IF(LEFT(K182,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M182" t="n">
+        <x:f>IF(LEFT(A182,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A183" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B183" s="63" t="str">
+        <x:v>Skeelo</x:v>
+      </x:c>
+      <x:c r="C183" s="63" t="str">
+        <x:v>Backend Engineer I</x:v>
+      </x:c>
+      <x:c r="D183" s="63" t="str">
+        <x:v>Desenvolvimento backend</x:v>
+      </x:c>
+      <x:c r="E183" s="63" t="str">
+        <x:v>Remoto Brasil; modalidade de contratação e remuneração não divulgadas</x:v>
+      </x:c>
+      <x:c r="F183" s="63" t="str">
+        <x:v>https://ats.rippling.com/skeelo/jobs/4009c7eb-ec6d-43cc-bbb7-be859bc7cb34</x:v>
+      </x:c>
+      <x:c r="G183" s="63" t="str">
+        <x:v>Nenhuma avaliação declarada no envio</x:v>
+      </x:c>
+      <x:c r="H183" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal. Preparar exemplos de APIs, Node.js em projetos práticos, PostgreSQL, Git, Docker e observabilidade.</x:v>
+      </x:c>
+      <x:c r="I183" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J183" s="63" t="str">
+        <x:v>Portal Rippling confirmou o envio. Pretensão informada: R$ 5.000 brutos/mês, negociável; inglês B1 e espanhol A2 foram declarados de forma factual.</x:v>
+      </x:c>
+      <x:c r="K183" s="63" t="str">
+        <x:v>Portal — candidatura confirmada 02/10</x:v>
+      </x:c>
+      <x:c r="L183" t="n">
+        <x:f>IF(LEFT(K183,3)="Sim",1,0)+IF(LEFT(K183,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M183" t="n">
+        <x:f>IF(LEFT(A183,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A184" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B184" s="63" t="str">
+        <x:v>Bullla</x:v>
+      </x:c>
+      <x:c r="C184" s="63" t="str">
+        <x:v>Analista de Dados Júnior</x:v>
+      </x:c>
+      <x:c r="D184" s="63" t="str">
+        <x:v>Dados e BI</x:v>
+      </x:c>
+      <x:c r="E184" s="63" t="str">
+        <x:v>São Paulo/SP; híbrido; CLT; remuneração a combinar</x:v>
+      </x:c>
+      <x:c r="F184" s="63" t="str">
+        <x:v>https://atracaodetalentos.totvs.app/oportunidadesbullla/61/analista-de-dados-junior</x:v>
+      </x:c>
+      <x:c r="G184" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal; não havia avaliação na submissão</x:v>
+      </x:c>
+      <x:c r="H184" s="63" t="str">
+        <x:v>Preparar exemplos de SQL, Python, automação, APIs e análise de dados. Não apresentar experiência formal de BI além do que for comprovável.</x:v>
+      </x:c>
+      <x:c r="I184" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J184" s="63" t="str">
+        <x:v>TOTVS RH confirmou: candidatura enviada com sucesso. Aderência em SQL, Python, Git, automação e dados; PySpark/Scala/Databricks ficam como pontos de estudo.</x:v>
+      </x:c>
+      <x:c r="K184" s="63" t="str">
+        <x:v>Portal — candidatura confirmada 02/10</x:v>
+      </x:c>
+      <x:c r="L184" t="n">
+        <x:f>IF(LEFT(K184,3)="Sim",1,0)+IF(LEFT(K184,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M184" t="n">
+        <x:f>IF(LEFT(A184,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A185" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B185" s="63" t="str">
+        <x:v>Viceri SEIDOR</x:v>
+      </x:c>
+      <x:c r="C185" s="63" t="str">
+        <x:v>Pessoa Desenvolvedora Full Stack Júnior — Front-End e Cloud Azure</x:v>
+      </x:c>
+      <x:c r="D185" s="63" t="str">
+        <x:v>Desenvolvimento full stack</x:v>
+      </x:c>
+      <x:c r="E185" s="63" t="str">
+        <x:v>Remoto; efetivo; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F185" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G185" s="63" t="str">
+        <x:v>Mapeamento comportamental, atenção/raciocínio lógico e teste técnico guiado podem ocorrer depois — realizar pessoalmente</x:v>
+      </x:c>
+      <x:c r="H185" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal. Revisar Angular, Node.js, Azure, OAuth 2.0, CI/CD e Docker antes de entrevistas ou testes futuros.</x:v>
+      </x:c>
+      <x:c r="I185" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J185" s="63" t="str">
+        <x:v>Candidatura finalizada na Gupy. Pretensão informada: R$ 5.000 CLT, negociável. Texto personalizado conectou Performance Lab, NOW PRO, TypeScript, APIs, Git, Docker e evolução transparente em Angular/Node/Azure.</x:v>
+      </x:c>
+      <x:c r="K185" s="63" t="str">
+        <x:v>Sim — candidatura finalizada na Gupy 02/10</x:v>
+      </x:c>
+      <x:c r="L185" t="n">
+        <x:f>IF(LEFT(K185,3)="Sim",1,0)+IF(LEFT(K185,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M185" t="n">
+        <x:f>IF(LEFT(A185,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A186" s="63" t="str">
+        <x:v>Eliminada — requisito técnico</x:v>
+      </x:c>
+      <x:c r="B186" s="63" t="str">
+        <x:v>Atento TI</x:v>
+      </x:c>
+      <x:c r="C186" s="63" t="str">
+        <x:v>Desenvolvedor Full Stack Pleno (.NET | SQL Server | Cloud)</x:v>
+      </x:c>
+      <x:c r="D186" s="63" t="str">
+        <x:v>Desenvolvimento full stack</x:v>
+      </x:c>
+      <x:c r="E186" s="63" t="str">
+        <x:v>Modalidade não declarada; salário oficial R$ 4.030; efetivo</x:v>
+      </x:c>
+      <x:c r="F186" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G186" s="63" t="str">
+        <x:v>Encerrada pelo filtro eliminatório do portal</x:v>
+      </x:c>
+      <x:c r="H186" s="63" t="str">
+        <x:v>Não reaplicar. Priorizar estudo prático de SQL Server e SSIS somente se houver interesse em vagas semelhantes.</x:v>
+      </x:c>
+      <x:c r="I186" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J186" s="63" t="str">
+        <x:v>A Gupy eliminou a candidatura pelo requisito obrigatório de experiência com SQL Server. A resposta foi mantida factual: há experiência com PostgreSQL/SQL, não com SQL Server; SSIS também foi informado como não.</x:v>
+      </x:c>
+      <x:c r="K186" s="63" t="str">
+        <x:v>Não — eliminada por requisito obrigatório 02/10</x:v>
+      </x:c>
+      <x:c r="L186" t="n">
+        <x:f>IF(LEFT(K186,3)="Sim",1,0)+IF(LEFT(K186,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M186" t="n">
+        <x:f>IF(LEFT(A186,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187" ht="66" hidden="0" customHeight="1">
+      <x:c r="A187" s="63" t="str">
+        <x:v>Eliminada — requisitos técnicos</x:v>
+      </x:c>
+      <x:c r="B187" s="63" t="str">
+        <x:v>Cuattro Live &amp; Digital</x:v>
+      </x:c>
+      <x:c r="C187" s="63" t="str">
+        <x:v>Desenvolvedor(a) de Software Júnior | Full-Stack | Produtos Digitais</x:v>
+      </x:c>
+      <x:c r="D187" s="63" t="str">
+        <x:v>Desenvolvimento full stack e IA</x:v>
+      </x:c>
+      <x:c r="E187" s="63" t="str">
+        <x:v>São Paulo/SP; híbrido 3x/semana; PJ; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F187" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G187" s="63" t="str">
+        <x:v>Encerrada pelo filtro eliminatório do portal</x:v>
+      </x:c>
+      <x:c r="H187" s="63" t="str">
+        <x:v>Não reaplicar. Se quiser mirar vagas semelhantes, consolidar evidências de Node.js prático e NoSQL em projeto real antes de nova candidatura.</x:v>
+      </x:c>
+      <x:c r="I187" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J187" s="63" t="str">
+        <x:v>A Gupy eliminou a candidatura por respostas bloqueadas previamente para experiência prática em Node.js e NoSQL. Os campos estavam travados e não foram alterados; a apresentação foi atualizada de forma factual com Performance Lab antes da finalização.</x:v>
+      </x:c>
+      <x:c r="K187" s="63" t="str">
+        <x:v>Não — eliminada por requisitos obrigatórios 02/10</x:v>
+      </x:c>
+      <x:c r="L187" t="n">
+        <x:f>IF(LEFT(K187,3)="Sim",1,0)+IF(LEFT(K187,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M187" t="n">
+        <x:f>IF(LEFT(A187,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A188" s="63" t="str">
+        <x:v>Pendente — login/cadastro</x:v>
+      </x:c>
+      <x:c r="B188" s="63" t="str">
+        <x:v>Lyncas</x:v>
+      </x:c>
+      <x:c r="C188" s="63" t="str">
+        <x:v>Desenvolvedor Full Stack Júnior (Node.js e React)</x:v>
+      </x:c>
+      <x:c r="D188" s="63" t="str">
+        <x:v>Desenvolvimento full stack</x:v>
+      </x:c>
+      <x:c r="E188" s="63" t="str">
+        <x:v>São Paulo/SP; híbrido; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F188" s="63" t="str">
+        <x:v>https://www.netvagas.com.br/empresa/anuncios/a2167432/desenvolvedor-fullstack-junior-node-e-react-hibrido-sp-fln-joinville-ou-poa/?apply=2</x:v>
+      </x:c>
+      <x:c r="G188" s="63" t="str">
+        <x:v>Nenhuma avaliação acessível sem login</x:v>
+      </x:c>
+      <x:c r="H188" s="63" t="str">
+        <x:v>Efetuar login/cadastro no NetVagas/InHire, revisar o anúncio atual e personalizar com React, TypeScript, APIs, PostgreSQL, Git, Docker e Node.js em projetos práticos.</x:v>
+      </x:c>
+      <x:c r="I188" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J188" s="63" t="str">
+        <x:v>Vaga válida e compatível, mas o fluxo externo exige login/cadastro antes de redirecionar para a candidatura. Nenhuma senha foi criada ou presumida.</x:v>
+      </x:c>
+      <x:c r="K188" s="63" t="str">
+        <x:v>Não — login/cadastro externo pendente</x:v>
+      </x:c>
+      <x:c r="L188" t="n">
+        <x:f>IF(LEFT(K188,3)="Sim",1,0)+IF(LEFT(K188,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M188" t="n">
+        <x:f>IF(LEFT(A188,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A189" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B189" s="63" t="str">
+        <x:v>Suhai Seguradora</x:v>
+      </x:c>
+      <x:c r="C189" s="63" t="str">
+        <x:v>Analista de Dados Júnior</x:v>
+      </x:c>
+      <x:c r="D189" s="63" t="str">
+        <x:v>Dados e Analytics</x:v>
+      </x:c>
+      <x:c r="E189" s="63" t="str">
+        <x:v>São Paulo/SP; híbrido; efetivo; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F189" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G189" s="63" t="str">
+        <x:v>Mapeamento comportamental pode ocorrer depois — realizar pessoalmente</x:v>
+      </x:c>
+      <x:c r="H189" s="63" t="str">
+        <x:v>Acompanhar e-mail e portal. Estudar Power BI e Databricks; consolidar exemplos de SQL, Python, limpeza de dados, automação e Excel.</x:v>
+      </x:c>
+      <x:c r="I189" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J189" s="63" t="str">
+        <x:v>Candidatura finalizada na Gupy com apresentação personalizada para dados e Analytics. Respostas já bloqueadas pelo portal declaravam SQL e Python, não Power BI; não foram alteradas.</x:v>
+      </x:c>
+      <x:c r="K189" s="63" t="str">
+        <x:v>Sim — candidatura finalizada na Gupy 02/10</x:v>
+      </x:c>
+      <x:c r="L189" t="n">
+        <x:f>IF(LEFT(K189,3)="Sim",1,0)+IF(LEFT(K189,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M189" t="n">
+        <x:f>IF(LEFT(A189,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A190" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B190" s="63" t="str">
+        <x:v>JETSOFT</x:v>
+      </x:c>
+      <x:c r="C190" s="63" t="str">
+        <x:v>Desenvolvedor(a) Fullstack</x:v>
+      </x:c>
+      <x:c r="D190" s="63" t="str">
+        <x:v>Desenvolvimento full stack e IA</x:v>
+      </x:c>
+      <x:c r="E190" s="63" t="str">
+        <x:v>São Paulo/SP ou Vale do Paraíba/SP; híbrido; CLT; remuneração oficial a combinar</x:v>
+      </x:c>
+      <x:c r="F190" s="63" t="str">
+        <x:v>https://www.catho.com.br/vagas/desenvolvedora-fullstack/38135336/</x:v>
+      </x:c>
+      <x:c r="G190" s="63" t="str">
+        <x:v>Nenhuma avaliação declarada na candidatura</x:v>
+      </x:c>
+      <x:c r="H190" s="63" t="str">
+        <x:v>Acompanhar e-mail e Catho. Preparar exemplos de React, TypeScript, Python, APIs REST, SQL, Git, testes e integrações com IA.</x:v>
+      </x:c>
+      <x:c r="I190" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J190" s="63" t="str">
+        <x:v>Candidatura confirmada na Catho com a mensagem 'CV enviado!'. Foram respondidas de forma factual as perguntas sobre backend em Python, APIs REST, SQL, experiência profissional full stack e React/TypeScript.</x:v>
+      </x:c>
+      <x:c r="K190" s="63" t="str">
+        <x:v>Portal — CV enviado 02/10</x:v>
+      </x:c>
+      <x:c r="L190" t="n">
+        <x:f>IF(LEFT(K190,3)="Sim",1,0)+IF(LEFT(K190,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M190" t="n">
+        <x:f>IF(LEFT(A190,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A191" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B191" s="63" t="str">
+        <x:v>MEOSST Tecnologia Ltda.</x:v>
+      </x:c>
+      <x:c r="C191" s="63" t="str">
+        <x:v>Desenvolvedor Full Stack Pleno</x:v>
+      </x:c>
+      <x:c r="D191" s="63" t="str">
+        <x:v>Desenvolvimento full stack, integrações e IA</x:v>
+      </x:c>
+      <x:c r="E191" s="63" t="str">
+        <x:v>São Paulo/SP; PJ; 44 horas semanais; salário oficial R$ 3.500</x:v>
+      </x:c>
+      <x:c r="F191" s="63" t="str">
+        <x:v>https://www.catho.com.br/vagas/desenvolvedor-full-stack-pleno/37943370/</x:v>
+      </x:c>
+      <x:c r="G191" s="63" t="str">
+        <x:v>Nenhuma avaliação declarada na candidatura</x:v>
+      </x:c>
+      <x:c r="H191" s="63" t="str">
+        <x:v>Acompanhar e-mail e Catho. Preparar exemplos de frontend, backend, APIs, integrações, SQL, JSON, Git, automação e publicação de aplicações.</x:v>
+      </x:c>
+      <x:c r="I191" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J191" s="63" t="str">
+        <x:v>Candidatura confirmada na Catho com a mensagem 'CV enviado!'. Embora o título seja pleno, a descrição não exigia anos mínimos e disse que não era necessário dominar todas as tecnologias listadas.</x:v>
+      </x:c>
+      <x:c r="K191" s="63" t="str">
+        <x:v>Portal — CV enviado 02/10</x:v>
+      </x:c>
+      <x:c r="L191" t="n">
+        <x:f>IF(LEFT(K191,3)="Sim",1,0)+IF(LEFT(K191,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M191" t="n">
+        <x:f>IF(LEFT(A191,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192" ht="66" hidden="0" customHeight="1">
+      <x:c r="A192" s="63" t="str">
+        <x:v>Pendente — confirmar requisito de tempo</x:v>
+      </x:c>
+      <x:c r="B192" s="63" t="str">
+        <x:v>NOVVAX Tecnologia</x:v>
+      </x:c>
+      <x:c r="C192" s="63" t="str">
+        <x:v>Desenvolvedor Full Stack</x:v>
+      </x:c>
+      <x:c r="D192" s="63" t="str">
+        <x:v>Desenvolvimento full stack</x:v>
+      </x:c>
+      <x:c r="E192" s="63" t="str">
+        <x:v>São Paulo/SP; híbrido inicial 2 dias; PJ; salário oficial a partir de R$ 3.000</x:v>
+      </x:c>
+      <x:c r="F192" s="63" t="str">
+        <x:v>https://www.catho.com.br/vagas/desenvolvedor-full-stack/37858394/</x:v>
+      </x:c>
+      <x:c r="G192" s="63" t="str">
+        <x:v>Sem avaliação acessada; formulário pergunta sobre mínimo de 2 anos de atuação full stack</x:v>
+      </x:c>
+      <x:c r="H192" s="63" t="str">
+        <x:v>Confirmar a duração comprovável de experiência profissional full stack antes de responder. A vaga pede React, Python, PHP, PostgreSQL, MongoDB e Git; MongoDB também é gap atual.</x:v>
+      </x:c>
+      <x:c r="I192" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J192" s="63" t="str">
+        <x:v>Vaga revisada e não enviada: o formulário exige confirmação de pelo menos dois anos de atuação como desenvolvedor full stack. A informação disponível confirma experiência profissional, mas não estabelece esse período com segurança.</x:v>
+      </x:c>
+      <x:c r="K192" s="63" t="str">
+        <x:v>Não — requisito de tempo ainda sem confirmação</x:v>
+      </x:c>
+      <x:c r="L192" t="n">
+        <x:f>IF(LEFT(K192,3)="Sim",1,0)+IF(LEFT(K192,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M192" t="n">
+        <x:f>IF(LEFT(A192,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A193" s="63" t="str">
+        <x:v>Pendente — gaps obrigatórios</x:v>
+      </x:c>
+      <x:c r="B193" s="63" t="str">
+        <x:v>Interação - Soluções Inteligentes em Educação</x:v>
+      </x:c>
+      <x:c r="C193" s="63" t="str">
+        <x:v>Desenvolvedor(a) FullStack - Plataforma Web Gamificada</x:v>
+      </x:c>
+      <x:c r="D193" s="63" t="str">
+        <x:v>Desenvolvimento full stack e IA</x:v>
+      </x:c>
+      <x:c r="E193" s="63" t="str">
+        <x:v>Remoto; PJ temporário de 3 meses; 40 horas semanais; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F193" s="63" t="str">
+        <x:v>https://www.catho.com.br/vagas/desenvolvedora-fullstack-plataforma-web-gamificada/38407663/</x:v>
+      </x:c>
+      <x:c r="G193" s="63" t="str">
+        <x:v>Nenhuma avaliação acessada; candidatura não iniciada</x:v>
+      </x:c>
+      <x:c r="H193" s="63" t="str">
+        <x:v>Revisar somente após consolidar Node.js, Drizzle ORM, BullMQ/Redis e pnpm workspaces/monorepo. Não apresentar esses requisitos como experiência atual.</x:v>
+      </x:c>
+      <x:c r="I193" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J193" s="63" t="str">
+        <x:v>Vaga remota de alto interesse em IA, educação e gamificação, mas a descrição trata Node.js, Drizzle, BullMQ/Redis e monorepo como obrigatórios. Não enviada para evitar resposta imprecisa.</x:v>
+      </x:c>
+      <x:c r="K193" s="63" t="str">
+        <x:v>Não — gaps obrigatórios atuais</x:v>
+      </x:c>
+      <x:c r="L193" t="n">
+        <x:f>IF(LEFT(K193,3)="Sim",1,0)+IF(LEFT(K193,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M193" t="n">
+        <x:f>IF(LEFT(A193,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194">
+      <x:c r="A194" s="32" t="str">
         <x:v>Nota: ‘Sim’ significa recibo de e-mail localizado; ‘Portal’ significa confirmação/etapa verificada no portal. E-mails de inscrição iniciada não são tratados como candidatura enviada. Não há dados pessoais sensíveis nesta planilha.</x:v>
       </x:c>
-      <x:c r="B180" s="63"/>
-      <x:c r="C180" s="63"/>
-      <x:c r="D180" s="63"/>
-      <x:c r="E180" s="63"/>
-      <x:c r="F180" s="63"/>
-      <x:c r="G180" s="63"/>
-      <x:c r="H180" s="63"/>
-      <x:c r="I180" s="63"/>
-      <x:c r="J180" s="63"/>
-      <x:c r="K180" s="63"/>
+      <x:c r="B194" s="63"/>
+      <x:c r="C194" s="63"/>
+      <x:c r="D194" s="63"/>
+      <x:c r="E194" s="63"/>
+      <x:c r="F194" s="63"/>
+      <x:c r="G194" s="63"/>
+      <x:c r="H194" s="63"/>
+      <x:c r="I194" s="63"/>
+      <x:c r="J194" s="63"/>
+      <x:c r="K194" s="63"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A180:K180"/>
+    <x:mergeCell ref="A194:K194"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A10:A108">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Enviada"/>
@@ -8193,7 +8795,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59c410af76c540fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c3bc002fc164135"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10639,6 +11241,351 @@
         <x:v>Revalidar os anúncios um a um antes de candidatar; não duplicar as candidaturas já registradas.</x:v>
       </x:c>
     </x:row>
+    <x:row r="110">
+      <x:c r="A110" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B110" s="28" t="str">
+        <x:v>Gupy</x:v>
+      </x:c>
+      <x:c r="C110" s="28" t="str">
+        <x:v>Perfil global</x:v>
+      </x:c>
+      <x:c r="D110" s="28" t="str">
+        <x:v>Currículo e experiência atualizados</x:v>
+      </x:c>
+      <x:c r="E110" s="28" t="str">
+        <x:v>O perfil foi atualizado com a experiência profissional full stack na Performance Lab e a atuação autônoma via CNPJ em software, automação, PHP, frontend, scraping e integrações de APIs. A plataforma informa que alterações de currículo são refletidas nas candidaturas ativas.</x:v>
+      </x:c>
+      <x:c r="F110" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G110" s="30" t="str">
+        <x:v>Usar o perfil como fonte nas próximas vagas Gupy; revisar somente perguntas específicas de cada empresa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B111" s="28" t="str">
+        <x:v>InfoJobs</x:v>
+      </x:c>
+      <x:c r="C111" s="28" t="str">
+        <x:v>Perfil e pretensão</x:v>
+      </x:c>
+      <x:c r="D111" s="28" t="str">
+        <x:v>Resumo atualizado</x:v>
+      </x:c>
+      <x:c r="E111" s="28" t="str">
+        <x:v>O resumo foi atualizado de forma factual com Performance Lab, .NET/C#, React/TypeScript, PostgreSQL, APIs, automação e experiência autônoma. A pretensão mínima foi ajustada para R$ 3.000.</x:v>
+      </x:c>
+      <x:c r="F111" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G111" s="30" t="str">
+        <x:v>Acompanhar convites e usar o currículo mestre nas novas candidaturas.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B112" s="28" t="str">
+        <x:v>UOL EdTech / Gupy</x:v>
+      </x:c>
+      <x:c r="C112" s="28" t="str">
+        <x:v>Engenheiro de Software Jr. (Node.js / React.js)</x:v>
+      </x:c>
+      <x:c r="D112" s="28" t="str">
+        <x:v>Candidatura finalizada</x:v>
+      </x:c>
+      <x:c r="E112" s="28" t="str">
+        <x:v>O formulário foi concluído e a Gupy exibiu a confirmação de candidatura finalizada. A apresentação foi personalizada com experiência profissional full stack factual, sem exagerar experiência em Node.js.</x:v>
+      </x:c>
+      <x:c r="F112" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G112" s="30" t="str">
+        <x:v>Acompanhar e-mail e portal. Uma etapa futura de teste deve ser realizada pessoalmente pelo candidato, se for solicitada.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B113" s="28" t="str">
+        <x:v>Afya / Gupy</x:v>
+      </x:c>
+      <x:c r="C113" s="28" t="str">
+        <x:v>Analista de Dados Júnior</x:v>
+      </x:c>
+      <x:c r="D113" s="28" t="str">
+        <x:v>Candidatura validada</x:v>
+      </x:c>
+      <x:c r="E113" s="28" t="str">
+        <x:v>A candidatura já existente foi revisada e a Gupy exibiu confirmação de candidatura finalizada após a personalização factual voltada a SQL, Python, dados, automação e produto B2B.</x:v>
+      </x:c>
+      <x:c r="F113" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G113" s="30" t="str">
+        <x:v>Não duplicar a candidatura; acompanhar e-mail e portal.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B114" s="28" t="str">
+        <x:v>B2Finance / H&amp;CO</x:v>
+      </x:c>
+      <x:c r="C114" s="28" t="str">
+        <x:v>Full Stack Júnior</x:v>
+      </x:c>
+      <x:c r="D114" s="28" t="str">
+        <x:v>Duplicidade evitada</x:v>
+      </x:c>
+      <x:c r="E114" s="28" t="str">
+        <x:v>O portal InfoJobs/Pandapé reconheceu a participação já existente com o e-mail cadastrado. Nenhuma candidatura duplicada foi enviada.</x:v>
+      </x:c>
+      <x:c r="F114" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G114" s="30" t="str">
+        <x:v>Acompanhar e-mail e portal.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B115" s="28" t="str">
+        <x:v>Serasa Experian</x:v>
+      </x:c>
+      <x:c r="C115" s="28" t="str">
+        <x:v>Analista de Desenvolvimento de Software I — Backend Java</x:v>
+      </x:c>
+      <x:c r="D115" s="28" t="str">
+        <x:v>Formulário preparado</x:v>
+      </x:c>
+      <x:c r="E115" s="28" t="str">
+        <x:v>A vaga home office foi validada e o formulário SmartRecruiters foi aberto. O portal exige anexar o PDF local antes do envio; a mensagem de apresentação foi preparada de forma factual.</x:v>
+      </x:c>
+      <x:c r="F115" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G115" s="30" t="str">
+        <x:v>Anexar o currículo mestre e enviar somente após revisão final do formulário.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B116" s="28" t="str">
+        <x:v>Firefox / perfis</x:v>
+      </x:c>
+      <x:c r="C116" s="28" t="str">
+        <x:v>Sessão e perfil TOTVS RH</x:v>
+      </x:c>
+      <x:c r="D116" s="28" t="str">
+        <x:v>Conexão restabelecida e perfil corrigido</x:v>
+      </x:c>
+      <x:c r="E116" s="28" t="str">
+        <x:v>O Firefox voltou a responder. No perfil TOTVS RH, o cargo-alvo foi corrigido para Desenvolvedor Full Stack, o resumo profissional foi reescrito de forma técnica, a faixa desejada foi atualizada para R$ 3.000–R$ 7.000, o LinkedIn foi corrigido e Performance Lab foi adicionada como experiência profissional; a Falcon foi mantida como experiência comercial com término em nov/2025.</x:v>
+      </x:c>
+      <x:c r="F116" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G116" s="30" t="str">
+        <x:v>Anexo de currículo depende de upload local no portal; usar o PDF mestre atual quando o controle de upload estiver disponível.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B117" s="28" t="str">
+        <x:v>SoftExpert, Skeelo e Bullla</x:v>
+      </x:c>
+      <x:c r="C117" s="28" t="str">
+        <x:v>Três candidaturas técnicas</x:v>
+      </x:c>
+      <x:c r="D117" s="28" t="str">
+        <x:v>Candidaturas confirmadas</x:v>
+      </x:c>
+      <x:c r="E117" s="28" t="str">
+        <x:v>Foram confirmadas candidaturas para Full Stack Jr. remoto na SoftExpert, Backend Engineer I remoto na Skeelo e Analista de Dados Jr. híbrido na Bullla. As apresentações foram adaptadas ao cargo e mantiveram Performance Lab, NOW PRO e os gaps técnicos de forma honesta.</x:v>
+      </x:c>
+      <x:c r="F117" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G117" s="30" t="str">
+        <x:v>Acompanhar e-mail e portal. Qualquer avaliação comportamental, técnica ou entrevista deve ser realizada pessoalmente pelo candidato.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B118" s="28" t="str">
+        <x:v>Gupy</x:v>
+      </x:c>
+      <x:c r="C118" s="28" t="str">
+        <x:v>Viceri, ISA Saúde e Construmarket</x:v>
+      </x:c>
+      <x:c r="D118" s="28" t="str">
+        <x:v>Três candidaturas personalizadas finalizadas</x:v>
+      </x:c>
+      <x:c r="E118" s="28" t="str">
+        <x:v>Foram finalizadas candidaturas para Viceri Full Stack Jr. remoto, ISA Saúde Desenvolvedor Jr. híbrido em São Paulo e Construmarket Desenvolvedor Jr. remoto. Cada texto foi adaptado aos requisitos reais, destacando Performance Lab, .NET/C#, React/TypeScript, PostgreSQL, APIs, integrações e pontos de estudo sem inflar experiência.</x:v>
+      </x:c>
+      <x:c r="F118" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G118" s="30" t="str">
+        <x:v>Viceri e Construmarket podem encaminhar avaliação comportamental/lógica/técnica em fase futura; não iniciar avaliações sem o candidato presente.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B119" s="28" t="str">
+        <x:v>Gupy</x:v>
+      </x:c>
+      <x:c r="C119" s="28" t="str">
+        <x:v>Atento TI e Cuattro</x:v>
+      </x:c>
+      <x:c r="D119" s="28" t="str">
+        <x:v>Filtros técnicos identificados</x:v>
+      </x:c>
+      <x:c r="E119" s="28" t="str">
+        <x:v>As duas candidaturas foram finalizadas com respostas factuais. A Atento eliminou por SQL Server obrigatório; a Cuattro eliminou por Node.js prático e NoSQL. Na Cuattro, as respostas eliminatórias estavam previamente bloqueadas e não foram alteradas.</x:v>
+      </x:c>
+      <x:c r="F119" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G119" s="30" t="str">
+        <x:v>Usar os filtros como orientação de estudo e evitar reaplicação duplicada nas mesmas vagas.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B120" s="28" t="str">
+        <x:v>Gupy</x:v>
+      </x:c>
+      <x:c r="C120" s="28" t="str">
+        <x:v>Suhai Seguradora - Analista de Dados Júnior</x:v>
+      </x:c>
+      <x:c r="D120" s="28" t="str">
+        <x:v>Candidatura personalizada finalizada</x:v>
+      </x:c>
+      <x:c r="E120" s="28" t="str">
+        <x:v>Foi finalizada a candidatura híbrida em São Paulo para Analista de Dados Júnior. A apresentação destacou SQL, Python, PostgreSQL, automação, dados operacionais, Excel avançado e Performance Lab sem alegar domínio em Power BI ou Databricks.</x:v>
+      </x:c>
+      <x:c r="F120" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G120" s="30" t="str">
+        <x:v>Mapeamento comportamental futuro deve ser realizado pessoalmente pelo candidato.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B121" s="28" t="str">
+        <x:v>Catho</x:v>
+      </x:c>
+      <x:c r="C121" s="28" t="str">
+        <x:v>Perfil profissional</x:v>
+      </x:c>
+      <x:c r="D121" s="28" t="str">
+        <x:v>Perfil e experiências atualizados</x:v>
+      </x:c>
+      <x:c r="E121" s="28" t="str">
+        <x:v>O perfil foi alinhado ao currículo mestre: objetivo Desenvolvedor Full Stack, pretensão a partir de R$ 3.000, resumo com Performance Lab/KNOTEN e NOW PRO, competências técnicas atualizadas e duas experiências profissionais descritas com foco full stack.</x:v>
+      </x:c>
+      <x:c r="F121" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G121" s="30" t="str">
+        <x:v>O portal confirmou cada atualização. Não refazer testes de habilidade em nome do candidato.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B122" s="28" t="str">
+        <x:v>Catho</x:v>
+      </x:c>
+      <x:c r="C122" s="28" t="str">
+        <x:v>JETSOFT e MEOSST</x:v>
+      </x:c>
+      <x:c r="D122" s="28" t="str">
+        <x:v>Duas candidaturas confirmadas</x:v>
+      </x:c>
+      <x:c r="E122" s="28" t="str">
+        <x:v>Foram enviadas candidaturas para Desenvolvedor(a) Fullstack CLT híbrido na JETSOFT e Desenvolvedor Full Stack Pleno PJ na MEOSST. Ambas exibiram a confirmação 'CV enviado!'. A JETSOFT tem stack muito aderente; a MEOSST declara salário oficial de R$ 3.500 e aceita base de programação sem domínio de todas as tecnologias.</x:v>
+      </x:c>
+      <x:c r="F122" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G122" s="30" t="str">
+        <x:v>Acompanhar e-mail e Catho. Qualquer avaliação ou entrevista deve ser realizada pessoalmente pelo candidato.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B123" s="28" t="str">
+        <x:v>Catho</x:v>
+      </x:c>
+      <x:c r="C123" s="28" t="str">
+        <x:v>NOVVAX Tecnologia</x:v>
+      </x:c>
+      <x:c r="D123" s="28" t="str">
+        <x:v>Requisito de tempo pendente</x:v>
+      </x:c>
+      <x:c r="E123" s="28" t="str">
+        <x:v>A vaga híbrida PJ a partir de R$ 3.000 foi revisada. O formulário pergunta se o candidato atende ao mínimo de dois anos de atuação full stack; como esse tempo não foi confirmado nas informações disponíveis, a candidatura não foi enviada nem houve resposta inventada.</x:v>
+      </x:c>
+      <x:c r="F123" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G123" s="30" t="str">
+        <x:v>Confirmar a duração comprovável de experiência full stack antes de retomar o envio.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B124" s="28" t="str">
+        <x:v>Catho</x:v>
+      </x:c>
+      <x:c r="C124" s="28" t="str">
+        <x:v>Interação - Soluções Inteligentes em Educação</x:v>
+      </x:c>
+      <x:c r="D124" s="28" t="str">
+        <x:v>Vaga remota revisada; gaps obrigatórios registrados</x:v>
+      </x:c>
+      <x:c r="E124" s="28" t="str">
+        <x:v>A vaga temporária remota de plataforma web gamificada foi avaliada como interessante para IA aplicada, porém exige Node.js, Drizzle ORM, BullMQ/Redis e pnpm workspaces/monorepo como requisitos obrigatórios. A candidatura não foi enviada e nenhum requisito foi afirmado sem evidência.</x:v>
+      </x:c>
+      <x:c r="F124" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G124" s="30" t="str">
+        <x:v>Retomar apenas após ganhar prática verificável nessas ferramentas ou se a empresa flexibilizar os requisitos.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F6:F59">
     <x:cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="Concluído"/>
@@ -10650,7 +11597,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd37e52654137471b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R336fa3f484854196"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Registra Minsait e atualiza acompanhamento publico
</commit_message>
<xml_diff>
--- a/planilhas/Controle_Candidaturas_Fintech_Guilherme_PUBLICO.xlsx
+++ b/planilhas/Controle_Candidaturas_Fintech_Guilherme_PUBLICO.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidaturas" sheetId="1" r:id="Rf3f3cbbff1874fc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log de auditoria" sheetId="2" r:id="R6f36761ee7774604"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidaturas" sheetId="1" r:id="R730e6fbc231542cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log de auditoria" sheetId="2" r:id="R43ccba5771694894"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -503,7 +503,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CandidaturasTable" displayName="CandidaturasTable" ref="A9:K193" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CandidaturasTable" displayName="CandidaturasTable" ref="A9:K196" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Status"/>
     <x:tableColumn id="2" name="Empresa"/>
@@ -793,24 +793,24 @@
         <x:v>Candidaturas confirmadas</x:v>
       </x:c>
       <x:c r="B7" s="9" t="n">
-        <x:f>SUM(L10:L193)</x:f>
-        <x:v>92</x:v>
+        <x:f>SUM(L10:L196)</x:f>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="C7" s="8"/>
       <x:c r="D7" s="8" t="str">
         <x:v>Itens em controle</x:v>
       </x:c>
       <x:c r="E7" s="9" t="n">
-        <x:f>COUNTA(A10:A193)</x:f>
-        <x:v>184</x:v>
+        <x:f>COUNTA(A10:A196)</x:f>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="F7" s="8"/>
       <x:c r="G7" s="8" t="str">
         <x:v>Pendentes</x:v>
       </x:c>
       <x:c r="H7" s="9" t="n">
-        <x:f>SUM(M10:M193)</x:f>
-        <x:v>82</x:v>
+        <x:f>SUM(M10:M196)</x:f>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
@@ -7986,9 +7986,9 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="176" ht="52.79999923706055" hidden="0" customHeight="1">
+    <x:row r="176" ht="66" hidden="0" customHeight="1">
       <x:c r="A176" s="63" t="str">
-        <x:v>Pendente — verificar duplicidade</x:v>
+        <x:v>Enviada</x:v>
       </x:c>
       <x:c r="B176" s="63" t="str">
         <x:v>SCS Saneamento</x:v>
@@ -8006,27 +8006,27 @@
         <x:v>https://scs-saneamento.pandape.infojobs.com.br/Detail/3683559</x:v>
       </x:c>
       <x:c r="G176" s="63" t="str">
-        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+        <x:v>Nenhuma avaliação declarada no momento; acompanhar portal e e-mail</x:v>
       </x:c>
       <x:c r="H176" s="63" t="str">
-        <x:v>Checar se existe candidatura anterior antes de iniciar. Se não houver, personalizar com React, Node, PostgreSQL/MySQL, APIs REST e testes; Kotlin é ponto de estudo.</x:v>
+        <x:v>Acompanhar portal e e-mail. Preparar exemplos de React, APIs REST, PostgreSQL/MySQL, Git, testes, integração de sistemas e documentação; Kotlin segue como ponto de estudo.</x:v>
       </x:c>
       <x:c r="I176" s="63" t="str">
         <x:v>02/10/2026</x:v>
       </x:c>
       <x:c r="J176" s="63" t="str">
-        <x:v>Triagem de São Paulo/Grande SP: vaga júnior de alta aderência e salário divulgado. Foi marcada para revisar duplicidade porque há registro histórico de possível candidatura semelhante fora do link atual.</x:v>
+        <x:v>O portal Pandapé confirmou que o e-mail cadastrado já foi utilizado nesta vaga e que o candidato já participa do processo seletivo. A descrição exige React, Kotlin, Node.js, APIs REST, PostgreSQL/MySQL, Git e testes; Kotlin é o principal ponto de desenvolvimento atual.</x:v>
       </x:c>
       <x:c r="K176" s="63" t="str">
-        <x:v>Não — candidatura ainda não iniciada</x:v>
+        <x:v>Portal — participação já existente confirmada em 02/10</x:v>
       </x:c>
       <x:c r="L176" t="n">
         <x:f>IF(LEFT(K176,3)="Sim",1,0)+IF(LEFT(K176,6)="Portal",1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M176" t="n">
         <x:f>IF(LEFT(A176,8)="Pendente",1,0)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="177" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -8760,24 +8760,153 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="194">
-      <x:c r="A194" s="32" t="str">
+    <x:row r="194" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A194" s="63" t="str">
+        <x:v>Pendente — requisitos obrigatórios</x:v>
+      </x:c>
+      <x:c r="B194" s="63" t="str">
+        <x:v>Neohype Digital</x:v>
+      </x:c>
+      <x:c r="C194" s="63" t="str">
+        <x:v>Desenvolvedor Full Stack (C# | .NET)</x:v>
+      </x:c>
+      <x:c r="D194" s="63" t="str">
+        <x:v>Desenvolvimento full stack</x:v>
+      </x:c>
+      <x:c r="E194" s="63" t="str">
+        <x:v>São Paulo/SP; híbrido; efetivo; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F194" s="63" t="str">
+        <x:v>Acessar na plataforma (link privado removido)</x:v>
+      </x:c>
+      <x:c r="G194" s="63" t="str">
+        <x:v>Nenhuma avaliação iniciada; formulário ainda não enviado</x:v>
+      </x:c>
+      <x:c r="H194" s="63" t="str">
+        <x:v>Não enviar sem evidência de uso profissional nos períodos exigidos. O formulário só oferece 1–2, 3–4 ou mais de 5 anos para C#/.NET, React/Angular, SQL Server e RabbitMQ/Hangfire; não há opção para ausência ou período inferior a um ano.</x:v>
+      </x:c>
+      <x:c r="I194" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J194" s="63" t="str">
+        <x:v>A vaga é híbrida e tem aderência em .NET, React, PostgreSQL, APIs, Git, testes, Docker e cloud, mas trata SQL Server, RabbitMQ e Hangfire como experiência obrigatória. O formulário também não permite declarar experiência inferior a um ano, portanto a candidatura não foi enviada nem recebeu resposta imprecisa.</x:v>
+      </x:c>
+      <x:c r="K194" s="63" t="str">
+        <x:v>Não — requisitos obrigatórios sem resposta factual disponível</x:v>
+      </x:c>
+      <x:c r="L194" t="n">
+        <x:f>IF(LEFT(K194,3)="Sim",1,0)+IF(LEFT(K194,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M194" t="n">
+        <x:f>IF(LEFT(A194,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A195" s="63" t="str">
+        <x:v>Encerrada — inscrições fechadas</x:v>
+      </x:c>
+      <x:c r="B195" s="63" t="str">
+        <x:v>Tokio Marine</x:v>
+      </x:c>
+      <x:c r="C195" s="63" t="str">
+        <x:v>Analista de Dados Júnior (Precificação e Inteligência de Negócios)</x:v>
+      </x:c>
+      <x:c r="D195" s="63" t="str">
+        <x:v>Dados, ETL e analytics</x:v>
+      </x:c>
+      <x:c r="E195" s="63" t="str">
+        <x:v>São Paulo/SP; híbrido; efetivo; remuneração não divulgada</x:v>
+      </x:c>
+      <x:c r="F195" s="63" t="str">
+        <x:v>https://tokiomarine.gupy.io/jobs/12024259</x:v>
+      </x:c>
+      <x:c r="G195" s="63" t="str">
+        <x:v>Não iniciada; etapas futuras listavam fit cultural e testes complementares</x:v>
+      </x:c>
+      <x:c r="H195" s="63" t="str">
+        <x:v>Não reaplicar nesta publicação. Monitorar novas vagas júnior de dados/analytics da Tokio Marine.</x:v>
+      </x:c>
+      <x:c r="I195" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J195" s="63" t="str">
+        <x:v>O anúncio foi revalidado no portal oficial e as inscrições já estavam encerradas. A descrição era aderente em SQL, Python, ETL, modelagem e automação; Power BI, Airflow e domínio de seguros eram pontos de desenvolvimento.</x:v>
+      </x:c>
+      <x:c r="K195" s="63" t="str">
+        <x:v>Não aplicável — vaga encerrada na conferência de 02/10</x:v>
+      </x:c>
+      <x:c r="L195" t="n">
+        <x:f>IF(LEFT(K195,3)="Sim",1,0)+IF(LEFT(K195,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M195" t="n">
+        <x:f>IF(LEFT(A195,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A196" s="63" t="str">
+        <x:v>Pendente — acesso ao anúncio</x:v>
+      </x:c>
+      <x:c r="B196" s="63" t="str">
+        <x:v>MOST Specialist Technologies</x:v>
+      </x:c>
+      <x:c r="C196" s="63" t="str">
+        <x:v>Full Stack Developer (Python) — Hiperautomação</x:v>
+      </x:c>
+      <x:c r="D196" s="63" t="str">
+        <x:v>Python, automação e desenvolvimento full stack</x:v>
+      </x:c>
+      <x:c r="E196" s="63" t="str">
+        <x:v>Remoto; estágio 6 horas/dia; remuneração divulgada no Indeed: R$ 4.000/mês</x:v>
+      </x:c>
+      <x:c r="F196" s="63" t="str">
+        <x:v>https://br.indeed.com/viewjob?jk=8056a8178617f40a</x:v>
+      </x:c>
+      <x:c r="G196" s="63" t="str">
+        <x:v>Desafio técnico por e-mail é mencionado — realizar pessoalmente se a candidatura avançar</x:v>
+      </x:c>
+      <x:c r="H196" s="63" t="str">
+        <x:v>Revalidar por rota oficial ou após verificação humana do Indeed. Destacar Python, APIs, Docker, automação, dados, Git, Linux, TypeScript e CI/CD/AWS como experiência ou conhecimento factual.</x:v>
+      </x:c>
+      <x:c r="I196" s="63" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="J196" s="63" t="str">
+        <x:v>Pesquisa identificou alta aderência técnica e remuneração acima do piso. O anúncio menciona desafio técnico posterior por e-mail; não foi iniciado. A rota do Indeed ficou protegida por verificação nesta sessão.</x:v>
+      </x:c>
+      <x:c r="K196" s="63" t="str">
+        <x:v>Não — acesso ao anúncio bloqueado por verificação do Indeed</x:v>
+      </x:c>
+      <x:c r="L196" t="n">
+        <x:f>IF(LEFT(K196,3)="Sim",1,0)+IF(LEFT(K196,6)="Portal",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M196" t="n">
+        <x:f>IF(LEFT(A196,8)="Pendente",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197">
+      <x:c r="A197" s="32" t="str">
         <x:v>Nota: ‘Sim’ significa recibo de e-mail localizado; ‘Portal’ significa confirmação/etapa verificada no portal. E-mails de inscrição iniciada não são tratados como candidatura enviada. Não há dados pessoais sensíveis nesta planilha.</x:v>
       </x:c>
-      <x:c r="B194" s="63"/>
-      <x:c r="C194" s="63"/>
-      <x:c r="D194" s="63"/>
-      <x:c r="E194" s="63"/>
-      <x:c r="F194" s="63"/>
-      <x:c r="G194" s="63"/>
-      <x:c r="H194" s="63"/>
-      <x:c r="I194" s="63"/>
-      <x:c r="J194" s="63"/>
-      <x:c r="K194" s="63"/>
+      <x:c r="B197" s="63"/>
+      <x:c r="C197" s="63"/>
+      <x:c r="D197" s="63"/>
+      <x:c r="E197" s="63"/>
+      <x:c r="F197" s="63"/>
+      <x:c r="G197" s="63"/>
+      <x:c r="H197" s="63"/>
+      <x:c r="I197" s="63"/>
+      <x:c r="J197" s="63"/>
+      <x:c r="K197" s="63"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A194:K194"/>
+    <x:mergeCell ref="A197:K197"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A10:A108">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Enviada"/>
@@ -8795,7 +8924,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c3bc002fc164135"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f54b5a672774490"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11499,22 +11628,22 @@
         <x:v>02/10/2026</x:v>
       </x:c>
       <x:c r="B121" s="28" t="str">
-        <x:v>Catho</x:v>
+        <x:v>Gupy</x:v>
       </x:c>
       <x:c r="C121" s="28" t="str">
-        <x:v>Perfil profissional</x:v>
+        <x:v>Minsait - Analista de Dados Jr - Osasco/SP</x:v>
       </x:c>
       <x:c r="D121" s="28" t="str">
-        <x:v>Perfil e experiências atualizados</x:v>
+        <x:v>Candidatura personalizada finalizada</x:v>
       </x:c>
       <x:c r="E121" s="28" t="str">
-        <x:v>O perfil foi alinhado ao currículo mestre: objetivo Desenvolvedor Full Stack, pretensão a partir de R$ 3.000, resumo com Performance Lab/KNOTEN e NOW PRO, competências técnicas atualizadas e duas experiências profissionais descritas com foco full stack.</x:v>
+        <x:v>Foi concluída a candidatura CLT híbrida para dados, automação e meios de pagamento em Osasco. A apresentação conectou o trabalho full stack na Performance Lab/KNOTEN a Python, SQL, PostgreSQL, APIs, automação, testes e análise de dados, deixando R, SAS e contexto bancário como pontos de aprofundamento. A empresa informa que uma entrevista técnica futura será gravada; nenhum teste ou entrevista foi iniciado.</x:v>
       </x:c>
       <x:c r="F121" s="29" t="str">
         <x:v>Concluído</x:v>
       </x:c>
       <x:c r="G121" s="30" t="str">
-        <x:v>O portal confirmou cada atualização. Não refazer testes de habilidade em nome do candidato.</x:v>
+        <x:v>Acompanhar e-mail e portal. Se houver entrevista técnica gravada, ela deve ser realizada pessoalmente pelo candidato.</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
@@ -11525,19 +11654,19 @@
         <x:v>Catho</x:v>
       </x:c>
       <x:c r="C122" s="28" t="str">
-        <x:v>JETSOFT e MEOSST</x:v>
+        <x:v>Perfil profissional</x:v>
       </x:c>
       <x:c r="D122" s="28" t="str">
-        <x:v>Duas candidaturas confirmadas</x:v>
+        <x:v>Perfil e experiências atualizados</x:v>
       </x:c>
       <x:c r="E122" s="28" t="str">
-        <x:v>Foram enviadas candidaturas para Desenvolvedor(a) Fullstack CLT híbrido na JETSOFT e Desenvolvedor Full Stack Pleno PJ na MEOSST. Ambas exibiram a confirmação 'CV enviado!'. A JETSOFT tem stack muito aderente; a MEOSST declara salário oficial de R$ 3.500 e aceita base de programação sem domínio de todas as tecnologias.</x:v>
+        <x:v>O perfil foi alinhado ao currículo mestre: objetivo Desenvolvedor Full Stack, pretensão a partir de R$ 3.000, resumo com Performance Lab/KNOTEN e NOW PRO, competências técnicas atualizadas e duas experiências profissionais descritas com foco full stack.</x:v>
       </x:c>
       <x:c r="F122" s="29" t="str">
         <x:v>Concluído</x:v>
       </x:c>
       <x:c r="G122" s="30" t="str">
-        <x:v>Acompanhar e-mail e Catho. Qualquer avaliação ou entrevista deve ser realizada pessoalmente pelo candidato.</x:v>
+        <x:v>O portal confirmou cada atualização. Não refazer testes de habilidade em nome do candidato.</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
@@ -11548,19 +11677,19 @@
         <x:v>Catho</x:v>
       </x:c>
       <x:c r="C123" s="28" t="str">
-        <x:v>NOVVAX Tecnologia</x:v>
+        <x:v>JETSOFT e MEOSST</x:v>
       </x:c>
       <x:c r="D123" s="28" t="str">
-        <x:v>Requisito de tempo pendente</x:v>
+        <x:v>Duas candidaturas confirmadas</x:v>
       </x:c>
       <x:c r="E123" s="28" t="str">
-        <x:v>A vaga híbrida PJ a partir de R$ 3.000 foi revisada. O formulário pergunta se o candidato atende ao mínimo de dois anos de atuação full stack; como esse tempo não foi confirmado nas informações disponíveis, a candidatura não foi enviada nem houve resposta inventada.</x:v>
+        <x:v>Foram enviadas candidaturas para Desenvolvedor(a) Fullstack CLT híbrido na JETSOFT e Desenvolvedor Full Stack Pleno PJ na MEOSST. Ambas exibiram a confirmação 'CV enviado!'. A JETSOFT tem stack muito aderente; a MEOSST declara salário oficial de R$ 3.500 e aceita base de programação sem domínio de todas as tecnologias.</x:v>
       </x:c>
       <x:c r="F123" s="29" t="str">
-        <x:v>Pendente</x:v>
+        <x:v>Concluído</x:v>
       </x:c>
       <x:c r="G123" s="30" t="str">
-        <x:v>Confirmar a duração comprovável de experiência full stack antes de retomar o envio.</x:v>
+        <x:v>Acompanhar e-mail e Catho. Qualquer avaliação ou entrevista deve ser realizada pessoalmente pelo candidato.</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
@@ -11571,19 +11700,134 @@
         <x:v>Catho</x:v>
       </x:c>
       <x:c r="C124" s="28" t="str">
-        <x:v>Interação - Soluções Inteligentes em Educação</x:v>
+        <x:v>NOVVAX Tecnologia</x:v>
       </x:c>
       <x:c r="D124" s="28" t="str">
-        <x:v>Vaga remota revisada; gaps obrigatórios registrados</x:v>
+        <x:v>Requisito de tempo pendente</x:v>
       </x:c>
       <x:c r="E124" s="28" t="str">
-        <x:v>A vaga temporária remota de plataforma web gamificada foi avaliada como interessante para IA aplicada, porém exige Node.js, Drizzle ORM, BullMQ/Redis e pnpm workspaces/monorepo como requisitos obrigatórios. A candidatura não foi enviada e nenhum requisito foi afirmado sem evidência.</x:v>
+        <x:v>A vaga híbrida PJ a partir de R$ 3.000 foi revisada. O formulário pergunta se o candidato atende ao mínimo de dois anos de atuação full stack; como esse tempo não foi confirmado nas informações disponíveis, a candidatura não foi enviada nem houve resposta inventada.</x:v>
       </x:c>
       <x:c r="F124" s="29" t="str">
         <x:v>Pendente</x:v>
       </x:c>
       <x:c r="G124" s="30" t="str">
+        <x:v>Confirmar a duração comprovável de experiência full stack antes de retomar o envio.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B125" s="28" t="str">
+        <x:v>Catho</x:v>
+      </x:c>
+      <x:c r="C125" s="28" t="str">
+        <x:v>Interação - Soluções Inteligentes em Educação</x:v>
+      </x:c>
+      <x:c r="D125" s="28" t="str">
+        <x:v>Vaga remota revisada; gaps obrigatórios registrados</x:v>
+      </x:c>
+      <x:c r="E125" s="28" t="str">
+        <x:v>A vaga temporária remota de plataforma web gamificada foi avaliada como interessante para IA aplicada, porém exige Node.js, Drizzle ORM, BullMQ/Redis e pnpm workspaces/monorepo como requisitos obrigatórios. A candidatura não foi enviada e nenhum requisito foi afirmado sem evidência.</x:v>
+      </x:c>
+      <x:c r="F125" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G125" s="30" t="str">
         <x:v>Retomar apenas após ganhar prática verificável nessas ferramentas ou se a empresa flexibilizar os requisitos.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B126" s="28" t="str">
+        <x:v>Gupy</x:v>
+      </x:c>
+      <x:c r="C126" s="28" t="str">
+        <x:v>Neohype Digital - Desenvolvedor Full Stack</x:v>
+      </x:c>
+      <x:c r="D126" s="28" t="str">
+        <x:v>Formulário interrompido por requisitos obrigatórios</x:v>
+      </x:c>
+      <x:c r="E126" s="28" t="str">
+        <x:v>A vaga híbrida foi revisada por ter boa aderência em .NET, React, PostgreSQL, APIs, testes e cloud. Porém, as respostas obrigatórias exigem no mínimo um a dois anos de uso profissional em C#/.NET, React/Angular, SQL Server e RabbitMQ/Hangfire, sem opção para experiência inferior ou inexistente. Nenhuma informação foi inventada e a candidatura não foi enviada.</x:v>
+      </x:c>
+      <x:c r="F126" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G126" s="30" t="str">
+        <x:v>Retomar somente se houver experiência verificável nos requisitos ou se a empresa disponibilizar alternativa de resposta.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B127" s="28" t="str">
+        <x:v>Gupy</x:v>
+      </x:c>
+      <x:c r="C127" s="28" t="str">
+        <x:v>Tokio Marine - Analista de Dados Júnior</x:v>
+      </x:c>
+      <x:c r="D127" s="28" t="str">
+        <x:v>Vaga revalidada como encerrada</x:v>
+      </x:c>
+      <x:c r="E127" s="28" t="str">
+        <x:v>O anúncio oficial de São Paulo híbrido foi aberto para conferência e informava candidaturas encerradas. Nenhuma candidatura foi iniciada. A vaga foi mantida no histórico apenas para registrar a revalidação e orientar monitoramento de oportunidades semelhantes.</x:v>
+      </x:c>
+      <x:c r="F127" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G127" s="30" t="str">
+        <x:v>Monitorar novas publicações de dados, ETL e analytics da Tokio Marine.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B128" s="28" t="str">
+        <x:v>Pandapé / InfoJobs</x:v>
+      </x:c>
+      <x:c r="C128" s="28" t="str">
+        <x:v>SCS Saneamento - Desenvolvedor Full Stack Júnior</x:v>
+      </x:c>
+      <x:c r="D128" s="28" t="str">
+        <x:v>Duplicidade confirmada</x:v>
+      </x:c>
+      <x:c r="E128" s="28" t="str">
+        <x:v>A vaga presencial PJ da Berrini foi revalidada, com salário divulgado de R$ 6.000 a R$ 6.500. Ao informar o e-mail, o Pandapé confirmou que o candidato já participa do processo seletivo; nenhuma candidatura duplicada foi enviada.</x:v>
+      </x:c>
+      <x:c r="F128" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G128" s="30" t="str">
+        <x:v>Acompanhar atualizações no e-mail. Kotlin é o principal ponto técnico a aprofundar para a vaga.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B129" s="28" t="str">
+        <x:v>Indeed</x:v>
+      </x:c>
+      <x:c r="C129" s="28" t="str">
+        <x:v>Black Lion, MOST Specialist Technologies e Juriscont / New Legal</x:v>
+      </x:c>
+      <x:c r="D129" s="28" t="str">
+        <x:v>Três oportunidades com piso salarial revalidado por pesquisa</x:v>
+      </x:c>
+      <x:c r="E129" s="28" t="str">
+        <x:v>Foram priorizadas uma vaga fintech híbrida de full stack júnior por R$ 3.000, uma oportunidade remota de hiperautomação/Python por R$ 4.000 e uma vaga CLT de full stack na Berrini por R$ 4.000 a R$ 5.500. A abertura pelo Indeed nesta sessão levou à tela de verificação Cloudflare; nenhuma automação de proteção foi tentada e nenhuma candidatura foi enviada.</x:v>
+      </x:c>
+      <x:c r="F129" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G129" s="30" t="str">
+        <x:v>Retomar via rota oficial, alertas de e-mail ou acesso humano ao Indeed; qualquer desafio técnico posterior deve ser feito pessoalmente pelo candidato.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -11597,7 +11841,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R336fa3f484854196"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref95d265de0c44ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza pendencias de candidatura no controle publico
</commit_message>
<xml_diff>
--- a/planilhas/Controle_Candidaturas_Fintech_Guilherme_PUBLICO.xlsx
+++ b/planilhas/Controle_Candidaturas_Fintech_Guilherme_PUBLICO.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidaturas" sheetId="1" r:id="R730e6fbc231542cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log de auditoria" sheetId="2" r:id="R43ccba5771694894"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidaturas" sheetId="1" r:id="Reedbf855ba47442c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log de auditoria" sheetId="2" r:id="Rf5bb673d66db457a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8029,9 +8029,9 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="177" ht="52.79999923706055" hidden="0" customHeight="1">
+    <x:row r="177" ht="66" hidden="0" customHeight="1">
       <x:c r="A177" s="63" t="str">
-        <x:v>Pendente — revalidar e candidatar</x:v>
+        <x:v>Pendente — formulário e upload</x:v>
       </x:c>
       <x:c r="B177" s="63" t="str">
         <x:v>Datum</x:v>
@@ -8049,19 +8049,19 @@
         <x:v>https://datum.jobs.recrut.ai/gender-predict/job/XV0CV0</x:v>
       </x:c>
       <x:c r="G177" s="63" t="str">
-        <x:v>Não informado; validar qualquer nova etapa antes de iniciar</x:v>
+        <x:v>Nenhuma avaliação acessada; formulário não enviado</x:v>
       </x:c>
       <x:c r="H177" s="63" t="str">
-        <x:v>Revalidar anúncio e personalizar com base em backend, APIs, SQL, Docker e capacidade de estudar Java; Java é diferencial/desenvolvimento a fortalecer.</x:v>
+        <x:v>Anexar o currículo mestre atualizado e preencher o CEP real antes do envio. Depois, personalizar com Java, APIs, SQL, Docker, integração de sistemas, testes e aprendizagem contínua.</x:v>
       </x:c>
       <x:c r="I177" s="63" t="str">
         <x:v>02/10/2026</x:v>
       </x:c>
       <x:c r="J177" s="63" t="str">
-        <x:v>Triagem de São Paulo/Grande SP: programa de início de carreira; experiência de um ano com Java aparece como desejável, não como requisito eliminatório. Nenhuma candidatura foi iniciada.</x:v>
+        <x:v>Anúncio oficial revalidado como ativo e muito compatível com início de carreira: conhecimento em Java é obrigatório e um ano profissional é apenas desejável. O formulário exige dados cadastrais, CEP e upload local obrigatório do currículo; não foi enviado sem esses itens.</x:v>
       </x:c>
       <x:c r="K177" s="63" t="str">
-        <x:v>Não — candidatura ainda não iniciada</x:v>
+        <x:v>Não — upload de currículo e CEP obrigatórios pendentes</x:v>
       </x:c>
       <x:c r="L177" t="n">
         <x:f>IF(LEFT(K177,3)="Sim",1,0)+IF(LEFT(K177,6)="Portal",1,0)</x:f>
@@ -8924,7 +8924,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f54b5a672774490"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f88cbebc9ed410a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11830,6 +11830,29 @@
         <x:v>Retomar via rota oficial, alertas de e-mail ou acesso humano ao Indeed; qualquer desafio técnico posterior deve ser feito pessoalmente pelo candidato.</x:v>
       </x:c>
     </x:row>
+    <x:row r="130">
+      <x:c r="A130" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B130" s="28" t="str">
+        <x:v>Recrut.AI / Datum</x:v>
+      </x:c>
+      <x:c r="C130" s="28" t="str">
+        <x:v>Pessoa Desenvolvedora Java Júnior (NextGen)</x:v>
+      </x:c>
+      <x:c r="D130" s="28" t="str">
+        <x:v>Vaga revalidada; formulário preparado</x:v>
+      </x:c>
+      <x:c r="E130" s="28" t="str">
+        <x:v>A vaga híbrida na Zona Sul está ativa e aceita pessoa em início de carreira com conhecimento em Java; experiência de um ano é desejável, não obrigatória. O formulário exige currículo por upload local e CEP real, por isso não foi enviado sem esses itens.</x:v>
+      </x:c>
+      <x:c r="F130" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G130" s="30" t="str">
+        <x:v>Anexar o currículo mestre e preencher o CEP no formulário aberto antes de enviar.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F6:F59">
     <x:cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="Concluído"/>
@@ -11841,7 +11864,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref95d265de0c44ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re722279ff8ed4430"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Registra pendencia factual da MOST
</commit_message>
<xml_diff>
--- a/planilhas/Controle_Candidaturas_Fintech_Guilherme_PUBLICO.xlsx
+++ b/planilhas/Controle_Candidaturas_Fintech_Guilherme_PUBLICO.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidaturas" sheetId="1" r:id="Reedbf855ba47442c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log de auditoria" sheetId="2" r:id="Rf5bb673d66db457a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidaturas" sheetId="1" r:id="R02707cd6597f4c15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log de auditoria" sheetId="2" r:id="Rcf8db25bccd4489f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8846,9 +8846,9 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="196" ht="52.79999923706055" hidden="0" customHeight="1">
+    <x:row r="196" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A196" s="63" t="str">
-        <x:v>Pendente — acesso ao anúncio</x:v>
+        <x:v>Pendente — formulário e requisitos</x:v>
       </x:c>
       <x:c r="B196" s="63" t="str">
         <x:v>MOST Specialist Technologies</x:v>
@@ -8866,19 +8866,19 @@
         <x:v>https://br.indeed.com/viewjob?jk=8056a8178617f40a</x:v>
       </x:c>
       <x:c r="G196" s="63" t="str">
-        <x:v>Desafio técnico por e-mail é mencionado — realizar pessoalmente se a candidatura avançar</x:v>
+        <x:v>Desafio técnico posterior e avaliação psicológica são previstos — realizar pessoalmente se a candidatura avançar</x:v>
       </x:c>
       <x:c r="H196" s="63" t="str">
-        <x:v>Revalidar por rota oficial ou após verificação humana do Indeed. Destacar Python, APIs, Docker, automação, dados, Git, Linux, TypeScript e CI/CD/AWS como experiência ou conhecimento factual.</x:v>
+        <x:v>Formulário oficial encontrado e revisado. Só retomar se houver como anexar o currículo e preencher a matriz técnica com evidência factual; ela exige nível para tecnologias como Django, multithread e MongoDB sem opção de 'sem experiência'.</x:v>
       </x:c>
       <x:c r="I196" s="63" t="str">
         <x:v>02/10/2026</x:v>
       </x:c>
       <x:c r="J196" s="63" t="str">
-        <x:v>Pesquisa identificou alta aderência técnica e remuneração acima do piso. O anúncio menciona desafio técnico posterior por e-mail; não foi iniciado. A rota do Indeed ficou protegida por verificação nesta sessão.</x:v>
+        <x:v>O site oficial confirma trabalho remoto e estágio de 6 horas com bolsa de R$ 4.000. O formulário oficial requer upload do currículo e grade obrigatória de tecnologias; ele não oferece resposta para ausência de experiência em Django, multithread e MongoDB. Não foi enviado para evitar declaração imprecisa.</x:v>
       </x:c>
       <x:c r="K196" s="63" t="str">
-        <x:v>Não — acesso ao anúncio bloqueado por verificação do Indeed</x:v>
+        <x:v>Não — formulário exige upload e níveis sem alternativa factual para todos os itens</x:v>
       </x:c>
       <x:c r="L196" t="n">
         <x:f>IF(LEFT(K196,3)="Sim",1,0)+IF(LEFT(K196,6)="Portal",1,0)</x:f>
@@ -8924,7 +8924,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f88cbebc9ed410a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda9b7dfea1e449a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11853,6 +11853,29 @@
         <x:v>Anexar o currículo mestre e preencher o CEP no formulário aberto antes de enviar.</x:v>
       </x:c>
     </x:row>
+    <x:row r="131">
+      <x:c r="A131" s="61" t="str">
+        <x:v>02/10/2026</x:v>
+      </x:c>
+      <x:c r="B131" s="28" t="str">
+        <x:v>MOST Specialist Technologies</x:v>
+      </x:c>
+      <x:c r="C131" s="28" t="str">
+        <x:v>Full Stack Developer (Python) - Hiperautomação</x:v>
+      </x:c>
+      <x:c r="D131" s="28" t="str">
+        <x:v>Formulário oficial revisado</x:v>
+      </x:c>
+      <x:c r="E131" s="28" t="str">
+        <x:v>A rota oficial confirmou home office e estágio de seis horas com bolsa de R$ 4.000. O formulário exige upload do currículo e uma matriz obrigatória que força escolha de nível para Django, multithread e MongoDB, sem alternativa para ausência de experiência. A candidatura não foi enviada para não declarar vivência inexistente.</x:v>
+      </x:c>
+      <x:c r="F131" s="29" t="str">
+        <x:v>Pendente</x:v>
+      </x:c>
+      <x:c r="G131" s="30" t="str">
+        <x:v>Retomar somente se o formulário permitir respostas factuais ou se houver experiência verificável nos itens exigidos. Qualquer desafio técnico e avaliação psicológica devem ser realizados pessoalmente.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F6:F59">
     <x:cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="Concluído"/>
@@ -11864,7 +11887,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re722279ff8ed4430"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45836b5406a942fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza acompanhamento de bancos e fintechs
</commit_message>
<xml_diff>
--- a/planilhas/Controle_Candidaturas_Fintech_Guilherme_PUBLICO.xlsx
+++ b/planilhas/Controle_Candidaturas_Fintech_Guilherme_PUBLICO.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidaturas" sheetId="1" r:id="R02707cd6597f4c15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log de auditoria" sheetId="2" r:id="Rcf8db25bccd4489f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidaturas" sheetId="1" r:id="R00f709b3f7104a39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log de auditoria" sheetId="2" r:id="Rf774f03803fa4635"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -503,7 +503,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CandidaturasTable" displayName="CandidaturasTable" ref="A9:K196" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CandidaturasTable" displayName="CandidaturasTable" ref="A9:K198" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Status"/>
     <x:tableColumn id="2" name="Empresa"/>
@@ -756,10 +756,10 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>Tecnologia, dados, IA e operações técnicas. Versão pública: dados pessoais e links privados removidos. Fonte atualizada em 02/10/2026.</x:v>
+        <x:v>Tecnologia, dados, IA, operações técnicas e negócios técnicos. Versão pública: dados pessoais e links privados removidos. Fonte atualizada em 03/10/2026.</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Tecnologia, dados, IA e operações técnicas. Currículo mestre e ciclo de candidaturas atualizados em 02/10/2026.</x:v>
+        <x:v>Tecnologia, dados, IA, operações técnicas e negócios técnicos. Currículo mestre e ciclo de candidaturas atualizados em 03/10/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -793,23 +793,23 @@
         <x:v>Candidaturas confirmadas</x:v>
       </x:c>
       <x:c r="B7" s="9" t="n">
-        <x:f>SUM(L10:L196)</x:f>
-        <x:v>93</x:v>
+        <x:f>SUM(L10:L198)</x:f>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="C7" s="8"/>
       <x:c r="D7" s="8" t="str">
         <x:v>Itens em controle</x:v>
       </x:c>
       <x:c r="E7" s="9" t="n">
-        <x:f>COUNTA(A10:A196)</x:f>
-        <x:v>187</x:v>
+        <x:f>COUNTA(A10:A198)</x:f>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="F7" s="8"/>
       <x:c r="G7" s="8" t="str">
         <x:v>Pendentes</x:v>
       </x:c>
       <x:c r="H7" s="9" t="n">
-        <x:f>SUM(M10:M196)</x:f>
+        <x:f>SUM(M10:M198)</x:f>
         <x:v>83</x:v>
       </x:c>
     </x:row>
@@ -1031,32 +1031,32 @@
         <x:v>Analista de Operações Júnior | Monitoração Python</x:v>
       </x:c>
       <x:c r="D14" s="15" t="str">
-        <x:v>Automação e dados</x:v>
+        <x:v>Automação, monitoração e dados</x:v>
       </x:c>
       <x:c r="E14" s="15" t="str">
-        <x:v>São Paulo, presencial</x:v>
+        <x:v>São Paulo/SP; presencial</x:v>
       </x:c>
       <x:c r="F14" s="16" t="str">
         <x:v>https://job-boards.greenhouse.io/c6bank/jobs/4712934005</x:v>
       </x:c>
       <x:c r="G14" s="18" t="str">
-        <x:v>Não informado</x:v>
+        <x:v>Nenhuma avaliação iniciada; acompanhar e-mail e MyGreenhouse</x:v>
       </x:c>
       <x:c r="H14" s="18" t="str">
-        <x:v>Acompanhar via MyGreenhouse</x:v>
+        <x:v>Acompanhar e-mail e MyGreenhouse. Se houver avaliação, entrevista ou teste, realizar pessoalmente.</x:v>
       </x:c>
       <x:c r="I14" s="19" t="str">
-        <x:v>18/09/2026</x:v>
+        <x:v>03/10/2026</x:v>
       </x:c>
       <x:c r="J14" s="18" t="str">
-        <x:v>Candidatura confirmada; currículo em texto e Python/SQL intermediários</x:v>
+        <x:v>Candidatura confirmada no Greenhouse com currículo e apresentação adaptados. Foram declarados Python e SQL em nível intermediário, além de automação, monitoração, APIs e experiência full stack factual.</x:v>
       </x:c>
       <x:c r="K14" s="24" t="str">
-        <x:v>Não localizado — auditoria 19/09</x:v>
+        <x:v>Sim — confirmação Greenhouse 03/10</x:v>
       </x:c>
       <x:c r="L14" t="n">
         <x:f>IF(LEFT(K14,3)="Sim",1,0)+IF(LEFT(K14,6)="Portal",1,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M14" t="n">
         <x:f>IF(LEFT(A14,8)="Pendente",1,0)</x:f>
@@ -1934,28 +1934,28 @@
         <x:v>[Crédito] Software Engineer II — C#</x:v>
       </x:c>
       <x:c r="D35" s="15" t="str">
-        <x:v>Desenvolvimento</x:v>
+        <x:v>Desenvolvimento de software em crédito</x:v>
       </x:c>
       <x:c r="E35" s="15" t="str">
-        <x:v>Remoto</x:v>
+        <x:v>Remoto; contratação e salário não divulgados</x:v>
       </x:c>
       <x:c r="F35" s="16" t="str">
         <x:v>https://job-boards.greenhouse.io/stone/jobs/7996581003</x:v>
       </x:c>
       <x:c r="G35" s="18" t="str">
-        <x:v>Não aplicável</x:v>
+        <x:v>Nenhuma avaliação iniciada; acompanhar e-mail e portal</x:v>
       </x:c>
       <x:c r="H35" s="18" t="str">
-        <x:v>Acompanhar candidatura / e-mail</x:v>
+        <x:v>Acompanhar e-mail e Greenhouse. Preparar exemplos factuais de C#/.NET, testes, Docker, CI/CD, APIs, PostgreSQL e dados.</x:v>
       </x:c>
       <x:c r="I35" s="19" t="str">
-        <x:v>18/09/2026</x:v>
+        <x:v>03/10/2026</x:v>
       </x:c>
       <x:c r="J35" s="18" t="str">
-        <x:v>Candidatura confirmada como júnior; C#/.NET, testes, Docker, CI/CD e dados; sem inflar padrões formais, ágil ou mensageria</x:v>
+        <x:v>Candidatura confirmada com enquadramento júnior informado na descrição. O texto foi personalizado com Performance Lab, C#/.NET, testes, Docker, CI/CD, APIs e dados, sem alegar experiência formal inexistente em mensageria, ágil ou padrões avançados.</x:v>
       </x:c>
       <x:c r="K35" s="24" t="str">
-        <x:v>Sim — recibo 18/09</x:v>
+        <x:v>Sim — confirmação Greenhouse 03/10</x:v>
       </x:c>
       <x:c r="L35" t="n">
         <x:f>IF(LEFT(K35,3)="Sim",1,0)+IF(LEFT(K35,6)="Portal",1,0)</x:f>
@@ -8889,24 +8889,110 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="197">
-      <x:c r="A197" s="32" t="str">
+    <x:row r="197" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A197" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B197" s="63" t="str">
+        <x:v>C6 Bank</x:v>
+      </x:c>
+      <x:c r="C197" s="63" t="str">
+        <x:v>Analista de Operações Júnior | Sustentação RPA (COE RPA)</x:v>
+      </x:c>
+      <x:c r="D197" s="63" t="str">
+        <x:v>Automação e operações técnicas</x:v>
+      </x:c>
+      <x:c r="E197" s="63" t="str">
+        <x:v>São Paulo/SP; modalidade não divulgada</x:v>
+      </x:c>
+      <x:c r="F197" s="63" t="str">
+        <x:v>https://job-boards.greenhouse.io/c6bank/jobs/4737668005</x:v>
+      </x:c>
+      <x:c r="G197" s="63" t="str">
+        <x:v>Nenhuma avaliação iniciada; acompanhar e-mail e portal</x:v>
+      </x:c>
+      <x:c r="H197" s="63" t="str">
+        <x:v>Acompanhar e-mail e MyGreenhouse. Se houver avaliação, entrevista ou teste, realizar pessoalmente.</x:v>
+      </x:c>
+      <x:c r="I197" s="63" t="str">
+        <x:v>03/10/2026</x:v>
+      </x:c>
+      <x:c r="J197" s="63" t="str">
+        <x:v>Candidatura confirmada no Greenhouse. A apresentação foi adaptada com automação, APIs, Python, SQL, integrações, Docker e experiência full stack factual; RPA corporativo foi tratado como frente de aprofundamento.</x:v>
+      </x:c>
+      <x:c r="K197" s="63" t="str">
+        <x:v>Sim — confirmação Greenhouse 03/10</x:v>
+      </x:c>
+      <x:c r="L197" t="n">
+        <x:f>IF(LEFT(K197,3)="Sim",1,0)+IF(LEFT(K197,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M197" t="n">
+        <x:f>IF(LEFT(A197,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198" ht="66" hidden="0" customHeight="1">
+      <x:c r="A198" s="63" t="str">
+        <x:v>Enviada</x:v>
+      </x:c>
+      <x:c r="B198" s="63" t="str">
+        <x:v>iFood</x:v>
+      </x:c>
+      <x:c r="C198" s="63" t="str">
+        <x:v>Analista de Negócios Pleno</x:v>
+      </x:c>
+      <x:c r="D198" s="63" t="str">
+        <x:v>Negócios, dados e tecnologia</x:v>
+      </x:c>
+      <x:c r="E198" s="63" t="str">
+        <x:v>Osasco/SP; modalidade conforme anúncio</x:v>
+      </x:c>
+      <x:c r="F198" s="63" t="str">
+        <x:v>https://job-boards.greenhouse.io/ifoodcarreiras/jobs/8696675002</x:v>
+      </x:c>
+      <x:c r="G198" s="63" t="str">
+        <x:v>Nenhuma avaliação iniciada; acompanhar e-mail e portal</x:v>
+      </x:c>
+      <x:c r="H198" s="63" t="str">
+        <x:v>Acompanhar e-mail e Greenhouse. Preparar exemplos factuais de B2B, melhoria de processos, dados, automação e desenvolvimento full stack.</x:v>
+      </x:c>
+      <x:c r="I198" s="63" t="str">
+        <x:v>03/10/2026</x:v>
+      </x:c>
+      <x:c r="J198" s="63" t="str">
+        <x:v>Candidatura confirmada no Greenhouse com texto personalizado. Foram conectados 12 anos de contexto B2B e a experiência profissional full stack, sem transformar a trajetória comercial em experiência de engenharia não comprovada.</x:v>
+      </x:c>
+      <x:c r="K198" s="63" t="str">
+        <x:v>Sim — confirmação Greenhouse 03/10</x:v>
+      </x:c>
+      <x:c r="L198" t="n">
+        <x:f>IF(LEFT(K198,3)="Sim",1,0)+IF(LEFT(K198,6)="Portal",1,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M198" t="n">
+        <x:f>IF(LEFT(A198,8)="Pendente",1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199">
+      <x:c r="A199" s="32" t="str">
         <x:v>Nota: ‘Sim’ significa recibo de e-mail localizado; ‘Portal’ significa confirmação/etapa verificada no portal. E-mails de inscrição iniciada não são tratados como candidatura enviada. Não há dados pessoais sensíveis nesta planilha.</x:v>
       </x:c>
-      <x:c r="B197" s="63"/>
-      <x:c r="C197" s="63"/>
-      <x:c r="D197" s="63"/>
-      <x:c r="E197" s="63"/>
-      <x:c r="F197" s="63"/>
-      <x:c r="G197" s="63"/>
-      <x:c r="H197" s="63"/>
-      <x:c r="I197" s="63"/>
-      <x:c r="J197" s="63"/>
-      <x:c r="K197" s="63"/>
+      <x:c r="B199" s="63"/>
+      <x:c r="C199" s="63"/>
+      <x:c r="D199" s="63"/>
+      <x:c r="E199" s="63"/>
+      <x:c r="F199" s="63"/>
+      <x:c r="G199" s="63"/>
+      <x:c r="H199" s="63"/>
+      <x:c r="I199" s="63"/>
+      <x:c r="J199" s="63"/>
+      <x:c r="K199" s="63"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A197:K197"/>
+    <x:mergeCell ref="A199:K199"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A10:A108">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Enviada"/>
@@ -8924,7 +9010,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda9b7dfea1e449a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33860743df3740ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11876,6 +11962,29 @@
         <x:v>Retomar somente se o formulário permitir respostas factuais ou se houver experiência verificável nos itens exigidos. Qualquer desafio técnico e avaliação psicológica devem ser realizados pessoalmente.</x:v>
       </x:c>
     </x:row>
+    <x:row r="132">
+      <x:c r="A132" s="61" t="str">
+        <x:v>03/10/2026</x:v>
+      </x:c>
+      <x:c r="B132" s="28" t="str">
+        <x:v>Bancos e fintechs</x:v>
+      </x:c>
+      <x:c r="C132" s="28" t="str">
+        <x:v>C6 Bank, Stone e iFood</x:v>
+      </x:c>
+      <x:c r="D132" s="28" t="str">
+        <x:v>Quatro confirmações revalidadas</x:v>
+      </x:c>
+      <x:c r="E132" s="28" t="str">
+        <x:v>Foram confirmadas candidaturas para C6 Monitoração Python, C6 Sustentação RPA, Stone Software Engineer C# remoto e iFood Analista de Negócios Pleno. As trilhas combinam desenvolvimento, automação, dados e contexto B2B sem enquadrar o candidato em funções puramente comerciais.</x:v>
+      </x:c>
+      <x:c r="F132" s="29" t="str">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="G132" s="30" t="str">
+        <x:v>Acompanhar e-mail e portais. Qualquer avaliação comportamental, técnica, vídeo ou áudio deve ser feita pessoalmente pelo candidato.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F6:F59">
     <x:cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="Concluído"/>
@@ -11887,7 +11996,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45836b5406a942fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R106832cd06d34130"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>